<commit_message>
Se agrega la sección de carga de ambientaciones en página CMS Productos, se agrega la opción Tiendanube en cuadro de URL de redes sociales. Se agrega el editor de backgroud y texto con su propio preview en página CMS Diseño
</commit_message>
<xml_diff>
--- a/BBDD.xlsx
+++ b/BBDD.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyectos\Web_Andez\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{004FE4DE-6D36-40CC-B083-C820EBD0BFC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C629E76-CA29-4CFC-A0EE-C5CC25ED779D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5D42B345-DB14-48C1-9A38-23908D3120ED}"/>
   </bookViews>
@@ -118,7 +118,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="200">
   <si>
     <t>Color</t>
   </si>
@@ -468,9 +468,6 @@
     <t>EsPortada</t>
   </si>
   <si>
-    <t>ImagenesAmbientaciones</t>
-  </si>
-  <si>
     <t>IdProducto</t>
   </si>
   <si>
@@ -577,6 +574,150 @@
   </si>
   <si>
     <t>Lun a Vier 8 a 16</t>
+  </si>
+  <si>
+    <t>ImagenesAmbientaciones (está en productos)</t>
+  </si>
+  <si>
+    <t>PaginaIndex</t>
+  </si>
+  <si>
+    <t>Posicion</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>LinkSN</t>
+  </si>
+  <si>
+    <t>LanzamientoSN</t>
+  </si>
+  <si>
+    <t>PausaSN</t>
+  </si>
+  <si>
+    <t>Monocomando Cross</t>
+  </si>
+  <si>
+    <t>Lavatorio Next</t>
+  </si>
+  <si>
+    <t>Jabonera Rejilla</t>
+  </si>
+  <si>
+    <t>Línea Cross</t>
+  </si>
+  <si>
+    <t>Línea Next</t>
+  </si>
+  <si>
+    <t>Linea Match</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Background</t>
+  </si>
+  <si>
+    <t>URLoCodigoHexadecimal</t>
+  </si>
+  <si>
+    <t>#F54927</t>
+  </si>
+  <si>
+    <t>#19548A</t>
+  </si>
+  <si>
+    <t>Paginas</t>
+  </si>
+  <si>
+    <t>Pagina</t>
+  </si>
+  <si>
+    <t>Index</t>
+  </si>
+  <si>
+    <t>TipoTexto</t>
+  </si>
+  <si>
+    <t>Parrafo</t>
+  </si>
+  <si>
+    <t>Frase</t>
+  </si>
+  <si>
+    <t>TextoPagina</t>
+  </si>
+  <si>
+    <t>ColorGradiente1</t>
+  </si>
+  <si>
+    <t>ColorGradiente2</t>
+  </si>
+  <si>
+    <t>ColorGradiente3</t>
+  </si>
+  <si>
+    <t>ColorGradiente4</t>
+  </si>
+  <si>
+    <t>ColorSolido</t>
+  </si>
+  <si>
+    <t>Angulo</t>
+  </si>
+  <si>
+    <t>Opacidad</t>
+  </si>
+  <si>
+    <t>Blur</t>
+  </si>
+  <si>
+    <t>Brillo</t>
+  </si>
+  <si>
+    <t>Contraste</t>
+  </si>
+  <si>
+    <t>EscalaGrises</t>
+  </si>
+  <si>
+    <t>URLBackground</t>
+  </si>
+  <si>
+    <t>Fuente</t>
+  </si>
+  <si>
+    <t>Arial</t>
+  </si>
+  <si>
+    <t>Time New Romans</t>
+  </si>
+  <si>
+    <t>Aptos Narrow</t>
+  </si>
+  <si>
+    <t>Columna5</t>
+  </si>
+  <si>
+    <t>Columna6</t>
+  </si>
+  <si>
+    <t>Columna7</t>
+  </si>
+  <si>
+    <t>IdTipoTexto</t>
+  </si>
+  <si>
+    <t>IdFuente</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>Tamaño</t>
   </si>
 </sst>
 </file>
@@ -743,7 +884,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -757,12 +898,18 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -772,21 +919,11 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="56">
+  <dxfs count="57">
     <dxf>
       <font>
         <b val="0"/>
@@ -806,80 +943,8 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor theme="0" tint="-0.14999847407452621"/>
         </patternFill>
       </fill>
     </dxf>
@@ -901,137 +966,153 @@
         <scheme val="minor"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1044,49 +1125,129 @@
     </dxf>
     <dxf>
       <fill>
-        <patternFill>
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9"/>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1277,7 +1438,7 @@
   <autoFilter ref="A13:E16" xr:uid="{D96833EF-4E6F-4FA0-A7A0-6E6817E2B38A}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{317907DD-843B-4FA4-8837-A0A78A4A0507}" name="ID"/>
-    <tableColumn id="5" xr3:uid="{E0921BEC-D870-4C51-B3FC-23E013804DC3}" name="CodigoColor" dataDxfId="55"/>
+    <tableColumn id="5" xr3:uid="{E0921BEC-D870-4C51-B3FC-23E013804DC3}" name="CodigoColor" dataDxfId="56"/>
     <tableColumn id="2" xr3:uid="{8053C3DC-ACA4-4AAB-9AFB-34FBDDEBC52B}" name="NombreColor"/>
     <tableColumn id="4" xr3:uid="{1D3A10F0-E8C4-471A-B4A8-2001816AFFF2}" name="URLColor"/>
     <tableColumn id="3" xr3:uid="{D04813E9-6E48-439B-A711-735DEB41533C}" name="Activo"/>
@@ -1310,8 +1471,8 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{C6605137-9E60-4417-BE9D-22DF41FEA57D}" name="ID"/>
     <tableColumn id="2" xr3:uid="{D82CDF84-BD14-4C63-ABBA-8F2236A9C0E4}" name="Pais"/>
-    <tableColumn id="3" xr3:uid="{FA78D055-E341-4362-A23A-0CCFC591E8FA}" name="Latitud" dataDxfId="52"/>
-    <tableColumn id="4" xr3:uid="{36EB177E-ACE1-4B78-A56A-A9F891312B25}" name="Longitud" dataDxfId="51"/>
+    <tableColumn id="3" xr3:uid="{FA78D055-E341-4362-A23A-0CCFC591E8FA}" name="Latitud" dataDxfId="53"/>
+    <tableColumn id="4" xr3:uid="{36EB177E-ACE1-4B78-A56A-A9F891312B25}" name="Longitud" dataDxfId="52"/>
     <tableColumn id="5" xr3:uid="{4122267C-292B-476B-8AB1-41CBE8A90AAF}" name="Zoom"/>
     <tableColumn id="7" xr3:uid="{0270C110-04E9-4179-AF06-958CA4E37E9B}" name="Activo"/>
   </tableColumns>
@@ -1320,14 +1481,14 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{EF32F6B3-AC45-462F-BE18-EFE2DD57FE9B}" name="Tabla17" displayName="Tabla17" ref="H41:L44" totalsRowShown="0" headerRowDxfId="50" dataDxfId="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{EF32F6B3-AC45-462F-BE18-EFE2DD57FE9B}" name="Tabla17" displayName="Tabla17" ref="H41:L44" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50">
   <autoFilter ref="H41:L44" xr:uid="{EF32F6B3-AC45-462F-BE18-EFE2DD57FE9B}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{C8F6ED57-5FD2-4FB3-A4A5-BC3965E98B15}" name="ID" dataDxfId="48"/>
-    <tableColumn id="2" xr3:uid="{65B99387-EDCD-429B-B81B-A4F58479A304}" name="IdProducto" dataDxfId="47"/>
-    <tableColumn id="3" xr3:uid="{5D9C0348-2DF4-47CC-977C-AAFB9F19E959}" name="Titulo" dataDxfId="46"/>
-    <tableColumn id="4" xr3:uid="{1CACB54F-DC9D-41AC-A04F-171EF34060DC}" name="URLImagen" dataDxfId="45"/>
-    <tableColumn id="7" xr3:uid="{824500A6-D872-42FD-9C38-60CB54869E2F}" name="Activo" dataDxfId="44"/>
+    <tableColumn id="1" xr3:uid="{C8F6ED57-5FD2-4FB3-A4A5-BC3965E98B15}" name="ID" dataDxfId="49"/>
+    <tableColumn id="2" xr3:uid="{65B99387-EDCD-429B-B81B-A4F58479A304}" name="IdProducto" dataDxfId="48"/>
+    <tableColumn id="3" xr3:uid="{5D9C0348-2DF4-47CC-977C-AAFB9F19E959}" name="Titulo" dataDxfId="47"/>
+    <tableColumn id="4" xr3:uid="{1CACB54F-DC9D-41AC-A04F-171EF34060DC}" name="URLImagen" dataDxfId="46"/>
+    <tableColumn id="7" xr3:uid="{824500A6-D872-42FD-9C38-60CB54869E2F}" name="Activo" dataDxfId="45"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1355,8 +1516,8 @@
     <tableColumn id="3" xr3:uid="{650899D4-4E19-437F-9FCF-B4D26F2AA0DB}" name="Direccion"/>
     <tableColumn id="4" xr3:uid="{1E07E83B-09DC-40FD-907E-40F4CBC0A570}" name="IdProvincia"/>
     <tableColumn id="5" xr3:uid="{6138418F-A367-4A68-8F05-2638E82A22BC}" name="Telefono"/>
-    <tableColumn id="6" xr3:uid="{80260CDA-43B3-49C5-B2E8-6D4D4EE4367B}" name="Latitud" dataDxfId="43"/>
-    <tableColumn id="7" xr3:uid="{D1025C6A-57D3-4E57-916D-CF79774C6EAF}" name="Longitud" dataDxfId="42"/>
+    <tableColumn id="6" xr3:uid="{80260CDA-43B3-49C5-B2E8-6D4D4EE4367B}" name="Latitud" dataDxfId="44"/>
+    <tableColumn id="7" xr3:uid="{D1025C6A-57D3-4E57-916D-CF79774C6EAF}" name="Longitud" dataDxfId="43"/>
     <tableColumn id="8" xr3:uid="{FACFCBBE-C8C5-4011-911D-7F4D64577C47}" name="IdPagina"/>
     <tableColumn id="9" xr3:uid="{3EE8280A-E1AE-43CB-8AA3-681D1032743D}" name="Activo"/>
   </tableColumns>
@@ -1365,13 +1526,13 @@
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{B6BCDECB-3201-4C98-AA8D-79812894A18B}" name="Tabla19" displayName="Tabla19" ref="K34:N37" totalsRowShown="0" headerRowDxfId="41" dataDxfId="40">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{B6BCDECB-3201-4C98-AA8D-79812894A18B}" name="Tabla19" displayName="Tabla19" ref="K34:N37" totalsRowShown="0" headerRowDxfId="42" dataDxfId="41">
   <autoFilter ref="K34:N37" xr:uid="{36798AE9-B843-4477-9F23-32045BDEF7D7}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{E050CEA3-2793-4698-9E45-C3447ADCD555}" name="ID" dataDxfId="39"/>
-    <tableColumn id="2" xr3:uid="{03295AE7-34B5-4134-9D2F-2268D15B310C}" name="IDProducto" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{1564E106-D50F-4573-A696-EE197325F0F3}" name="IDAtributo" dataDxfId="37"/>
-    <tableColumn id="4" xr3:uid="{5F701778-C720-415C-9979-8380EB9AB80C}" name="Activo" dataDxfId="36"/>
+    <tableColumn id="1" xr3:uid="{E050CEA3-2793-4698-9E45-C3447ADCD555}" name="ID" dataDxfId="40"/>
+    <tableColumn id="2" xr3:uid="{03295AE7-34B5-4134-9D2F-2268D15B310C}" name="IDProducto" dataDxfId="39"/>
+    <tableColumn id="3" xr3:uid="{1564E106-D50F-4573-A696-EE197325F0F3}" name="IDAtributo" dataDxfId="38"/>
+    <tableColumn id="4" xr3:uid="{5F701778-C720-415C-9979-8380EB9AB80C}" name="Activo" dataDxfId="37"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1384,8 +1545,8 @@
     <tableColumn id="1" xr3:uid="{76441B91-C9F3-418E-9F7A-2145EC66A51B}" name="ID"/>
     <tableColumn id="2" xr3:uid="{B7D7EADF-0604-4B90-A7CA-6537AE39152D}" name="Pronvincia"/>
     <tableColumn id="3" xr3:uid="{FBCCEEC7-DBEE-4480-8CBE-1F5805CA9202}" name="IdPais"/>
-    <tableColumn id="4" xr3:uid="{0A3D75EA-6C18-48E0-9489-C5D19B3AC70A}" name="Latitud" dataDxfId="35"/>
-    <tableColumn id="5" xr3:uid="{ACBD9873-D350-427F-993B-2B1B42296D9B}" name="Longitud" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{0A3D75EA-6C18-48E0-9489-C5D19B3AC70A}" name="Latitud" dataDxfId="36"/>
+    <tableColumn id="5" xr3:uid="{ACBD9873-D350-427F-993B-2B1B42296D9B}" name="Longitud" dataDxfId="35"/>
     <tableColumn id="6" xr3:uid="{957CA68C-6225-4C37-B8D5-8FF8C064FB1C}" name="Zoom"/>
     <tableColumn id="7" xr3:uid="{D19F9B22-3CC1-4E0E-B3DB-56D9B346F0CD}" name="Activo"/>
   </tableColumns>
@@ -1394,58 +1555,59 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{D66B8F6B-A06F-42EB-B1CE-F5AC470DCC17}" name="Tabla20" displayName="Tabla20" ref="A62:E65" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{D66B8F6B-A06F-42EB-B1CE-F5AC470DCC17}" name="Tabla20" displayName="Tabla20" ref="A62:E65" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
   <autoFilter ref="A62:E65" xr:uid="{6995137C-E78D-4F26-A126-F3AEFE2A2B13}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{7C1F763D-9A29-4F91-BB26-5F2CF68260F0}" name="ID" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{F0BF2187-ECA7-4173-9FAC-3BC72EFDB82F}" name="IdEmpresa" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{98E75056-4A9A-4C56-8FA5-EFD4D867777B}" name="Nombre" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{48A2AE2B-7A42-420C-8BB3-5F9F2AA01721}" name="Mail" dataDxfId="21">
+    <tableColumn id="1" xr3:uid="{7C1F763D-9A29-4F91-BB26-5F2CF68260F0}" name="ID" dataDxfId="32"/>
+    <tableColumn id="5" xr3:uid="{F0BF2187-ECA7-4173-9FAC-3BC72EFDB82F}" name="IdEmpresa" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{98E75056-4A9A-4C56-8FA5-EFD4D867777B}" name="Nombre" dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{48A2AE2B-7A42-420C-8BB3-5F9F2AA01721}" name="Mail" dataDxfId="29">
       <calculatedColumnFormula>CONCATENATE(C63,"@andez.com.ar")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{31D99612-66DC-4B54-A747-6C39765D7B66}" name="Activo" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{31D99612-66DC-4B54-A747-6C39765D7B66}" name="Activo" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{2B2EAABA-4403-411A-98F0-A8284D43302C}" name="Tabla2021" displayName="Tabla2021" ref="G62:K65" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{2B2EAABA-4403-411A-98F0-A8284D43302C}" name="Tabla2021" displayName="Tabla2021" ref="G62:K65" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
   <autoFilter ref="G62:K65" xr:uid="{89087EED-CE2D-441A-9746-B0BA56EA9A63}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{6D3F8F4E-2473-4BE6-A51E-C3C3E4C26133}" name="ID" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{8C181956-53C7-4FD2-BAAB-42B1CDE2E84E}" name="IdEmpresa" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{12B007DF-889A-4CDB-93CC-EBEFCBD3A3E9}" name="Nombre" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{A94B5F86-8442-44DD-9C03-77F51D7F5B8D}" name="Telefono" dataDxfId="16">
+    <tableColumn id="1" xr3:uid="{6D3F8F4E-2473-4BE6-A51E-C3C3E4C26133}" name="ID" dataDxfId="25"/>
+    <tableColumn id="5" xr3:uid="{8C181956-53C7-4FD2-BAAB-42B1CDE2E84E}" name="IdEmpresa" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{12B007DF-889A-4CDB-93CC-EBEFCBD3A3E9}" name="Nombre" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{A94B5F86-8442-44DD-9C03-77F51D7F5B8D}" name="Telefono" dataDxfId="22">
       <calculatedColumnFormula>CONCATENATE(I63,"@andez.com.ar")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{0E412ADD-9FF3-43E1-BDA1-A917D6B1E4D7}" name="Activo" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{0E412ADD-9FF3-43E1-BDA1-A917D6B1E4D7}" name="Activo" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{8F3FF2B6-156D-475C-B60E-2BBAE1F181CE}" name="Tabla21" displayName="Tabla21" ref="A69:E72" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28" tableBorderDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{8F3FF2B6-156D-475C-B60E-2BBAE1F181CE}" name="Tabla21" displayName="Tabla21" ref="A69:E72" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19" tableBorderDxfId="18">
   <autoFilter ref="A69:E72" xr:uid="{58000D4A-AEBA-4D49-B463-180C8FD8A937}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{E9F2D081-00F6-4B92-9DFE-6473CB6B3F38}" name="ID" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{FE107DC5-A1C2-4F54-BC82-5BBB32CCABC3}" name="IdEmpresa" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{DE65DD1F-F1BA-4548-A19A-4B9DD2857A6F}" name="Red" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{23F951D4-E519-45F7-81C5-69ED4EA385E4}" name="URLRed" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{E5F1016C-C8F1-4FEA-B687-B57CB00F2E70}" name="Activo" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{E9F2D081-00F6-4B92-9DFE-6473CB6B3F38}" name="ID" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{FE107DC5-A1C2-4F54-BC82-5BBB32CCABC3}" name="IdEmpresa" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{DE65DD1F-F1BA-4548-A19A-4B9DD2857A6F}" name="Red" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{23F951D4-E519-45F7-81C5-69ED4EA385E4}" name="URLRed" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{E5F1016C-C8F1-4FEA-B687-B57CB00F2E70}" name="Activo" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5C307171-21C3-4D19-9190-21EBBEF7C7BE}" name="Tabla13" displayName="Tabla13" ref="G13:J16" totalsRowShown="0">
-  <autoFilter ref="G13:J16" xr:uid="{5C307171-21C3-4D19-9190-21EBBEF7C7BE}"/>
-  <tableColumns count="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5C307171-21C3-4D19-9190-21EBBEF7C7BE}" name="Tabla13" displayName="Tabla13" ref="G13:K16" totalsRowShown="0">
+  <autoFilter ref="G13:K16" xr:uid="{5C307171-21C3-4D19-9190-21EBBEF7C7BE}"/>
+  <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{68AE05C3-BABF-43F5-8570-0421BA4C67E8}" name="ID"/>
     <tableColumn id="4" xr3:uid="{59F766FF-BD10-4A8B-9F9F-31F1C7687013}" name="CodigoLinea"/>
     <tableColumn id="2" xr3:uid="{6F05575C-428D-4038-A5FF-312E257A42E9}" name="NombreLinea"/>
+    <tableColumn id="5" xr3:uid="{E68168E7-9BED-421B-9270-741133D3D01A}" name="Descripcion"/>
     <tableColumn id="3" xr3:uid="{B831A1C2-04F5-4FEF-939E-BB8F988F8105}" name="Activo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1453,27 +1615,126 @@
 </file>
 
 <file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{C769ADF8-2405-479D-8112-7564F0940768}" name="Tabla22" displayName="Tabla22" ref="A76:J77" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{C769ADF8-2405-479D-8112-7564F0940768}" name="Tabla22" displayName="Tabla22" ref="A76:J77" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
   <autoFilter ref="A76:J77" xr:uid="{A2E83C68-75BA-4C98-B80E-E4E7E2B0B82C}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{173EAAD2-F12F-4372-8FA2-00B32059C1EB}" name="ID" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{3E7AAA46-3847-4587-A43F-E688C1582045}" name="RazonSocial" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{7727AE8E-759C-4DE1-86AE-BDFED86835D0}" name="CUIT" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{BBA783BB-BBBB-4233-929D-4BF68AFA091A}" name="Direccion" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{419A73DC-BE03-4D90-BE0C-9779F3EB2DDB}" name="Localidad" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{BE8C959F-F07F-4076-8E57-3EA25221B957}" name="Partido" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{DB60E2FA-C8A3-4C27-BCAB-41F7E5C99855}" name="IdProvincia" dataDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{EC23197E-97BD-4D2B-AF77-BAEDEAEEEB33}" name="CP" dataDxfId="2"/>
-    <tableColumn id="10" xr3:uid="{7234FBEF-54AA-4FBE-8D11-84EDF024DAB3}" name="Horario" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{2D33166C-2999-4BC9-8B00-7F06B4D84FF1}" name="Activo" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{173EAAD2-F12F-4372-8FA2-00B32059C1EB}" name="ID" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{3E7AAA46-3847-4587-A43F-E688C1582045}" name="RazonSocial" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{7727AE8E-759C-4DE1-86AE-BDFED86835D0}" name="CUIT" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{BBA783BB-BBBB-4233-929D-4BF68AFA091A}" name="Direccion" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{419A73DC-BE03-4D90-BE0C-9779F3EB2DDB}" name="Localidad" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{BE8C959F-F07F-4076-8E57-3EA25221B957}" name="Partido" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{DB60E2FA-C8A3-4C27-BCAB-41F7E5C99855}" name="IdProvincia" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{EC23197E-97BD-4D2B-AF77-BAEDEAEEEB33}" name="CP" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{7234FBEF-54AA-4FBE-8D11-84EDF024DAB3}" name="Horario" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{2D33166C-2999-4BC9-8B00-7F06B4D84FF1}" name="Activo" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{93610188-F7B2-40FB-B0A9-E18135492A82}" name="Tabla7" displayName="Tabla7" ref="A81:K84" totalsRowShown="0">
+  <autoFilter ref="A81:K84" xr:uid="{93610188-F7B2-40FB-B0A9-E18135492A82}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{1035A3C3-56C5-4CB6-B2AD-211341406B65}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{A5D7D600-3A71-4DD1-A6A0-88B6463C987F}" name="Posicion"/>
+    <tableColumn id="3" xr3:uid="{473E571D-8BE9-4BD5-B8BD-FC16062FBA4A}" name="Nombre"/>
+    <tableColumn id="4" xr3:uid="{BFCDC025-7291-43F4-BF51-02B5C205C0B1}" name="URLImagen"/>
+    <tableColumn id="5" xr3:uid="{1AD6DCB5-B8FB-43FC-88CE-E58B0DF75376}" name="Titulo"/>
+    <tableColumn id="6" xr3:uid="{782D732A-1C91-4938-BDF6-8C352984694E}" name="Descripcion" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{37200F4F-B540-4A63-9F27-255BD55AD0BD}" name="Link"/>
+    <tableColumn id="8" xr3:uid="{CB7E851F-8679-4467-A629-18DE76D9185B}" name="LinkSN"/>
+    <tableColumn id="9" xr3:uid="{DF01FB7D-3582-4808-83E6-C0BF4EDCA881}" name="LanzamientoSN"/>
+    <tableColumn id="10" xr3:uid="{29CA56A3-0BDD-4AEA-A3B6-65E562BFA47B}" name="PausaSN"/>
+    <tableColumn id="11" xr3:uid="{D16E7FAF-93EA-4266-8EED-9856A946F54F}" name="Activo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{68E94E33-CBEB-416E-8BE1-18A7BBEB19B8}" name="Tabla8" displayName="Tabla8" ref="A95:O98" totalsRowShown="0">
+  <autoFilter ref="A95:O98" xr:uid="{68E94E33-CBEB-416E-8BE1-18A7BBEB19B8}"/>
+  <tableColumns count="15">
+    <tableColumn id="1" xr3:uid="{1E8CA238-3595-4186-9A14-6CF4E7344108}" name="ID"/>
+    <tableColumn id="4" xr3:uid="{461BF0D3-CF94-41A1-8339-A826048D1E99}" name="IdPagina"/>
+    <tableColumn id="5" xr3:uid="{7E4F1EF2-7520-4E68-B2FD-D184EC1CB1C3}" name="URLBackground"/>
+    <tableColumn id="6" xr3:uid="{6C881594-A7F4-46D3-A368-B8C8A77D11C3}" name="ColorGradiente1"/>
+    <tableColumn id="7" xr3:uid="{9B4B354C-8699-4AA2-9FD9-649842AE57D0}" name="ColorGradiente2"/>
+    <tableColumn id="8" xr3:uid="{01CA6DE3-6CFE-4CAE-A373-396E0851DD53}" name="ColorGradiente3"/>
+    <tableColumn id="9" xr3:uid="{B1E44F0D-9D59-449B-9FD7-82DF6631C1CD}" name="ColorGradiente4"/>
+    <tableColumn id="11" xr3:uid="{949976C3-3839-4BA5-A7E3-099398B9F562}" name="Angulo"/>
+    <tableColumn id="12" xr3:uid="{336F208F-5CA7-41FC-9D9A-CEAD6888A253}" name="ColorSolido"/>
+    <tableColumn id="13" xr3:uid="{82ED43C4-B914-48D4-AD3A-1B643F79C195}" name="Opacidad"/>
+    <tableColumn id="14" xr3:uid="{C74DFCB1-08F4-4D7E-93E3-D5FCA7AECBE1}" name="Blur"/>
+    <tableColumn id="15" xr3:uid="{07161F10-4594-40BD-9768-AB20BAA38606}" name="Brillo"/>
+    <tableColumn id="16" xr3:uid="{8A7CAB8F-C50F-4BD0-A384-77BE5DA8EC95}" name="Contraste"/>
+    <tableColumn id="17" xr3:uid="{F3288458-6C0F-465C-AD4F-1638638D6820}" name="EscalaGrises"/>
+    <tableColumn id="3" xr3:uid="{98D04B2A-95D5-473E-B16A-3D1B213CF0F8}" name="Activo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="23" xr:uid="{64C12ADD-1837-419C-BEA6-D3673F298051}" name="Tabla23" displayName="Tabla23" ref="A88:B91" totalsRowShown="0">
+  <autoFilter ref="A88:B91" xr:uid="{64C12ADD-1837-419C-BEA6-D3673F298051}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{D824E0B3-B2F8-41D9-8175-BA69AC070A74}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{D3CD5024-B197-422F-BABD-F76BAD4C09D5}" name="Pagina"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{3BCDB15F-39E2-4D22-A5F3-7E0244C0226B}" name="Tabla2325" displayName="Tabla2325" ref="D88:F91" totalsRowShown="0">
+  <autoFilter ref="D88:F91" xr:uid="{3BCDB15F-39E2-4D22-A5F3-7E0244C0226B}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{2E670FCF-1D70-42EE-BF2D-43F65298CE3C}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{07314AF4-A0B1-4694-870D-5FF7668BF237}" name="Nombre"/>
+    <tableColumn id="3" xr3:uid="{6229BA29-18D1-47DD-995E-DDF7832AEC46}" name="Activo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{603B1BB5-0E4C-4377-B4E9-1203B7A1C3FB}" name="Tabla826" displayName="Tabla826" ref="A102:K105" totalsRowShown="0">
+  <autoFilter ref="A102:K105" xr:uid="{603B1BB5-0E4C-4377-B4E9-1203B7A1C3FB}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{62362053-8A80-4FF4-AB6D-40430AC5A5F4}" name="ID"/>
+    <tableColumn id="4" xr3:uid="{794753EA-92E6-4DA1-AA5F-DD6E6EE6ED37}" name="IdPagina"/>
+    <tableColumn id="5" xr3:uid="{7B2052E1-C43E-4046-BE46-97E55A7FBE0F}" name="IdTipoTexto"/>
+    <tableColumn id="6" xr3:uid="{A93952EC-78FC-4DD0-B380-1E659DE63DFD}" name="IdFuente"/>
+    <tableColumn id="7" xr3:uid="{BB786B7B-E29D-4A14-B248-C9584ED0A547}" name="Color"/>
+    <tableColumn id="8" xr3:uid="{FFCC595A-F6A5-43DB-94E4-BD4E0394F4ED}" name="Tamaño"/>
+    <tableColumn id="9" xr3:uid="{A8921874-6C7F-4FBA-936A-D4B602C93F67}" name="Columna5"/>
+    <tableColumn id="10" xr3:uid="{AF446AA5-2F2C-4048-99E1-18C03C00DFCF}" name="Columna6"/>
+    <tableColumn id="11" xr3:uid="{4DD925C6-883F-40E6-911F-7E9E42C2279C}" name="Columna7"/>
+    <tableColumn id="2" xr3:uid="{5FF0673F-C0BF-4E18-815C-61F99F9FEF74}" name="URLoCodigoHexadecimal"/>
+    <tableColumn id="3" xr3:uid="{3715AA2C-BDFD-4A0F-9EEC-4D0E838CD882}" name="Activo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="26" xr:uid="{0B42635A-3ED7-432B-A4A5-0CA9F365C85C}" name="Tabla232527" displayName="Tabla232527" ref="H88:J91" totalsRowShown="0">
+  <autoFilter ref="H88:J91" xr:uid="{0B42635A-3ED7-432B-A4A5-0CA9F365C85C}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{3FA20A71-CF47-4DAB-951A-7C4FC5084311}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{79A7F6F7-1859-4BB3-B79B-BFF30483BAB2}" name="Fuente"/>
+    <tableColumn id="3" xr3:uid="{F7077B09-954A-4A25-96B1-3B3866C4F1D9}" name="Activo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{43BE8E47-D1D9-436F-87A2-5F1A6301B5E5}" name="Tabla14" displayName="Tabla14" ref="L13:O16" totalsRowShown="0">
-  <autoFilter ref="L13:O16" xr:uid="{43BE8E47-D1D9-436F-87A2-5F1A6301B5E5}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{43BE8E47-D1D9-436F-87A2-5F1A6301B5E5}" name="Tabla14" displayName="Tabla14" ref="M13:P16" totalsRowShown="0">
+  <autoFilter ref="M13:P16" xr:uid="{43BE8E47-D1D9-436F-87A2-5F1A6301B5E5}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{1CA967F6-5220-415A-8D46-EDE2F99DB4E7}" name="ID"/>
     <tableColumn id="2" xr3:uid="{85968E26-C5C2-48F7-940F-A91CDCD7A74E}" name="NombreAtributo"/>
@@ -1507,7 +1768,7 @@
     <tableColumn id="4" xr3:uid="{33CF0639-7E0E-4323-ABAC-57E9E79BAC94}" name="URLManual"/>
     <tableColumn id="6" xr3:uid="{8FB3C041-5F4E-4C6B-BFEA-F7EF8CCA380F}" name="URLRepuestos"/>
     <tableColumn id="7" xr3:uid="{19883A37-D7EF-411E-B5D4-0F9C58EA4DF5}" name="URLPlanos"/>
-    <tableColumn id="5" xr3:uid="{9FBFC04D-E638-4A8E-BF60-60BF85B463B6}" name="Activo" dataDxfId="54"/>
+    <tableColumn id="5" xr3:uid="{9FBFC04D-E638-4A8E-BF60-60BF85B463B6}" name="Activo" dataDxfId="55"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1534,7 +1795,7 @@
   <autoFilter ref="A6:G9" xr:uid="{00F67F5D-77F7-41B7-A265-5E336044A6C5}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{F32EBD58-4145-475F-A8DD-60533C773560}" name="ID"/>
-    <tableColumn id="5" xr3:uid="{BA938A3C-223C-48BE-9D99-D519D9B88EDF}" name="Nombre" dataDxfId="53"/>
+    <tableColumn id="5" xr3:uid="{BA938A3C-223C-48BE-9D99-D519D9B88EDF}" name="Nombre" dataDxfId="54"/>
     <tableColumn id="2" xr3:uid="{BF58FE61-5919-4F9C-BC69-7F6F4B0BCCB1}" name="Apellido"/>
     <tableColumn id="4" xr3:uid="{B217BF12-7466-47C6-83EC-0600B0F7EE4B}" name="Mail">
       <calculatedColumnFormula>CONCATENATE(Tabla15[[#This Row],[Nombre]],Tabla15[[#This Row],[Apellido]],"@andez.com.ar")</calculatedColumnFormula>
@@ -1888,29 +2149,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD350C1D-1850-4BF9-ABCF-FA1A23EC1542}">
-  <dimension ref="A1:O77"/>
+  <dimension ref="A1:P105"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="28.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.21875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="24.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.5546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="27.21875" bestFit="1" customWidth="1"/>
     <col min="11" max="12" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="16" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="12.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B1" s="11" t="s">
         <v>105</v>
       </c>
@@ -1921,24 +2181,24 @@
         <v>107</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A5" s="22" t="s">
+    <row r="4" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A5" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="24"/>
-      <c r="I5" s="22" t="s">
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="18"/>
+      <c r="I5" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="J5" s="23"/>
-      <c r="K5" s="24"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="J5" s="17"/>
+      <c r="K5" s="18"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
@@ -1970,7 +2230,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>1</v>
       </c>
@@ -2003,7 +2263,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>2</v>
       </c>
@@ -2036,7 +2296,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>3</v>
       </c>
@@ -2069,8 +2329,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" s="19" t="s">
         <v>0</v>
       </c>
@@ -2083,15 +2343,16 @@
       </c>
       <c r="H12" s="20"/>
       <c r="I12" s="20"/>
-      <c r="J12" s="21"/>
-      <c r="L12" s="19" t="s">
+      <c r="J12" s="20"/>
+      <c r="K12" s="21"/>
+      <c r="M12" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="M12" s="20"/>
       <c r="N12" s="20"/>
-      <c r="O12" s="21"/>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="O12" s="20"/>
+      <c r="P12" s="21"/>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>1</v>
       </c>
@@ -2116,23 +2377,26 @@
       <c r="I13" t="s">
         <v>8</v>
       </c>
-      <c r="J13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="L13" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="M13" t="s">
+      <c r="J13" t="s">
+        <v>57</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="M13" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="N13" t="s">
         <v>14</v>
       </c>
-      <c r="N13" t="s">
+      <c r="O13" t="s">
         <v>13</v>
       </c>
-      <c r="O13" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P13" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>1</v>
       </c>
@@ -2157,23 +2421,26 @@
       <c r="I14" t="s">
         <v>110</v>
       </c>
-      <c r="J14" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="L14" s="1">
-        <v>1</v>
-      </c>
-      <c r="M14" t="s">
+      <c r="J14" t="s">
+        <v>58</v>
+      </c>
+      <c r="K14" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M14" s="1">
+        <v>1</v>
+      </c>
+      <c r="N14" t="s">
         <v>15</v>
       </c>
-      <c r="N14" t="s">
+      <c r="O14" t="s">
         <v>11</v>
       </c>
-      <c r="O14" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P14" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>2</v>
       </c>
@@ -2198,23 +2465,26 @@
       <c r="I15" t="s">
         <v>111</v>
       </c>
-      <c r="J15" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="L15" s="1">
+      <c r="J15" t="s">
+        <v>58</v>
+      </c>
+      <c r="K15" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M15" s="1">
         <v>2</v>
       </c>
-      <c r="M15" t="s">
+      <c r="N15" t="s">
         <v>16</v>
       </c>
-      <c r="N15" t="s">
+      <c r="O15" t="s">
         <v>11</v>
       </c>
-      <c r="O15" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="P15" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
         <v>3</v>
       </c>
@@ -2239,19 +2509,22 @@
       <c r="I16" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="J16" s="5" t="b">
+      <c r="J16" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="K16" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="L16" s="3">
-        <v>3</v>
-      </c>
-      <c r="M16" s="4" t="s">
+      <c r="M16" s="3">
+        <v>3</v>
+      </c>
+      <c r="N16" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="N16" s="4" t="s">
+      <c r="O16" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="O16" s="5" t="b">
+      <c r="P16" s="5" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2444,7 +2717,7 @@
         <v>66</v>
       </c>
       <c r="E27" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F27" t="s">
         <v>35</v>
@@ -2572,7 +2845,7 @@
       <c r="H33" s="20"/>
       <c r="I33" s="21"/>
       <c r="K33" s="19" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="L33" s="20"/>
       <c r="M33" s="20"/>
@@ -2752,13 +3025,13 @@
       <c r="D40" s="20"/>
       <c r="E40" s="20"/>
       <c r="F40" s="21"/>
-      <c r="H40" s="22" t="s">
-        <v>116</v>
-      </c>
-      <c r="I40" s="23"/>
-      <c r="J40" s="23"/>
-      <c r="K40" s="23"/>
-      <c r="L40" s="24"/>
+      <c r="H40" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="I40" s="20"/>
+      <c r="J40" s="20"/>
+      <c r="K40" s="20"/>
+      <c r="L40" s="21"/>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
@@ -2783,13 +3056,13 @@
         <v>1</v>
       </c>
       <c r="I41" t="s">
+        <v>116</v>
+      </c>
+      <c r="J41" t="s">
         <v>117</v>
       </c>
-      <c r="J41" t="s">
+      <c r="K41" t="s">
         <v>118</v>
-      </c>
-      <c r="K41" t="s">
-        <v>119</v>
       </c>
       <c r="L41" s="2" t="s">
         <v>3</v>
@@ -2821,7 +3094,7 @@
         <v>1</v>
       </c>
       <c r="J42" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="K42" t="s">
         <v>11</v>
@@ -2856,7 +3129,7 @@
         <v>1</v>
       </c>
       <c r="J43" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="K43" t="s">
         <v>11</v>
@@ -2888,10 +3161,10 @@
         <v>3</v>
       </c>
       <c r="I44" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="K44" s="4" t="s">
         <v>11</v>
@@ -3190,337 +3463,865 @@
     </row>
     <row r="60" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="61" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A61" s="22" t="s">
+      <c r="A61" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="B61" s="20"/>
+      <c r="C61" s="20"/>
+      <c r="D61" s="20"/>
+      <c r="E61" s="21"/>
+      <c r="G61" s="19" t="s">
         <v>136</v>
       </c>
-      <c r="B61" s="23"/>
-      <c r="C61" s="23"/>
-      <c r="D61" s="23"/>
-      <c r="E61" s="24"/>
-      <c r="G61" s="22" t="s">
-        <v>137</v>
-      </c>
-      <c r="H61" s="23"/>
-      <c r="I61" s="23"/>
-      <c r="J61" s="23"/>
-      <c r="K61" s="24"/>
+      <c r="H61" s="20"/>
+      <c r="I61" s="20"/>
+      <c r="J61" s="20"/>
+      <c r="K61" s="21"/>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A62" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="B62" s="25" t="s">
-        <v>139</v>
-      </c>
-      <c r="C62" s="25" t="s">
+      <c r="A62" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B62" t="s">
+        <v>138</v>
+      </c>
+      <c r="C62" t="s">
         <v>37</v>
       </c>
-      <c r="D62" s="25" t="s">
+      <c r="D62" t="s">
         <v>39</v>
       </c>
-      <c r="E62" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="G62" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="H62" s="25" t="s">
-        <v>139</v>
-      </c>
-      <c r="I62" s="25" t="s">
+      <c r="E62" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G62" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H62" t="s">
+        <v>138</v>
+      </c>
+      <c r="I62" t="s">
         <v>37</v>
       </c>
-      <c r="J62" s="25" t="s">
+      <c r="J62" t="s">
         <v>90</v>
       </c>
-      <c r="K62" s="14" t="s">
+      <c r="K62" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A63" s="13">
-        <v>1</v>
-      </c>
-      <c r="B63" s="25">
-        <v>1</v>
-      </c>
-      <c r="C63" s="25" t="s">
-        <v>123</v>
-      </c>
-      <c r="D63" s="25" t="str">
+      <c r="A63" s="1">
+        <v>1</v>
+      </c>
+      <c r="B63">
+        <v>1</v>
+      </c>
+      <c r="C63" t="s">
+        <v>122</v>
+      </c>
+      <c r="D63" t="str">
         <f>CONCATENATE(C63,"@andez.com.ar")</f>
         <v>Compras@andez.com.ar</v>
       </c>
-      <c r="E63" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="G63" s="13">
-        <v>1</v>
-      </c>
-      <c r="H63" s="25">
-        <v>1</v>
-      </c>
-      <c r="I63" s="25" t="s">
-        <v>126</v>
-      </c>
-      <c r="J63" s="25">
+      <c r="E63" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G63" s="1">
+        <v>1</v>
+      </c>
+      <c r="H63">
+        <v>1</v>
+      </c>
+      <c r="I63" t="s">
+        <v>125</v>
+      </c>
+      <c r="J63">
         <v>45552646</v>
       </c>
-      <c r="K63" s="14" t="b">
+      <c r="K63" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A64" s="13">
+      <c r="A64" s="1">
         <v>2</v>
       </c>
-      <c r="B64" s="25">
-        <v>1</v>
-      </c>
-      <c r="C64" s="25" t="s">
-        <v>124</v>
-      </c>
-      <c r="D64" s="25" t="str">
+      <c r="B64">
+        <v>1</v>
+      </c>
+      <c r="C64" t="s">
+        <v>123</v>
+      </c>
+      <c r="D64" t="str">
         <f t="shared" ref="D64:D65" si="0">CONCATENATE(C64,"@andez.com.ar")</f>
         <v>RRHH@andez.com.ar</v>
       </c>
-      <c r="E64" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="G64" s="13">
+      <c r="E64" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G64" s="1">
         <v>2</v>
       </c>
-      <c r="H64" s="25">
-        <v>1</v>
-      </c>
-      <c r="I64" s="25" t="s">
-        <v>127</v>
-      </c>
-      <c r="J64" s="25">
+      <c r="H64">
+        <v>1</v>
+      </c>
+      <c r="I64" t="s">
+        <v>126</v>
+      </c>
+      <c r="J64">
         <v>45552646</v>
       </c>
-      <c r="K64" s="14" t="b">
+      <c r="K64" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="65" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A65" s="15">
-        <v>3</v>
-      </c>
-      <c r="B65" s="16">
-        <v>1</v>
-      </c>
-      <c r="C65" s="16" t="s">
-        <v>125</v>
-      </c>
-      <c r="D65" s="16" t="str">
+      <c r="A65" s="3">
+        <v>3</v>
+      </c>
+      <c r="B65" s="4">
+        <v>1</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D65" s="4" t="str">
         <f t="shared" si="0"/>
         <v>Ventas@andez.com.ar</v>
       </c>
-      <c r="E65" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="G65" s="15">
-        <v>3</v>
-      </c>
-      <c r="H65" s="16">
-        <v>1</v>
-      </c>
-      <c r="I65" s="16" t="s">
-        <v>128</v>
-      </c>
-      <c r="J65" s="16">
+      <c r="E65" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G65" s="3">
+        <v>3</v>
+      </c>
+      <c r="H65" s="4">
+        <v>1</v>
+      </c>
+      <c r="I65" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="J65" s="4">
         <v>1545552646</v>
       </c>
-      <c r="K65" s="17" t="b">
+      <c r="K65" s="5" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="67" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="68" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A68" s="22" t="s">
+      <c r="A68" s="19" t="s">
+        <v>137</v>
+      </c>
+      <c r="B68" s="20"/>
+      <c r="C68" s="20"/>
+      <c r="D68" s="20"/>
+      <c r="E68" s="21"/>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A69" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B69" t="s">
         <v>138</v>
       </c>
-      <c r="B68" s="23"/>
-      <c r="C68" s="23"/>
-      <c r="D68" s="23"/>
-      <c r="E68" s="24"/>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A69" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="B69" s="25" t="s">
-        <v>139</v>
-      </c>
-      <c r="C69" s="25" t="s">
+      <c r="C69" t="s">
+        <v>128</v>
+      </c>
+      <c r="D69" t="s">
         <v>129</v>
       </c>
-      <c r="D69" s="25" t="s">
+      <c r="E69" s="13" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A70" s="1">
+        <v>1</v>
+      </c>
+      <c r="B70">
+        <v>1</v>
+      </c>
+      <c r="C70" t="s">
+        <v>131</v>
+      </c>
+      <c r="D70" t="s">
+        <v>11</v>
+      </c>
+      <c r="E70" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A71" s="1">
+        <v>2</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
         <v>130</v>
       </c>
-      <c r="E69" s="18" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A70" s="13">
-        <v>1</v>
-      </c>
-      <c r="B70" s="25">
-        <v>1</v>
-      </c>
-      <c r="C70" s="25" t="s">
+      <c r="D71" t="s">
+        <v>11</v>
+      </c>
+      <c r="E71" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A72" s="3">
+        <v>3</v>
+      </c>
+      <c r="B72" s="4">
+        <v>1</v>
+      </c>
+      <c r="C72" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="D70" s="25" t="s">
+      <c r="D72" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E70" s="14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A71" s="13">
-        <v>2</v>
-      </c>
-      <c r="B71" s="25">
-        <v>1</v>
-      </c>
-      <c r="C71" s="25" t="s">
-        <v>131</v>
-      </c>
-      <c r="D71" s="25" t="s">
-        <v>11</v>
-      </c>
-      <c r="E71" s="14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A72" s="15">
-        <v>3</v>
-      </c>
-      <c r="B72" s="16">
-        <v>1</v>
-      </c>
-      <c r="C72" s="16" t="s">
-        <v>133</v>
-      </c>
-      <c r="D72" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="E72" s="17" t="b">
+      <c r="E72" s="5" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="74" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="75" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A75" s="22" t="s">
+      <c r="A75" s="19" t="s">
+        <v>139</v>
+      </c>
+      <c r="B75" s="20"/>
+      <c r="C75" s="20"/>
+      <c r="D75" s="20"/>
+      <c r="E75" s="20"/>
+      <c r="F75" s="20"/>
+      <c r="G75" s="20"/>
+      <c r="H75" s="20"/>
+      <c r="I75" s="20"/>
+      <c r="J75" s="21"/>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A76" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B76" t="s">
+        <v>87</v>
+      </c>
+      <c r="C76" t="s">
+        <v>141</v>
+      </c>
+      <c r="D76" t="s">
+        <v>88</v>
+      </c>
+      <c r="E76" t="s">
+        <v>144</v>
+      </c>
+      <c r="F76" t="s">
+        <v>146</v>
+      </c>
+      <c r="G76" t="s">
+        <v>89</v>
+      </c>
+      <c r="H76" t="s">
+        <v>148</v>
+      </c>
+      <c r="I76" t="s">
+        <v>150</v>
+      </c>
+      <c r="J76" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A77" s="3">
+        <v>1</v>
+      </c>
+      <c r="B77" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="B75" s="23"/>
-      <c r="C75" s="23"/>
-      <c r="D75" s="23"/>
-      <c r="E75" s="23"/>
-      <c r="F75" s="23"/>
-      <c r="G75" s="23"/>
-      <c r="H75" s="23"/>
-      <c r="I75" s="23"/>
-      <c r="J75" s="24"/>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A76" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="B76" s="25" t="s">
-        <v>87</v>
-      </c>
-      <c r="C76" s="25" t="s">
+      <c r="C77" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="D76" s="25" t="s">
-        <v>88</v>
-      </c>
-      <c r="E76" s="25" t="s">
+      <c r="D77" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="E77" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="F76" s="25" t="s">
+      <c r="F77" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="G76" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="H76" s="25" t="s">
+      <c r="G77" s="4">
+        <v>2</v>
+      </c>
+      <c r="H77" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="I76" s="25" t="s">
+      <c r="I77" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="J76" s="14" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A77" s="15">
-        <v>1</v>
-      </c>
-      <c r="B77" s="16" t="s">
-        <v>141</v>
-      </c>
-      <c r="C77" s="16" t="s">
-        <v>143</v>
-      </c>
-      <c r="D77" s="16" t="s">
-        <v>144</v>
-      </c>
-      <c r="E77" s="16" t="s">
-        <v>146</v>
-      </c>
-      <c r="F77" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="G77" s="16">
+      <c r="J77" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A80" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="B80" s="20"/>
+      <c r="C80" s="20"/>
+      <c r="D80" s="20"/>
+      <c r="E80" s="20"/>
+      <c r="F80" s="20"/>
+      <c r="G80" s="20"/>
+      <c r="H80" s="20"/>
+      <c r="I80" s="20"/>
+      <c r="J80" s="20"/>
+      <c r="K80" s="21"/>
+    </row>
+    <row r="81" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A81" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B81" t="s">
+        <v>154</v>
+      </c>
+      <c r="C81" t="s">
+        <v>37</v>
+      </c>
+      <c r="D81" t="s">
+        <v>118</v>
+      </c>
+      <c r="E81" t="s">
+        <v>117</v>
+      </c>
+      <c r="F81" t="s">
+        <v>57</v>
+      </c>
+      <c r="G81" t="s">
+        <v>155</v>
+      </c>
+      <c r="H81" t="s">
+        <v>156</v>
+      </c>
+      <c r="I81" t="s">
+        <v>157</v>
+      </c>
+      <c r="J81" t="s">
+        <v>158</v>
+      </c>
+      <c r="K81" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="82" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A82" s="1">
+        <v>1</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>159</v>
+      </c>
+      <c r="D82" t="s">
+        <v>11</v>
+      </c>
+      <c r="E82" t="s">
+        <v>162</v>
+      </c>
+      <c r="F82" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="G82" t="s">
+        <v>11</v>
+      </c>
+      <c r="H82" t="b">
+        <v>1</v>
+      </c>
+      <c r="I82" t="b">
+        <v>1</v>
+      </c>
+      <c r="J82" t="b">
+        <v>0</v>
+      </c>
+      <c r="K82" s="8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A83" s="1">
         <v>2</v>
       </c>
-      <c r="H77" s="16" t="s">
-        <v>150</v>
-      </c>
-      <c r="I77" s="16" t="s">
-        <v>152</v>
-      </c>
-      <c r="J77" s="17" t="b">
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>160</v>
+      </c>
+      <c r="D83" t="s">
+        <v>11</v>
+      </c>
+      <c r="E83" t="s">
+        <v>163</v>
+      </c>
+      <c r="F83" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="G83" t="s">
+        <v>165</v>
+      </c>
+      <c r="H83" t="b">
+        <v>0</v>
+      </c>
+      <c r="I83" t="b">
+        <v>0</v>
+      </c>
+      <c r="J83" t="b">
+        <v>0</v>
+      </c>
+      <c r="K83" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A84" s="3">
+        <v>3</v>
+      </c>
+      <c r="B84" s="4">
+        <v>3</v>
+      </c>
+      <c r="C84" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="D84" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E84" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="F84" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="G84" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H84" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I84" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="J84" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="K84" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="87" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A87" s="16" t="s">
+        <v>170</v>
+      </c>
+      <c r="B87" s="18"/>
+      <c r="D87" s="16" t="s">
+        <v>173</v>
+      </c>
+      <c r="E87" s="17"/>
+      <c r="F87" s="18"/>
+      <c r="H87" s="16" t="s">
+        <v>189</v>
+      </c>
+      <c r="I87" s="17"/>
+      <c r="J87" s="18"/>
+    </row>
+    <row r="88" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A88" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="D88" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E88" t="s">
+        <v>37</v>
+      </c>
+      <c r="F88" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H88" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I88" t="s">
+        <v>189</v>
+      </c>
+      <c r="J88" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="89" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A89" s="1">
+        <v>1</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="D89" s="1">
+        <v>1</v>
+      </c>
+      <c r="E89" t="s">
+        <v>117</v>
+      </c>
+      <c r="F89" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H89" s="1">
+        <v>1</v>
+      </c>
+      <c r="I89" t="s">
+        <v>190</v>
+      </c>
+      <c r="J89" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A90" s="1">
+        <v>2</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D90" s="1">
+        <v>2</v>
+      </c>
+      <c r="E90" t="s">
+        <v>174</v>
+      </c>
+      <c r="F90" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H90" s="1">
+        <v>2</v>
+      </c>
+      <c r="I90" t="s">
+        <v>191</v>
+      </c>
+      <c r="J90" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A91" s="3">
+        <v>3</v>
+      </c>
+      <c r="B91" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D91" s="3">
+        <v>3</v>
+      </c>
+      <c r="E91" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="F91" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H91" s="3">
+        <v>3</v>
+      </c>
+      <c r="I91" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="J91" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="94" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A94" s="16" t="s">
+        <v>166</v>
+      </c>
+      <c r="B94" s="17"/>
+      <c r="C94" s="17"/>
+      <c r="D94" s="17"/>
+      <c r="E94" s="17"/>
+      <c r="F94" s="17"/>
+      <c r="G94" s="17"/>
+      <c r="H94" s="17"/>
+      <c r="I94" s="17"/>
+      <c r="J94" s="17"/>
+      <c r="K94" s="17"/>
+      <c r="L94" s="17"/>
+      <c r="M94" s="17"/>
+      <c r="N94" s="17"/>
+      <c r="O94" s="18"/>
+    </row>
+    <row r="95" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A95" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B95" t="s">
+        <v>91</v>
+      </c>
+      <c r="C95" t="s">
+        <v>188</v>
+      </c>
+      <c r="D95" t="s">
+        <v>177</v>
+      </c>
+      <c r="E95" t="s">
+        <v>178</v>
+      </c>
+      <c r="F95" t="s">
+        <v>179</v>
+      </c>
+      <c r="G95" t="s">
+        <v>180</v>
+      </c>
+      <c r="H95" t="s">
+        <v>182</v>
+      </c>
+      <c r="I95" t="s">
+        <v>181</v>
+      </c>
+      <c r="J95" t="s">
+        <v>183</v>
+      </c>
+      <c r="K95" t="s">
+        <v>184</v>
+      </c>
+      <c r="L95" t="s">
+        <v>185</v>
+      </c>
+      <c r="M95" t="s">
+        <v>186</v>
+      </c>
+      <c r="N95" t="s">
+        <v>187</v>
+      </c>
+      <c r="O95" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="96" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A96" s="1">
+        <v>1</v>
+      </c>
+      <c r="B96">
+        <v>1</v>
+      </c>
+      <c r="C96" t="s">
+        <v>11</v>
+      </c>
+      <c r="O96" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A97" s="1">
+        <v>2</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>11</v>
+      </c>
+      <c r="O97" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A98" s="3">
+        <v>3</v>
+      </c>
+      <c r="B98" s="4">
+        <v>3</v>
+      </c>
+      <c r="C98" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D98" s="4"/>
+      <c r="E98" s="4"/>
+      <c r="F98" s="4"/>
+      <c r="G98" s="4"/>
+      <c r="H98" s="4"/>
+      <c r="I98" s="4"/>
+      <c r="J98" s="4"/>
+      <c r="K98" s="4"/>
+      <c r="L98" s="4"/>
+      <c r="M98" s="4"/>
+      <c r="N98" s="4"/>
+      <c r="O98" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="101" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A101" s="16" t="s">
+        <v>176</v>
+      </c>
+      <c r="B101" s="17"/>
+      <c r="C101" s="17"/>
+      <c r="D101" s="18"/>
+    </row>
+    <row r="102" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A102" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B102" t="s">
+        <v>91</v>
+      </c>
+      <c r="C102" t="s">
+        <v>196</v>
+      </c>
+      <c r="D102" t="s">
+        <v>197</v>
+      </c>
+      <c r="E102" t="s">
+        <v>0</v>
+      </c>
+      <c r="F102" t="s">
+        <v>199</v>
+      </c>
+      <c r="G102" t="s">
+        <v>193</v>
+      </c>
+      <c r="H102" t="s">
+        <v>194</v>
+      </c>
+      <c r="I102" t="s">
+        <v>195</v>
+      </c>
+      <c r="J102" t="s">
+        <v>167</v>
+      </c>
+      <c r="K102" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="103" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A103" s="1">
+        <v>1</v>
+      </c>
+      <c r="B103">
+        <v>1</v>
+      </c>
+      <c r="C103">
+        <v>1</v>
+      </c>
+      <c r="D103">
+        <v>1</v>
+      </c>
+      <c r="E103" t="s">
+        <v>198</v>
+      </c>
+      <c r="F103">
+        <v>18</v>
+      </c>
+      <c r="J103" t="s">
+        <v>168</v>
+      </c>
+      <c r="K103" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A104" s="1">
+        <v>2</v>
+      </c>
+      <c r="B104">
+        <v>1</v>
+      </c>
+      <c r="C104">
+        <v>2</v>
+      </c>
+      <c r="D104">
+        <v>3</v>
+      </c>
+      <c r="E104" t="s">
+        <v>198</v>
+      </c>
+      <c r="F104">
+        <v>12</v>
+      </c>
+      <c r="J104" t="s">
+        <v>11</v>
+      </c>
+      <c r="K104" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A105" s="3">
+        <v>3</v>
+      </c>
+      <c r="B105" s="4">
+        <v>2</v>
+      </c>
+      <c r="C105" s="4">
+        <v>1</v>
+      </c>
+      <c r="D105" s="4">
+        <v>1</v>
+      </c>
+      <c r="E105" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="F105" s="4">
+        <v>18</v>
+      </c>
+      <c r="G105" s="4"/>
+      <c r="H105" s="4"/>
+      <c r="I105" s="4"/>
+      <c r="J105" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="K105" s="5" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="26">
+    <mergeCell ref="A87:B87"/>
+    <mergeCell ref="D87:F87"/>
+    <mergeCell ref="A101:D101"/>
+    <mergeCell ref="A80:K80"/>
+    <mergeCell ref="A94:O94"/>
+    <mergeCell ref="H87:J87"/>
+    <mergeCell ref="A61:E61"/>
+    <mergeCell ref="G61:K61"/>
+    <mergeCell ref="A68:E68"/>
+    <mergeCell ref="A75:J75"/>
+    <mergeCell ref="M12:P12"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A33:I33"/>
+    <mergeCell ref="K33:N33"/>
     <mergeCell ref="A47:D47"/>
     <mergeCell ref="I26:K26"/>
     <mergeCell ref="F47:L47"/>
     <mergeCell ref="H40:L40"/>
     <mergeCell ref="A54:I54"/>
     <mergeCell ref="A40:F40"/>
-    <mergeCell ref="A61:E61"/>
-    <mergeCell ref="G61:K61"/>
-    <mergeCell ref="A68:E68"/>
-    <mergeCell ref="A75:J75"/>
-    <mergeCell ref="L12:O12"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A33:I33"/>
     <mergeCell ref="I5:K5"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="G12:J12"/>
     <mergeCell ref="A26:G26"/>
     <mergeCell ref="F19:L19"/>
-    <mergeCell ref="K33:N33"/>
+    <mergeCell ref="G12:K12"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
-  <tableParts count="20">
+  <tableParts count="26">
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
     <tablePart r:id="rId5"/>
@@ -3541,6 +4342,12 @@
     <tablePart r:id="rId20"/>
     <tablePart r:id="rId21"/>
     <tablePart r:id="rId22"/>
+    <tablePart r:id="rId23"/>
+    <tablePart r:id="rId24"/>
+    <tablePart r:id="rId25"/>
+    <tablePart r:id="rId26"/>
+    <tablePart r:id="rId27"/>
+    <tablePart r:id="rId28"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Se agregan parrafos aclaratorios y mensajes de verificación en las páginas del CMS Diseño. Tambien se unifica el formato del texto de información.
</commit_message>
<xml_diff>
--- a/BBDD.xlsx
+++ b/BBDD.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyectos\Web_Andez\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C629E76-CA29-4CFC-A0EE-C5CC25ED779D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1DF4339-99C7-4AAB-8AAB-4C5C28C64006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5D42B345-DB14-48C1-9A38-23908D3120ED}"/>
   </bookViews>
@@ -118,7 +118,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="205">
   <si>
     <t>Color</t>
   </si>
@@ -615,21 +615,6 @@
     <t>Linea Match</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>Background</t>
-  </si>
-  <si>
-    <t>URLoCodigoHexadecimal</t>
-  </si>
-  <si>
-    <t>#F54927</t>
-  </si>
-  <si>
-    <t>#19548A</t>
-  </si>
-  <si>
     <t>Paginas</t>
   </si>
   <si>
@@ -648,9 +633,6 @@
     <t>Frase</t>
   </si>
   <si>
-    <t>TextoPagina</t>
-  </si>
-  <si>
     <t>ColorGradiente1</t>
   </si>
   <si>
@@ -696,18 +678,6 @@
     <t>Time New Romans</t>
   </si>
   <si>
-    <t>Aptos Narrow</t>
-  </si>
-  <si>
-    <t>Columna5</t>
-  </si>
-  <si>
-    <t>Columna6</t>
-  </si>
-  <si>
-    <t>Columna7</t>
-  </si>
-  <si>
     <t>IdTipoTexto</t>
   </si>
   <si>
@@ -718,6 +688,51 @@
   </si>
   <si>
     <t>Tamaño</t>
+  </si>
+  <si>
+    <t>Publicada</t>
+  </si>
+  <si>
+    <t>NULL</t>
+  </si>
+  <si>
+    <t>Mayuscula</t>
+  </si>
+  <si>
+    <t>Espaciado</t>
+  </si>
+  <si>
+    <t>IdBackground</t>
+  </si>
+  <si>
+    <t>EdicionTexto</t>
+  </si>
+  <si>
+    <t>EdicionBackground</t>
+  </si>
+  <si>
+    <t>IdEdicionTexto</t>
+  </si>
+  <si>
+    <t>DisenioPaginas</t>
+  </si>
+  <si>
+    <t>URLFuente</t>
+  </si>
+  <si>
+    <t>Arial, Helvetica, sans-serif</t>
+  </si>
+  <si>
+    <t>'Times New Roman', Times, serif</t>
+  </si>
+  <si>
+    <t>Courier New</t>
+  </si>
+  <si>
+    <t>'Courier New', Courier, monospace</t>
+  </si>
+  <si>
+    <t>Declaracion</t>
   </si>
 </sst>
 </file>
@@ -884,7 +899,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -899,8 +914,8 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -919,6 +934,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1481,13 +1497,14 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{EF32F6B3-AC45-462F-BE18-EFE2DD57FE9B}" name="Tabla17" displayName="Tabla17" ref="H41:L44" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50">
-  <autoFilter ref="H41:L44" xr:uid="{EF32F6B3-AC45-462F-BE18-EFE2DD57FE9B}"/>
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{EF32F6B3-AC45-462F-BE18-EFE2DD57FE9B}" name="Tabla17" displayName="Tabla17" ref="H41:M44" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50">
+  <autoFilter ref="H41:M44" xr:uid="{EF32F6B3-AC45-462F-BE18-EFE2DD57FE9B}"/>
+  <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{C8F6ED57-5FD2-4FB3-A4A5-BC3965E98B15}" name="ID" dataDxfId="49"/>
     <tableColumn id="2" xr3:uid="{65B99387-EDCD-429B-B81B-A4F58479A304}" name="IdProducto" dataDxfId="48"/>
     <tableColumn id="3" xr3:uid="{5D9C0348-2DF4-47CC-977C-AAFB9F19E959}" name="Titulo" dataDxfId="47"/>
     <tableColumn id="4" xr3:uid="{1CACB54F-DC9D-41AC-A04F-171EF34060DC}" name="URLImagen" dataDxfId="46"/>
+    <tableColumn id="5" xr3:uid="{E836C9A1-0FCD-4424-8667-FBB476A992FD}" name="Publicada"/>
     <tableColumn id="7" xr3:uid="{824500A6-D872-42FD-9C38-60CB54869E2F}" name="Activo" dataDxfId="45"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1634,11 +1651,12 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{93610188-F7B2-40FB-B0A9-E18135492A82}" name="Tabla7" displayName="Tabla7" ref="A81:K84" totalsRowShown="0">
-  <autoFilter ref="A81:K84" xr:uid="{93610188-F7B2-40FB-B0A9-E18135492A82}"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{93610188-F7B2-40FB-B0A9-E18135492A82}" name="Tabla7" displayName="Tabla7" ref="A81:L84" totalsRowShown="0">
+  <autoFilter ref="A81:L84" xr:uid="{93610188-F7B2-40FB-B0A9-E18135492A82}"/>
+  <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{1035A3C3-56C5-4CB6-B2AD-211341406B65}" name="ID"/>
     <tableColumn id="2" xr3:uid="{A5D7D600-3A71-4DD1-A6A0-88B6463C987F}" name="Posicion"/>
+    <tableColumn id="12" xr3:uid="{0DCF8682-7649-4A42-B056-5C7F147FE3A0}" name="IdEdicionTexto"/>
     <tableColumn id="3" xr3:uid="{473E571D-8BE9-4BD5-B8BD-FC16062FBA4A}" name="Nombre"/>
     <tableColumn id="4" xr3:uid="{BFCDC025-7291-43F4-BF51-02B5C205C0B1}" name="URLImagen"/>
     <tableColumn id="5" xr3:uid="{1AD6DCB5-B8FB-43FC-88CE-E58B0DF75376}" name="Titulo"/>
@@ -1654,11 +1672,10 @@
 </file>
 
 <file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{68E94E33-CBEB-416E-8BE1-18A7BBEB19B8}" name="Tabla8" displayName="Tabla8" ref="A95:O98" totalsRowShown="0">
-  <autoFilter ref="A95:O98" xr:uid="{68E94E33-CBEB-416E-8BE1-18A7BBEB19B8}"/>
-  <tableColumns count="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{68E94E33-CBEB-416E-8BE1-18A7BBEB19B8}" name="Tabla8" displayName="Tabla8" ref="A95:N98" totalsRowShown="0">
+  <autoFilter ref="A95:N98" xr:uid="{68E94E33-CBEB-416E-8BE1-18A7BBEB19B8}"/>
+  <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{1E8CA238-3595-4186-9A14-6CF4E7344108}" name="ID"/>
-    <tableColumn id="4" xr3:uid="{461BF0D3-CF94-41A1-8339-A826048D1E99}" name="IdPagina"/>
     <tableColumn id="5" xr3:uid="{7E4F1EF2-7520-4E68-B2FD-D184EC1CB1C3}" name="URLBackground"/>
     <tableColumn id="6" xr3:uid="{6C881594-A7F4-46D3-A368-B8C8A77D11C3}" name="ColorGradiente1"/>
     <tableColumn id="7" xr3:uid="{9B4B354C-8699-4AA2-9FD9-649842AE57D0}" name="ColorGradiente2"/>
@@ -1701,19 +1718,17 @@
 </file>
 
 <file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{603B1BB5-0E4C-4377-B4E9-1203B7A1C3FB}" name="Tabla826" displayName="Tabla826" ref="A102:K105" totalsRowShown="0">
-  <autoFilter ref="A102:K105" xr:uid="{603B1BB5-0E4C-4377-B4E9-1203B7A1C3FB}"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{603B1BB5-0E4C-4377-B4E9-1203B7A1C3FB}" name="Tabla826" displayName="Tabla826" ref="A102:I105" totalsRowShown="0">
+  <autoFilter ref="A102:I105" xr:uid="{603B1BB5-0E4C-4377-B4E9-1203B7A1C3FB}"/>
+  <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{62362053-8A80-4FF4-AB6D-40430AC5A5F4}" name="ID"/>
-    <tableColumn id="4" xr3:uid="{794753EA-92E6-4DA1-AA5F-DD6E6EE6ED37}" name="IdPagina"/>
     <tableColumn id="5" xr3:uid="{7B2052E1-C43E-4046-BE46-97E55A7FBE0F}" name="IdTipoTexto"/>
     <tableColumn id="6" xr3:uid="{A93952EC-78FC-4DD0-B380-1E659DE63DFD}" name="IdFuente"/>
     <tableColumn id="7" xr3:uid="{BB786B7B-E29D-4A14-B248-C9584ED0A547}" name="Color"/>
     <tableColumn id="8" xr3:uid="{FFCC595A-F6A5-43DB-94E4-BD4E0394F4ED}" name="Tamaño"/>
-    <tableColumn id="9" xr3:uid="{A8921874-6C7F-4FBA-936A-D4B602C93F67}" name="Columna5"/>
-    <tableColumn id="10" xr3:uid="{AF446AA5-2F2C-4048-99E1-18C03C00DFCF}" name="Columna6"/>
-    <tableColumn id="11" xr3:uid="{4DD925C6-883F-40E6-911F-7E9E42C2279C}" name="Columna7"/>
-    <tableColumn id="2" xr3:uid="{5FF0673F-C0BF-4E18-815C-61F99F9FEF74}" name="URLoCodigoHexadecimal"/>
+    <tableColumn id="9" xr3:uid="{A8921874-6C7F-4FBA-936A-D4B602C93F67}" name="Mayuscula"/>
+    <tableColumn id="10" xr3:uid="{AF446AA5-2F2C-4048-99E1-18C03C00DFCF}" name="Contraste"/>
+    <tableColumn id="11" xr3:uid="{4DD925C6-883F-40E6-911F-7E9E42C2279C}" name="Espaciado"/>
     <tableColumn id="3" xr3:uid="{3715AA2C-BDFD-4A0F-9EEC-4D0E838CD882}" name="Activo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1721,12 +1736,28 @@
 </file>
 
 <file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="26" xr:uid="{0B42635A-3ED7-432B-A4A5-0CA9F365C85C}" name="Tabla232527" displayName="Tabla232527" ref="H88:J91" totalsRowShown="0">
-  <autoFilter ref="H88:J91" xr:uid="{0B42635A-3ED7-432B-A4A5-0CA9F365C85C}"/>
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="26" xr:uid="{0B42635A-3ED7-432B-A4A5-0CA9F365C85C}" name="Tabla232527" displayName="Tabla232527" ref="H88:L91" totalsRowShown="0">
+  <autoFilter ref="H88:L91" xr:uid="{0B42635A-3ED7-432B-A4A5-0CA9F365C85C}"/>
+  <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{3FA20A71-CF47-4DAB-951A-7C4FC5084311}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{79A7F6F7-1859-4BB3-B79B-BFF30483BAB2}" name="Fuente"/>
+    <tableColumn id="2" xr3:uid="{79A7F6F7-1859-4BB3-B79B-BFF30483BAB2}" name="Nombre"/>
+    <tableColumn id="5" xr3:uid="{48F19664-7170-46E7-8830-804ED59C4F30}" name="Declaracion"/>
+    <tableColumn id="4" xr3:uid="{098E8492-CDA9-4DF7-B3B0-2DABDE9A52CD}" name="URLFuente"/>
     <tableColumn id="3" xr3:uid="{F7077B09-954A-4A25-96B1-3B3866C4F1D9}" name="Activo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{B5376336-314C-4E5C-9773-BCBED3F2A22E}" name="Tabla27" displayName="Tabla27" ref="A109:E112" totalsRowShown="0">
+  <autoFilter ref="A109:E112" xr:uid="{B5376336-314C-4E5C-9773-BCBED3F2A22E}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{5FE15933-BCF6-468F-AF7F-09630168B046}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{B7750034-1E27-4E92-856C-30E5F48E7B9E}" name="IdPagina"/>
+    <tableColumn id="3" xr3:uid="{61419E12-5C48-471B-A94C-365D61B394C2}" name="IdBackground"/>
+    <tableColumn id="4" xr3:uid="{3B4A719A-180B-4B39-9C10-B58CA3A5C88C}" name="IdEdicionTexto"/>
+    <tableColumn id="5" xr3:uid="{4B5372AE-F961-4286-86FB-E03ECC3B0166}" name="Activo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2149,20 +2180,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD350C1D-1850-4BF9-ABCF-FA1A23EC1542}">
-  <dimension ref="A1:P105"/>
+  <dimension ref="A1:P112"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="28.77734375" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="24.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="26.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.88671875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.5546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="27.21875" bestFit="1" customWidth="1"/>
     <col min="11" max="12" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="18.109375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="12.21875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11.33203125" bestFit="1" customWidth="1"/>
@@ -3031,7 +3062,8 @@
       <c r="I40" s="20"/>
       <c r="J40" s="20"/>
       <c r="K40" s="20"/>
-      <c r="L40" s="21"/>
+      <c r="L40" s="20"/>
+      <c r="M40" s="21"/>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
@@ -3064,7 +3096,10 @@
       <c r="K41" t="s">
         <v>118</v>
       </c>
-      <c r="L41" s="2" t="s">
+      <c r="L41" t="s">
+        <v>190</v>
+      </c>
+      <c r="M41" s="2" t="s">
         <v>3</v>
       </c>
     </row>
@@ -3099,7 +3134,10 @@
       <c r="K42" t="s">
         <v>11</v>
       </c>
-      <c r="L42" s="2" t="b">
+      <c r="L42" t="b">
+        <v>1</v>
+      </c>
+      <c r="M42" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3134,7 +3172,10 @@
       <c r="K43" t="s">
         <v>11</v>
       </c>
-      <c r="L43" s="2" t="b">
+      <c r="L43" t="b">
+        <v>1</v>
+      </c>
+      <c r="M43" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3169,7 +3210,10 @@
       <c r="K44" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="L44" s="5" t="b">
+      <c r="L44" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="M44" s="5" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3554,7 +3598,7 @@
         <v>123</v>
       </c>
       <c r="D64" t="str">
-        <f t="shared" ref="D64:D65" si="0">CONCATENATE(C64,"@andez.com.ar")</f>
+        <f>CONCATENATE(C64,"@andez.com.ar")</f>
         <v>RRHH@andez.com.ar</v>
       </c>
       <c r="E64" s="2" t="b">
@@ -3576,7 +3620,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A65" s="3">
         <v>3</v>
       </c>
@@ -3587,7 +3631,7 @@
         <v>124</v>
       </c>
       <c r="D65" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(C65,"@andez.com.ar")</f>
         <v>Ventas@andez.com.ar</v>
       </c>
       <c r="E65" s="5" t="b">
@@ -3609,8 +3653,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A68" s="19" t="s">
         <v>137</v>
       </c>
@@ -3619,7 +3663,7 @@
       <c r="D68" s="20"/>
       <c r="E68" s="21"/>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
         <v>1</v>
       </c>
@@ -3636,7 +3680,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A70" s="1">
         <v>1</v>
       </c>
@@ -3653,7 +3697,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A71" s="1">
         <v>2</v>
       </c>
@@ -3670,7 +3714,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A72" s="3">
         <v>3</v>
       </c>
@@ -3687,8 +3731,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A75" s="19" t="s">
         <v>139</v>
       </c>
@@ -3702,7 +3746,7 @@
       <c r="I75" s="20"/>
       <c r="J75" s="21"/>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
         <v>1</v>
       </c>
@@ -3734,7 +3778,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="77" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A77" s="3">
         <v>1</v>
       </c>
@@ -3766,8 +3810,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="80" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A80" s="19" t="s">
         <v>153</v>
       </c>
@@ -3780,9 +3824,10 @@
       <c r="H80" s="20"/>
       <c r="I80" s="20"/>
       <c r="J80" s="20"/>
-      <c r="K80" s="21"/>
-    </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="K80" s="20"/>
+      <c r="L80" s="21"/>
+    </row>
+    <row r="81" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
         <v>1</v>
       </c>
@@ -3790,92 +3835,98 @@
         <v>154</v>
       </c>
       <c r="C81" t="s">
+        <v>197</v>
+      </c>
+      <c r="D81" t="s">
         <v>37</v>
       </c>
-      <c r="D81" t="s">
+      <c r="E81" t="s">
         <v>118</v>
       </c>
-      <c r="E81" t="s">
+      <c r="F81" t="s">
         <v>117</v>
       </c>
-      <c r="F81" t="s">
+      <c r="G81" t="s">
         <v>57</v>
       </c>
-      <c r="G81" t="s">
+      <c r="H81" t="s">
         <v>155</v>
       </c>
-      <c r="H81" t="s">
+      <c r="I81" t="s">
         <v>156</v>
       </c>
-      <c r="I81" t="s">
+      <c r="J81" t="s">
         <v>157</v>
       </c>
-      <c r="J81" t="s">
+      <c r="K81" t="s">
         <v>158</v>
       </c>
-      <c r="K81" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="L81" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A82" s="1">
         <v>1</v>
       </c>
       <c r="B82">
         <v>1</v>
       </c>
-      <c r="C82" t="s">
+      <c r="C82">
+        <v>1</v>
+      </c>
+      <c r="D82" t="s">
         <v>159</v>
       </c>
-      <c r="D82" t="s">
+      <c r="E82" t="s">
         <v>11</v>
       </c>
-      <c r="E82" t="s">
+      <c r="F82" t="s">
         <v>162</v>
       </c>
-      <c r="F82" s="14" t="s">
+      <c r="G82" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="G82" t="s">
+      <c r="H82" t="s">
         <v>11</v>
       </c>
-      <c r="H82" t="b">
-        <v>1</v>
-      </c>
       <c r="I82" t="b">
         <v>1</v>
       </c>
       <c r="J82" t="b">
+        <v>1</v>
+      </c>
+      <c r="K82" t="b">
         <v>0</v>
       </c>
-      <c r="K82" s="8" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="L82" s="8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A83" s="1">
         <v>2</v>
       </c>
       <c r="B83">
         <v>2</v>
       </c>
-      <c r="C83" t="s">
+      <c r="C83">
+        <v>5</v>
+      </c>
+      <c r="D83" t="s">
         <v>160</v>
       </c>
-      <c r="D83" t="s">
+      <c r="E83" t="s">
         <v>11</v>
       </c>
-      <c r="E83" t="s">
+      <c r="F83" t="s">
         <v>163</v>
       </c>
-      <c r="F83" s="14" t="s">
+      <c r="G83" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="G83" t="s">
-        <v>165</v>
-      </c>
-      <c r="H83" t="b">
-        <v>0</v>
+      <c r="H83" t="s">
+        <v>191</v>
       </c>
       <c r="I83" t="b">
         <v>0</v>
@@ -3883,68 +3934,76 @@
       <c r="J83" t="b">
         <v>0</v>
       </c>
-      <c r="K83" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="84" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K83" t="b">
+        <v>0</v>
+      </c>
+      <c r="L83" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A84" s="3">
         <v>3</v>
       </c>
       <c r="B84" s="4">
         <v>3</v>
       </c>
-      <c r="C84" s="4" t="s">
+      <c r="C84" s="4">
+        <v>2</v>
+      </c>
+      <c r="D84" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="D84" s="4" t="s">
+      <c r="E84" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E84" s="4" t="s">
+      <c r="F84" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="F84" s="15" t="s">
+      <c r="G84" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="G84" s="4" t="s">
+      <c r="H84" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="H84" s="4" t="b">
-        <v>1</v>
-      </c>
       <c r="I84" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J84" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="K84" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="86" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="87" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A87" s="16" t="s">
-        <v>170</v>
-      </c>
-      <c r="B87" s="18"/>
-      <c r="D87" s="16" t="s">
-        <v>173</v>
-      </c>
-      <c r="E87" s="17"/>
-      <c r="F87" s="18"/>
-      <c r="H87" s="16" t="s">
-        <v>189</v>
-      </c>
-      <c r="I87" s="17"/>
-      <c r="J87" s="18"/>
-    </row>
-    <row r="88" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="K84" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L84" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="87" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A87" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="B87" s="21"/>
+      <c r="D87" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="E87" s="20"/>
+      <c r="F87" s="21"/>
+      <c r="H87" s="19" t="s">
+        <v>183</v>
+      </c>
+      <c r="I87" s="20"/>
+      <c r="J87" s="20"/>
+      <c r="K87" s="20"/>
+      <c r="L87" s="21"/>
+    </row>
+    <row r="88" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="D88" s="1" t="s">
         <v>1</v>
@@ -3958,19 +4017,25 @@
       <c r="H88" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="I88" t="s">
-        <v>189</v>
-      </c>
-      <c r="J88" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="89" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="I88" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="J88" s="22" t="s">
+        <v>204</v>
+      </c>
+      <c r="K88" s="22" t="s">
+        <v>199</v>
+      </c>
+      <c r="L88" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="89" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A89" s="1">
         <v>1</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="D89" s="1">
         <v>1</v>
@@ -3984,14 +4049,20 @@
       <c r="H89" s="1">
         <v>1</v>
       </c>
-      <c r="I89" t="s">
-        <v>190</v>
-      </c>
-      <c r="J89" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="90" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="I89" s="22" t="s">
+        <v>184</v>
+      </c>
+      <c r="J89" s="22" t="s">
+        <v>200</v>
+      </c>
+      <c r="K89" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="L89" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A90" s="1">
         <v>2</v>
       </c>
@@ -4002,7 +4073,7 @@
         <v>2</v>
       </c>
       <c r="E90" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="F90" s="2" t="b">
         <v>1</v>
@@ -4010,14 +4081,20 @@
       <c r="H90" s="1">
         <v>2</v>
       </c>
-      <c r="I90" t="s">
+      <c r="I90" s="22" t="s">
+        <v>185</v>
+      </c>
+      <c r="J90" s="22" t="s">
+        <v>201</v>
+      </c>
+      <c r="K90" s="22" t="s">
         <v>191</v>
       </c>
-      <c r="J90" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="91" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="L90" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A91" s="3">
         <v>3</v>
       </c>
@@ -4028,274 +4105,437 @@
         <v>3</v>
       </c>
       <c r="E91" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="F91" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H91" s="3">
+        <v>3</v>
+      </c>
+      <c r="I91" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="J91" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="K91" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="L91" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="94" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A94" s="19" t="s">
+        <v>196</v>
+      </c>
+      <c r="B94" s="20"/>
+      <c r="C94" s="20"/>
+      <c r="D94" s="20"/>
+      <c r="E94" s="20"/>
+      <c r="F94" s="20"/>
+      <c r="G94" s="20"/>
+      <c r="H94" s="20"/>
+      <c r="I94" s="20"/>
+      <c r="J94" s="20"/>
+      <c r="K94" s="20"/>
+      <c r="L94" s="20"/>
+      <c r="M94" s="20"/>
+      <c r="N94" s="21"/>
+    </row>
+    <row r="95" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A95" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B95" t="s">
+        <v>182</v>
+      </c>
+      <c r="C95" t="s">
+        <v>171</v>
+      </c>
+      <c r="D95" t="s">
+        <v>172</v>
+      </c>
+      <c r="E95" t="s">
+        <v>173</v>
+      </c>
+      <c r="F95" t="s">
+        <v>174</v>
+      </c>
+      <c r="G95" t="s">
+        <v>176</v>
+      </c>
+      <c r="H95" t="s">
         <v>175</v>
       </c>
-      <c r="F91" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="H91" s="3">
-        <v>3</v>
-      </c>
-      <c r="I91" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="J91" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="93" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="94" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A94" s="16" t="s">
-        <v>166</v>
-      </c>
-      <c r="B94" s="17"/>
-      <c r="C94" s="17"/>
-      <c r="D94" s="17"/>
-      <c r="E94" s="17"/>
-      <c r="F94" s="17"/>
-      <c r="G94" s="17"/>
-      <c r="H94" s="17"/>
-      <c r="I94" s="17"/>
-      <c r="J94" s="17"/>
-      <c r="K94" s="17"/>
-      <c r="L94" s="17"/>
-      <c r="M94" s="17"/>
-      <c r="N94" s="17"/>
-      <c r="O94" s="18"/>
-    </row>
-    <row r="95" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A95" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B95" t="s">
-        <v>91</v>
-      </c>
-      <c r="C95" t="s">
-        <v>188</v>
-      </c>
-      <c r="D95" t="s">
+      <c r="I95" t="s">
         <v>177</v>
       </c>
-      <c r="E95" t="s">
+      <c r="J95" t="s">
         <v>178</v>
       </c>
-      <c r="F95" t="s">
+      <c r="K95" t="s">
         <v>179</v>
       </c>
-      <c r="G95" t="s">
+      <c r="L95" t="s">
         <v>180</v>
       </c>
-      <c r="H95" t="s">
-        <v>182</v>
-      </c>
-      <c r="I95" t="s">
+      <c r="M95" t="s">
         <v>181</v>
       </c>
-      <c r="J95" t="s">
-        <v>183</v>
-      </c>
-      <c r="K95" t="s">
-        <v>184</v>
-      </c>
-      <c r="L95" t="s">
-        <v>185</v>
-      </c>
-      <c r="M95" t="s">
-        <v>186</v>
-      </c>
-      <c r="N95" t="s">
-        <v>187</v>
-      </c>
-      <c r="O95" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="96" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N95" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="96" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A96" s="1">
         <v>1</v>
       </c>
-      <c r="B96">
-        <v>1</v>
+      <c r="B96" t="s">
+        <v>11</v>
       </c>
       <c r="C96" t="s">
-        <v>11</v>
-      </c>
-      <c r="O96" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="97" spans="1:15" x14ac:dyDescent="0.3">
+        <v>191</v>
+      </c>
+      <c r="D96" t="s">
+        <v>191</v>
+      </c>
+      <c r="E96" t="s">
+        <v>191</v>
+      </c>
+      <c r="F96" t="s">
+        <v>191</v>
+      </c>
+      <c r="G96" t="s">
+        <v>191</v>
+      </c>
+      <c r="H96" t="s">
+        <v>191</v>
+      </c>
+      <c r="I96" t="s">
+        <v>191</v>
+      </c>
+      <c r="J96" t="s">
+        <v>191</v>
+      </c>
+      <c r="K96" t="s">
+        <v>191</v>
+      </c>
+      <c r="L96" t="s">
+        <v>191</v>
+      </c>
+      <c r="M96" t="s">
+        <v>191</v>
+      </c>
+      <c r="N96" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A97" s="1">
         <v>2</v>
       </c>
-      <c r="B97">
-        <v>2</v>
+      <c r="B97" t="s">
+        <v>11</v>
       </c>
       <c r="C97" t="s">
+        <v>191</v>
+      </c>
+      <c r="D97" t="s">
+        <v>191</v>
+      </c>
+      <c r="E97" t="s">
+        <v>191</v>
+      </c>
+      <c r="F97" t="s">
+        <v>191</v>
+      </c>
+      <c r="G97" t="s">
+        <v>191</v>
+      </c>
+      <c r="H97" t="s">
+        <v>191</v>
+      </c>
+      <c r="I97" t="s">
+        <v>191</v>
+      </c>
+      <c r="J97" t="s">
+        <v>191</v>
+      </c>
+      <c r="K97" t="s">
+        <v>191</v>
+      </c>
+      <c r="L97" t="s">
+        <v>191</v>
+      </c>
+      <c r="M97" t="s">
+        <v>191</v>
+      </c>
+      <c r="N97" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A98" s="3">
+        <v>3</v>
+      </c>
+      <c r="B98" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="O97" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="98" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A98" s="3">
-        <v>3</v>
-      </c>
-      <c r="B98" s="4">
-        <v>3</v>
-      </c>
-      <c r="C98" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D98" s="4"/>
-      <c r="E98" s="4"/>
-      <c r="F98" s="4"/>
-      <c r="G98" s="4"/>
-      <c r="H98" s="4"/>
-      <c r="I98" s="4"/>
-      <c r="J98" s="4"/>
-      <c r="K98" s="4"/>
-      <c r="L98" s="4"/>
-      <c r="M98" s="4"/>
-      <c r="N98" s="4"/>
-      <c r="O98" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="100" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="101" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A101" s="16" t="s">
-        <v>176</v>
-      </c>
-      <c r="B101" s="17"/>
-      <c r="C101" s="17"/>
-      <c r="D101" s="18"/>
-    </row>
-    <row r="102" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="C98" t="s">
+        <v>191</v>
+      </c>
+      <c r="D98" t="s">
+        <v>191</v>
+      </c>
+      <c r="E98" t="s">
+        <v>191</v>
+      </c>
+      <c r="F98" t="s">
+        <v>191</v>
+      </c>
+      <c r="G98" t="s">
+        <v>191</v>
+      </c>
+      <c r="H98" t="s">
+        <v>191</v>
+      </c>
+      <c r="I98" t="s">
+        <v>191</v>
+      </c>
+      <c r="J98" t="s">
+        <v>191</v>
+      </c>
+      <c r="K98" t="s">
+        <v>191</v>
+      </c>
+      <c r="L98" t="s">
+        <v>191</v>
+      </c>
+      <c r="M98" t="s">
+        <v>191</v>
+      </c>
+      <c r="N98" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="101" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A101" s="19" t="s">
+        <v>195</v>
+      </c>
+      <c r="B101" s="20"/>
+      <c r="C101" s="20"/>
+      <c r="D101" s="20"/>
+      <c r="E101" s="20"/>
+      <c r="F101" s="20"/>
+      <c r="G101" s="20"/>
+      <c r="H101" s="20"/>
+      <c r="I101" s="21"/>
+    </row>
+    <row r="102" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B102" t="s">
-        <v>91</v>
+        <v>186</v>
       </c>
       <c r="C102" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="D102" t="s">
-        <v>197</v>
+        <v>0</v>
       </c>
       <c r="E102" t="s">
+        <v>189</v>
+      </c>
+      <c r="F102" t="s">
+        <v>192</v>
+      </c>
+      <c r="G102" t="s">
+        <v>180</v>
+      </c>
+      <c r="H102" t="s">
+        <v>193</v>
+      </c>
+      <c r="I102" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="103" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A103" s="1">
+        <v>1</v>
+      </c>
+      <c r="B103">
+        <v>1</v>
+      </c>
+      <c r="C103">
+        <v>1</v>
+      </c>
+      <c r="D103" t="s">
+        <v>188</v>
+      </c>
+      <c r="E103">
+        <v>18</v>
+      </c>
+      <c r="F103" t="b">
         <v>0</v>
       </c>
-      <c r="F102" t="s">
-        <v>199</v>
-      </c>
-      <c r="G102" t="s">
-        <v>193</v>
-      </c>
-      <c r="H102" t="s">
-        <v>194</v>
-      </c>
-      <c r="I102" t="s">
-        <v>195</v>
-      </c>
-      <c r="J102" t="s">
-        <v>167</v>
-      </c>
-      <c r="K102" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="103" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A103" s="1">
-        <v>1</v>
-      </c>
-      <c r="B103">
-        <v>1</v>
-      </c>
-      <c r="C103">
-        <v>1</v>
-      </c>
-      <c r="D103">
-        <v>1</v>
-      </c>
-      <c r="E103" t="s">
-        <v>198</v>
-      </c>
-      <c r="F103">
-        <v>18</v>
-      </c>
-      <c r="J103" t="s">
-        <v>168</v>
-      </c>
-      <c r="K103" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="104" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="G103" t="b">
+        <v>0</v>
+      </c>
+      <c r="H103">
+        <v>0</v>
+      </c>
+      <c r="I103" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A104" s="1">
         <v>2</v>
       </c>
       <c r="B104">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C104">
+        <v>3</v>
+      </c>
+      <c r="D104" t="s">
+        <v>188</v>
+      </c>
+      <c r="E104">
+        <v>12</v>
+      </c>
+      <c r="F104" t="b">
+        <v>0</v>
+      </c>
+      <c r="G104" t="b">
+        <v>0</v>
+      </c>
+      <c r="H104">
+        <v>0</v>
+      </c>
+      <c r="I104" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A105" s="3">
+        <v>3</v>
+      </c>
+      <c r="B105" s="4">
+        <v>1</v>
+      </c>
+      <c r="C105" s="4">
+        <v>1</v>
+      </c>
+      <c r="D105" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="E105" s="4">
+        <v>18</v>
+      </c>
+      <c r="F105" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G105" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H105" s="4">
+        <v>0</v>
+      </c>
+      <c r="I105" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="108" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A108" s="19" t="s">
+        <v>198</v>
+      </c>
+      <c r="B108" s="20"/>
+      <c r="C108" s="20"/>
+      <c r="D108" s="20"/>
+      <c r="E108" s="21"/>
+    </row>
+    <row r="109" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A109" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B109" t="s">
+        <v>91</v>
+      </c>
+      <c r="C109" t="s">
+        <v>194</v>
+      </c>
+      <c r="D109" t="s">
+        <v>197</v>
+      </c>
+      <c r="E109" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="110" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A110" s="1">
+        <v>1</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110">
         <v>2</v>
       </c>
-      <c r="D104">
-        <v>3</v>
-      </c>
-      <c r="E104" t="s">
-        <v>198</v>
-      </c>
-      <c r="F104">
-        <v>12</v>
-      </c>
-      <c r="J104" t="s">
-        <v>11</v>
-      </c>
-      <c r="K104" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="105" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A105" s="3">
-        <v>3</v>
-      </c>
-      <c r="B105" s="4">
+      <c r="D110">
+        <v>6</v>
+      </c>
+      <c r="E110" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A111" s="1">
         <v>2</v>
       </c>
-      <c r="C105" s="4">
-        <v>1</v>
-      </c>
-      <c r="D105" s="4">
-        <v>1</v>
-      </c>
-      <c r="E105" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="F105" s="4">
-        <v>18</v>
-      </c>
-      <c r="G105" s="4"/>
-      <c r="H105" s="4"/>
-      <c r="I105" s="4"/>
-      <c r="J105" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="K105" s="5" t="b">
+      <c r="B111">
+        <v>2</v>
+      </c>
+      <c r="C111">
+        <v>4</v>
+      </c>
+      <c r="D111">
+        <v>6</v>
+      </c>
+      <c r="E111" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A112" s="3">
+        <v>3</v>
+      </c>
+      <c r="B112" s="4">
+        <v>4</v>
+      </c>
+      <c r="C112" s="4">
+        <v>4</v>
+      </c>
+      <c r="D112" s="4">
+        <v>5</v>
+      </c>
+      <c r="E112" s="5" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="26">
-    <mergeCell ref="A87:B87"/>
-    <mergeCell ref="D87:F87"/>
-    <mergeCell ref="A101:D101"/>
-    <mergeCell ref="A80:K80"/>
-    <mergeCell ref="A94:O94"/>
-    <mergeCell ref="H87:J87"/>
+  <mergeCells count="27">
+    <mergeCell ref="I5:K5"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="F19:L19"/>
+    <mergeCell ref="G12:K12"/>
     <mergeCell ref="A61:E61"/>
     <mergeCell ref="G61:K61"/>
     <mergeCell ref="A68:E68"/>
@@ -4308,20 +4548,22 @@
     <mergeCell ref="A47:D47"/>
     <mergeCell ref="I26:K26"/>
     <mergeCell ref="F47:L47"/>
-    <mergeCell ref="H40:L40"/>
     <mergeCell ref="A54:I54"/>
     <mergeCell ref="A40:F40"/>
-    <mergeCell ref="I5:K5"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A26:G26"/>
-    <mergeCell ref="F19:L19"/>
-    <mergeCell ref="G12:K12"/>
+    <mergeCell ref="H40:M40"/>
+    <mergeCell ref="A108:E108"/>
+    <mergeCell ref="A94:N94"/>
+    <mergeCell ref="A80:L80"/>
+    <mergeCell ref="A101:I101"/>
+    <mergeCell ref="A87:B87"/>
+    <mergeCell ref="D87:F87"/>
+    <mergeCell ref="H87:L87"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
-  <tableParts count="26">
+  <tableParts count="27">
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
     <tablePart r:id="rId5"/>
@@ -4348,6 +4590,7 @@
     <tablePart r:id="rId26"/>
     <tablePart r:id="rId27"/>
     <tablePart r:id="rId28"/>
+    <tablePart r:id="rId29"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Se agrega archivo js para menu del aministrador. Se crea CRM Inbox para módulo de postventa.
</commit_message>
<xml_diff>
--- a/BBDD.xlsx
+++ b/BBDD.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyectos\Web_Andez\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1DF4339-99C7-4AAB-8AAB-4C5C28C64006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15B1C643-F7F9-46F1-B661-7A89AD096A01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5D42B345-DB14-48C1-9A38-23908D3120ED}"/>
   </bookViews>
@@ -118,7 +118,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="222">
   <si>
     <t>Color</t>
   </si>
@@ -733,6 +733,57 @@
   </si>
   <si>
     <t>Declaracion</t>
+  </si>
+  <si>
+    <t>ClientesPostventa</t>
+  </si>
+  <si>
+    <t>NombreApellido</t>
+  </si>
+  <si>
+    <t>Piso</t>
+  </si>
+  <si>
+    <t>Departamente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CodigoPostal </t>
+  </si>
+  <si>
+    <t>Jose Perez</t>
+  </si>
+  <si>
+    <t>Maria Gomez</t>
+  </si>
+  <si>
+    <t>Natalia Martinez</t>
+  </si>
+  <si>
+    <t>aaaa@gmail.com</t>
+  </si>
+  <si>
+    <t>dddd@gmail.com</t>
+  </si>
+  <si>
+    <t>fffff@gmail.com</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Mitre 2223</t>
+  </si>
+  <si>
+    <t>DatosCompra</t>
+  </si>
+  <si>
+    <t>IdDistribuidor</t>
+  </si>
+  <si>
+    <t>FechaCompra</t>
+  </si>
+  <si>
+    <t>Factura</t>
   </si>
 </sst>
 </file>
@@ -899,7 +950,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -935,6 +986,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1758,6 +1812,41 @@
     <tableColumn id="3" xr3:uid="{61419E12-5C48-471B-A94C-365D61B394C2}" name="IdBackground"/>
     <tableColumn id="4" xr3:uid="{3B4A719A-180B-4B39-9C10-B58CA3A5C88C}" name="IdEdicionTexto"/>
     <tableColumn id="5" xr3:uid="{4B5372AE-F961-4286-86FB-E03ECC3B0166}" name="Activo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="28" xr:uid="{E5C72C39-AEF7-4120-A1E5-FF7EB5A3BF17}" name="Tabla28" displayName="Tabla28" ref="A116:K119" totalsRowShown="0">
+  <autoFilter ref="A116:K119" xr:uid="{E5C72C39-AEF7-4120-A1E5-FF7EB5A3BF17}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{68690C7C-4428-4270-97EF-F62ECCF7314E}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{4ED8A294-C798-4D37-9F33-B2D6E944F3F4}" name="NombreApellido"/>
+    <tableColumn id="3" xr3:uid="{58ED13BD-9B17-4772-85AE-6842EAEE71E5}" name="Mail" dataCellStyle="Hipervínculo"/>
+    <tableColumn id="4" xr3:uid="{94F35AE4-BB92-4E59-9201-C44956F3D992}" name="Telefono"/>
+    <tableColumn id="5" xr3:uid="{B1749734-A73F-4D73-AA3D-233EA5C9D90A}" name="Direccion"/>
+    <tableColumn id="6" xr3:uid="{34C9AECC-F209-4DEB-9823-F29D4B16D927}" name="Piso"/>
+    <tableColumn id="7" xr3:uid="{C0537B94-D9CA-4EAF-B400-6B36DD29ACEF}" name="Departamente"/>
+    <tableColumn id="8" xr3:uid="{3361C285-84BA-43DF-9B87-BBEA471C74DB}" name="Localidad"/>
+    <tableColumn id="9" xr3:uid="{31F8994E-756A-43E8-ADCF-36CDB3FECA27}" name="IdProvincia"/>
+    <tableColumn id="10" xr3:uid="{41A026C6-9E4F-4D56-911F-854C5718C114}" name="CodigoPostal "/>
+    <tableColumn id="11" xr3:uid="{F8363EAB-1F66-4EC1-BD18-A407969A23F0}" name="Activo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{1DA5C3FF-DEDA-4FD9-B41A-F3E2538CE824}" name="Tabla29" displayName="Tabla29" ref="A123:F126" totalsRowShown="0">
+  <autoFilter ref="A123:F126" xr:uid="{1DA5C3FF-DEDA-4FD9-B41A-F3E2538CE824}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{26411AE4-B531-46EC-A743-601E7189E434}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{2448A646-7614-46EE-BE66-4A39153E5F8A}" name="IdDistribuidor"/>
+    <tableColumn id="3" xr3:uid="{57960469-7CA4-4F5E-823C-0725B5B59DA9}" name="FechaCompra"/>
+    <tableColumn id="4" xr3:uid="{B4511E1E-8880-4F6B-AB2B-5BE00AA0F941}" name="Factura"/>
+    <tableColumn id="5" xr3:uid="{BA1A06F9-6164-4B4F-BDD1-319BC1E813A6}" name="IdProducto"/>
+    <tableColumn id="6" xr3:uid="{3C17DB6E-6062-4A4B-975F-FA7E04D0DE6E}" name="Activo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2180,7 +2269,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD350C1D-1850-4BF9-ABCF-FA1A23EC1542}">
-  <dimension ref="A1:P112"/>
+  <dimension ref="A1:P126"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.77734375" bestFit="1" customWidth="1"/>
@@ -4017,13 +4106,13 @@
       <c r="H88" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="I88" s="22" t="s">
+      <c r="I88" t="s">
         <v>37</v>
       </c>
-      <c r="J88" s="22" t="s">
+      <c r="J88" t="s">
         <v>204</v>
       </c>
-      <c r="K88" s="22" t="s">
+      <c r="K88" t="s">
         <v>199</v>
       </c>
       <c r="L88" s="2" t="s">
@@ -4049,13 +4138,13 @@
       <c r="H89" s="1">
         <v>1</v>
       </c>
-      <c r="I89" s="22" t="s">
+      <c r="I89" t="s">
         <v>184</v>
       </c>
-      <c r="J89" s="22" t="s">
+      <c r="J89" t="s">
         <v>200</v>
       </c>
-      <c r="K89" s="22" t="s">
+      <c r="K89" t="s">
         <v>191</v>
       </c>
       <c r="L89" s="2" t="b">
@@ -4081,13 +4170,13 @@
       <c r="H90" s="1">
         <v>2</v>
       </c>
-      <c r="I90" s="22" t="s">
+      <c r="I90" t="s">
         <v>185</v>
       </c>
-      <c r="J90" s="22" t="s">
+      <c r="J90" t="s">
         <v>201</v>
       </c>
-      <c r="K90" s="22" t="s">
+      <c r="K90" t="s">
         <v>191</v>
       </c>
       <c r="L90" s="2" t="b">
@@ -4529,13 +4618,264 @@
         <v>1</v>
       </c>
     </row>
+    <row r="114" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="115" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A115" s="16" t="s">
+        <v>205</v>
+      </c>
+      <c r="B115" s="17"/>
+      <c r="C115" s="17"/>
+      <c r="D115" s="17"/>
+      <c r="E115" s="17"/>
+      <c r="F115" s="17"/>
+      <c r="G115" s="17"/>
+      <c r="H115" s="17"/>
+      <c r="I115" s="17"/>
+      <c r="J115" s="17"/>
+      <c r="K115" s="18"/>
+    </row>
+    <row r="116" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A116" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B116" s="22" t="s">
+        <v>206</v>
+      </c>
+      <c r="C116" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="D116" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="E116" s="22" t="s">
+        <v>88</v>
+      </c>
+      <c r="F116" s="22" t="s">
+        <v>207</v>
+      </c>
+      <c r="G116" s="22" t="s">
+        <v>208</v>
+      </c>
+      <c r="H116" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="I116" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="J116" s="22" t="s">
+        <v>209</v>
+      </c>
+      <c r="K116" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A117" s="1">
+        <v>1</v>
+      </c>
+      <c r="B117" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="C117" s="23" t="s">
+        <v>213</v>
+      </c>
+      <c r="D117" s="22">
+        <v>5555511111</v>
+      </c>
+      <c r="E117" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="F117" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="G117" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="H117" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="I117" s="22">
+        <v>1</v>
+      </c>
+      <c r="J117" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="K117" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A118" s="1">
+        <v>2</v>
+      </c>
+      <c r="B118" s="22" t="s">
+        <v>211</v>
+      </c>
+      <c r="C118" s="23" t="s">
+        <v>214</v>
+      </c>
+      <c r="D118" s="22">
+        <v>5555522222</v>
+      </c>
+      <c r="E118" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="F118" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="G118" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="H118" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="I118" s="22">
+        <v>1</v>
+      </c>
+      <c r="J118" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="K118" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A119" s="3">
+        <v>3</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="C119" s="24" t="s">
+        <v>215</v>
+      </c>
+      <c r="D119" s="4">
+        <v>5555533332</v>
+      </c>
+      <c r="E119" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="F119" s="4">
+        <v>2</v>
+      </c>
+      <c r="G119" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="H119" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="I119" s="4">
+        <v>1</v>
+      </c>
+      <c r="J119" s="4">
+        <v>1605</v>
+      </c>
+      <c r="K119" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="122" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A122" s="16" t="s">
+        <v>218</v>
+      </c>
+      <c r="B122" s="17"/>
+      <c r="C122" s="17"/>
+      <c r="D122" s="17"/>
+      <c r="E122" s="17"/>
+      <c r="F122" s="18"/>
+    </row>
+    <row r="123" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A123" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B123" s="22" t="s">
+        <v>219</v>
+      </c>
+      <c r="C123" s="22" t="s">
+        <v>220</v>
+      </c>
+      <c r="D123" s="22" t="s">
+        <v>221</v>
+      </c>
+      <c r="E123" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="F123" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="124" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A124" s="1">
+        <v>1</v>
+      </c>
+      <c r="B124" s="22">
+        <v>1</v>
+      </c>
+      <c r="C124" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="D124" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="E124" s="22">
+        <v>1</v>
+      </c>
+      <c r="F124" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A125" s="1">
+        <v>2</v>
+      </c>
+      <c r="B125" s="22">
+        <v>2</v>
+      </c>
+      <c r="C125" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="D125" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="E125" s="22">
+        <v>2</v>
+      </c>
+      <c r="F125" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A126" s="3">
+        <v>3</v>
+      </c>
+      <c r="B126" s="4">
+        <v>2</v>
+      </c>
+      <c r="C126" s="25">
+        <v>44724</v>
+      </c>
+      <c r="D126" s="4">
+        <v>33223</v>
+      </c>
+      <c r="E126" s="4">
+        <v>3</v>
+      </c>
+      <c r="F126" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="27">
-    <mergeCell ref="I5:K5"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A26:G26"/>
-    <mergeCell ref="F19:L19"/>
-    <mergeCell ref="G12:K12"/>
+  <mergeCells count="29">
+    <mergeCell ref="A115:K115"/>
+    <mergeCell ref="A122:F122"/>
+    <mergeCell ref="A108:E108"/>
+    <mergeCell ref="A94:N94"/>
+    <mergeCell ref="A80:L80"/>
+    <mergeCell ref="A101:I101"/>
+    <mergeCell ref="A87:B87"/>
+    <mergeCell ref="D87:F87"/>
+    <mergeCell ref="H87:L87"/>
     <mergeCell ref="A61:E61"/>
     <mergeCell ref="G61:K61"/>
     <mergeCell ref="A68:E68"/>
@@ -4551,19 +4891,17 @@
     <mergeCell ref="A54:I54"/>
     <mergeCell ref="A40:F40"/>
     <mergeCell ref="H40:M40"/>
-    <mergeCell ref="A108:E108"/>
-    <mergeCell ref="A94:N94"/>
-    <mergeCell ref="A80:L80"/>
-    <mergeCell ref="A101:I101"/>
-    <mergeCell ref="A87:B87"/>
-    <mergeCell ref="D87:F87"/>
-    <mergeCell ref="H87:L87"/>
+    <mergeCell ref="I5:K5"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="F19:L19"/>
+    <mergeCell ref="G12:K12"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
-  <tableParts count="27">
+  <tableParts count="29">
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
     <tablePart r:id="rId5"/>
@@ -4591,6 +4929,8 @@
     <tablePart r:id="rId27"/>
     <tablePart r:id="rId28"/>
     <tablePart r:id="rId29"/>
+    <tablePart r:id="rId30"/>
+    <tablePart r:id="rId31"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Se agrega categoría Subtipo de producto a CMS página Línea. Se modifica el formulario web de postventa y se cambian inputs por select. Se agrega manejo de estados en CRM Formulario y registro de modificaciones. Se crea CRM Casos para módulo de postventa con el consolidado de casos en forma de tabla.
</commit_message>
<xml_diff>
--- a/BBDD.xlsx
+++ b/BBDD.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyectos\Web_Andez\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15B1C643-F7F9-46F1-B661-7A89AD096A01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F396AEE-830D-45C7-BF5C-F510F77D9436}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5D42B345-DB14-48C1-9A38-23908D3120ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -118,7 +119,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="283">
   <si>
     <t>Color</t>
   </si>
@@ -744,9 +745,6 @@
     <t>Piso</t>
   </si>
   <si>
-    <t>Departamente</t>
-  </si>
-  <si>
     <t xml:space="preserve">CodigoPostal </t>
   </si>
   <si>
@@ -784,6 +782,192 @@
   </si>
   <si>
     <t>Factura</t>
+  </si>
+  <si>
+    <t>Subtipo</t>
+  </si>
+  <si>
+    <t>SubtipoProducto</t>
+  </si>
+  <si>
+    <t>Griferia para baño</t>
+  </si>
+  <si>
+    <t>Griferia para cocina</t>
+  </si>
+  <si>
+    <t>NombreBarrio</t>
+  </si>
+  <si>
+    <t>DNI</t>
+  </si>
+  <si>
+    <t>Numeracion</t>
+  </si>
+  <si>
+    <t>DtoLote</t>
+  </si>
+  <si>
+    <t>IdCliente</t>
+  </si>
+  <si>
+    <t>IdFormaContacto</t>
+  </si>
+  <si>
+    <t>Casos</t>
+  </si>
+  <si>
+    <t>Fecha1erContacto</t>
+  </si>
+  <si>
+    <t>Fecha1eraRespuesta</t>
+  </si>
+  <si>
+    <t>FechaCierre</t>
+  </si>
+  <si>
+    <t>IdMotivoContacto</t>
+  </si>
+  <si>
+    <t>IdCodigoReclamo</t>
+  </si>
+  <si>
+    <t>IdEstadoReclamo</t>
+  </si>
+  <si>
+    <t>Consulta</t>
+  </si>
+  <si>
+    <t>Solucion</t>
+  </si>
+  <si>
+    <t>IdDatosCompra</t>
+  </si>
+  <si>
+    <t>FechaOT</t>
+  </si>
+  <si>
+    <t>NumeroOT</t>
+  </si>
+  <si>
+    <t>Repuesto</t>
+  </si>
+  <si>
+    <t>Cantidad</t>
+  </si>
+  <si>
+    <t>Cierre ceramico</t>
+  </si>
+  <si>
+    <t>Aireador TT</t>
+  </si>
+  <si>
+    <t>IdTipoRespuesto</t>
+  </si>
+  <si>
+    <t>IdModoSolucion</t>
+  </si>
+  <si>
+    <t>Observaciones</t>
+  </si>
+  <si>
+    <t>NumTiendanube</t>
+  </si>
+  <si>
+    <t>NumOperacionML</t>
+  </si>
+  <si>
+    <t>FechaCompraTNyML</t>
+  </si>
+  <si>
+    <t>MontoCompra</t>
+  </si>
+  <si>
+    <t>NumFacturaRepuesto</t>
+  </si>
+  <si>
+    <t>NumGuiaCorreo</t>
+  </si>
+  <si>
+    <t>IdRegistro</t>
+  </si>
+  <si>
+    <t>EstadoReclamo</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>Abierto</t>
+  </si>
+  <si>
+    <t>Cerrado</t>
+  </si>
+  <si>
+    <t>Pedido a fábrica</t>
+  </si>
+  <si>
+    <t>ModoSolucion</t>
+  </si>
+  <si>
+    <t>Retira en fábrica</t>
+  </si>
+  <si>
+    <t>Envio a distribuidor</t>
+  </si>
+  <si>
+    <t>Envio a domicilio</t>
+  </si>
+  <si>
+    <t>TipoRepuesto</t>
+  </si>
+  <si>
+    <t>Convencional</t>
+  </si>
+  <si>
+    <t>No Convencional</t>
+  </si>
+  <si>
+    <t>Ninguno</t>
+  </si>
+  <si>
+    <t>FormaContacto</t>
+  </si>
+  <si>
+    <t>Web</t>
+  </si>
+  <si>
+    <t>MotivoContacto</t>
+  </si>
+  <si>
+    <t>CodigoMotivo</t>
+  </si>
+  <si>
+    <t>Repuesto en garantia</t>
+  </si>
+  <si>
+    <t>Falla de fabricacion</t>
+  </si>
+  <si>
+    <t>Faltante</t>
+  </si>
+  <si>
+    <t>RegistroPostventa</t>
+  </si>
+  <si>
+    <t>Fecha</t>
+  </si>
+  <si>
+    <t>Registro</t>
+  </si>
+  <si>
+    <t>Zona</t>
+  </si>
+  <si>
+    <t>Litoral</t>
+  </si>
+  <si>
+    <t>Centro</t>
   </si>
 </sst>
 </file>
@@ -950,7 +1134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -967,6 +1151,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -976,24 +1170,54 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="57">
+  <dxfs count="62">
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor theme="0" tint="-0.14999847407452621"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="d/m/yyyy"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor theme="0" tint="-0.14999847407452621"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor theme="0" tint="-0.14999847407452621"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="d/m/yyyy"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1322,12 +1546,6 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1508,7 +1726,7 @@
   <autoFilter ref="A13:E16" xr:uid="{D96833EF-4E6F-4FA0-A7A0-6E6817E2B38A}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{317907DD-843B-4FA4-8837-A0A78A4A0507}" name="ID"/>
-    <tableColumn id="5" xr3:uid="{E0921BEC-D870-4C51-B3FC-23E013804DC3}" name="CodigoColor" dataDxfId="56"/>
+    <tableColumn id="5" xr3:uid="{E0921BEC-D870-4C51-B3FC-23E013804DC3}" name="CodigoColor" dataDxfId="61"/>
     <tableColumn id="2" xr3:uid="{8053C3DC-ACA4-4AAB-9AFB-34FBDDEBC52B}" name="NombreColor"/>
     <tableColumn id="4" xr3:uid="{1D3A10F0-E8C4-471A-B4A8-2001816AFFF2}" name="URLColor"/>
     <tableColumn id="3" xr3:uid="{D04813E9-6E48-439B-A711-735DEB41533C}" name="Activo"/>
@@ -1541,8 +1759,8 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{C6605137-9E60-4417-BE9D-22DF41FEA57D}" name="ID"/>
     <tableColumn id="2" xr3:uid="{D82CDF84-BD14-4C63-ABBA-8F2236A9C0E4}" name="Pais"/>
-    <tableColumn id="3" xr3:uid="{FA78D055-E341-4362-A23A-0CCFC591E8FA}" name="Latitud" dataDxfId="53"/>
-    <tableColumn id="4" xr3:uid="{36EB177E-ACE1-4B78-A56A-A9F891312B25}" name="Longitud" dataDxfId="52"/>
+    <tableColumn id="3" xr3:uid="{FA78D055-E341-4362-A23A-0CCFC591E8FA}" name="Latitud" dataDxfId="58"/>
+    <tableColumn id="4" xr3:uid="{36EB177E-ACE1-4B78-A56A-A9F891312B25}" name="Longitud" dataDxfId="57"/>
     <tableColumn id="5" xr3:uid="{4122267C-292B-476B-8AB1-41CBE8A90AAF}" name="Zoom"/>
     <tableColumn id="7" xr3:uid="{0270C110-04E9-4179-AF06-958CA4E37E9B}" name="Activo"/>
   </tableColumns>
@@ -1551,15 +1769,15 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{EF32F6B3-AC45-462F-BE18-EFE2DD57FE9B}" name="Tabla17" displayName="Tabla17" ref="H41:M44" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{EF32F6B3-AC45-462F-BE18-EFE2DD57FE9B}" name="Tabla17" displayName="Tabla17" ref="H41:M44" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
   <autoFilter ref="H41:M44" xr:uid="{EF32F6B3-AC45-462F-BE18-EFE2DD57FE9B}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{C8F6ED57-5FD2-4FB3-A4A5-BC3965E98B15}" name="ID" dataDxfId="49"/>
-    <tableColumn id="2" xr3:uid="{65B99387-EDCD-429B-B81B-A4F58479A304}" name="IdProducto" dataDxfId="48"/>
-    <tableColumn id="3" xr3:uid="{5D9C0348-2DF4-47CC-977C-AAFB9F19E959}" name="Titulo" dataDxfId="47"/>
-    <tableColumn id="4" xr3:uid="{1CACB54F-DC9D-41AC-A04F-171EF34060DC}" name="URLImagen" dataDxfId="46"/>
+    <tableColumn id="1" xr3:uid="{C8F6ED57-5FD2-4FB3-A4A5-BC3965E98B15}" name="ID" dataDxfId="54"/>
+    <tableColumn id="2" xr3:uid="{65B99387-EDCD-429B-B81B-A4F58479A304}" name="IdProducto" dataDxfId="53"/>
+    <tableColumn id="3" xr3:uid="{5D9C0348-2DF4-47CC-977C-AAFB9F19E959}" name="Titulo" dataDxfId="52"/>
+    <tableColumn id="4" xr3:uid="{1CACB54F-DC9D-41AC-A04F-171EF34060DC}" name="URLImagen" dataDxfId="51"/>
     <tableColumn id="5" xr3:uid="{E836C9A1-0FCD-4424-8667-FBB476A992FD}" name="Publicada"/>
-    <tableColumn id="7" xr3:uid="{824500A6-D872-42FD-9C38-60CB54869E2F}" name="Activo" dataDxfId="45"/>
+    <tableColumn id="7" xr3:uid="{824500A6-D872-42FD-9C38-60CB54869E2F}" name="Activo" dataDxfId="50"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1587,8 +1805,8 @@
     <tableColumn id="3" xr3:uid="{650899D4-4E19-437F-9FCF-B4D26F2AA0DB}" name="Direccion"/>
     <tableColumn id="4" xr3:uid="{1E07E83B-09DC-40FD-907E-40F4CBC0A570}" name="IdProvincia"/>
     <tableColumn id="5" xr3:uid="{6138418F-A367-4A68-8F05-2638E82A22BC}" name="Telefono"/>
-    <tableColumn id="6" xr3:uid="{80260CDA-43B3-49C5-B2E8-6D4D4EE4367B}" name="Latitud" dataDxfId="44"/>
-    <tableColumn id="7" xr3:uid="{D1025C6A-57D3-4E57-916D-CF79774C6EAF}" name="Longitud" dataDxfId="43"/>
+    <tableColumn id="6" xr3:uid="{80260CDA-43B3-49C5-B2E8-6D4D4EE4367B}" name="Latitud" dataDxfId="49"/>
+    <tableColumn id="7" xr3:uid="{D1025C6A-57D3-4E57-916D-CF79774C6EAF}" name="Longitud" dataDxfId="48"/>
     <tableColumn id="8" xr3:uid="{FACFCBBE-C8C5-4011-911D-7F4D64577C47}" name="IdPagina"/>
     <tableColumn id="9" xr3:uid="{3EE8280A-E1AE-43CB-8AA3-681D1032743D}" name="Activo"/>
   </tableColumns>
@@ -1597,28 +1815,29 @@
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{B6BCDECB-3201-4C98-AA8D-79812894A18B}" name="Tabla19" displayName="Tabla19" ref="K34:N37" totalsRowShown="0" headerRowDxfId="42" dataDxfId="41">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{B6BCDECB-3201-4C98-AA8D-79812894A18B}" name="Tabla19" displayName="Tabla19" ref="K34:N37" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46">
   <autoFilter ref="K34:N37" xr:uid="{36798AE9-B843-4477-9F23-32045BDEF7D7}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{E050CEA3-2793-4698-9E45-C3447ADCD555}" name="ID" dataDxfId="40"/>
-    <tableColumn id="2" xr3:uid="{03295AE7-34B5-4134-9D2F-2268D15B310C}" name="IDProducto" dataDxfId="39"/>
-    <tableColumn id="3" xr3:uid="{1564E106-D50F-4573-A696-EE197325F0F3}" name="IDAtributo" dataDxfId="38"/>
-    <tableColumn id="4" xr3:uid="{5F701778-C720-415C-9979-8380EB9AB80C}" name="Activo" dataDxfId="37"/>
+    <tableColumn id="1" xr3:uid="{E050CEA3-2793-4698-9E45-C3447ADCD555}" name="ID" dataDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{03295AE7-34B5-4134-9D2F-2268D15B310C}" name="IDProducto" dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{1564E106-D50F-4573-A696-EE197325F0F3}" name="IDAtributo" dataDxfId="43"/>
+    <tableColumn id="4" xr3:uid="{5F701778-C720-415C-9979-8380EB9AB80C}" name="Activo" dataDxfId="42"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{7637683B-2521-4501-AE41-E6F0058D9D80}" name="Tabla1719" displayName="Tabla1719" ref="F48:L51" totalsRowShown="0">
-  <autoFilter ref="F48:L51" xr:uid="{05CA7051-E28E-4B32-9032-EE45922419A6}"/>
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{7637683B-2521-4501-AE41-E6F0058D9D80}" name="Tabla1719" displayName="Tabla1719" ref="F48:M51" totalsRowShown="0">
+  <autoFilter ref="F48:M51" xr:uid="{05CA7051-E28E-4B32-9032-EE45922419A6}"/>
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{76441B91-C9F3-418E-9F7A-2145EC66A51B}" name="ID"/>
     <tableColumn id="2" xr3:uid="{B7D7EADF-0604-4B90-A7CA-6537AE39152D}" name="Pronvincia"/>
     <tableColumn id="3" xr3:uid="{FBCCEEC7-DBEE-4480-8CBE-1F5805CA9202}" name="IdPais"/>
-    <tableColumn id="4" xr3:uid="{0A3D75EA-6C18-48E0-9489-C5D19B3AC70A}" name="Latitud" dataDxfId="36"/>
-    <tableColumn id="5" xr3:uid="{ACBD9873-D350-427F-993B-2B1B42296D9B}" name="Longitud" dataDxfId="35"/>
+    <tableColumn id="4" xr3:uid="{0A3D75EA-6C18-48E0-9489-C5D19B3AC70A}" name="Latitud" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{ACBD9873-D350-427F-993B-2B1B42296D9B}" name="Longitud" dataDxfId="0"/>
     <tableColumn id="6" xr3:uid="{957CA68C-6225-4C37-B8D5-8FF8C064FB1C}" name="Zoom"/>
+    <tableColumn id="8" xr3:uid="{33319F29-BC62-4963-B0AA-34AC0E216488}" name="Zona"/>
     <tableColumn id="7" xr3:uid="{D19F9B22-3CC1-4E0E-B3DB-56D9B346F0CD}" name="Activo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1626,46 +1845,46 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{D66B8F6B-A06F-42EB-B1CE-F5AC470DCC17}" name="Tabla20" displayName="Tabla20" ref="A62:E65" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{D66B8F6B-A06F-42EB-B1CE-F5AC470DCC17}" name="Tabla20" displayName="Tabla20" ref="A62:E65" totalsRowShown="0" headerRowDxfId="41" dataDxfId="40">
   <autoFilter ref="A62:E65" xr:uid="{6995137C-E78D-4F26-A126-F3AEFE2A2B13}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{7C1F763D-9A29-4F91-BB26-5F2CF68260F0}" name="ID" dataDxfId="32"/>
-    <tableColumn id="5" xr3:uid="{F0BF2187-ECA7-4173-9FAC-3BC72EFDB82F}" name="IdEmpresa" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{98E75056-4A9A-4C56-8FA5-EFD4D867777B}" name="Nombre" dataDxfId="30"/>
-    <tableColumn id="3" xr3:uid="{48A2AE2B-7A42-420C-8BB3-5F9F2AA01721}" name="Mail" dataDxfId="29">
+    <tableColumn id="1" xr3:uid="{7C1F763D-9A29-4F91-BB26-5F2CF68260F0}" name="ID" dataDxfId="39"/>
+    <tableColumn id="5" xr3:uid="{F0BF2187-ECA7-4173-9FAC-3BC72EFDB82F}" name="IdEmpresa" dataDxfId="38"/>
+    <tableColumn id="2" xr3:uid="{98E75056-4A9A-4C56-8FA5-EFD4D867777B}" name="Nombre" dataDxfId="37"/>
+    <tableColumn id="3" xr3:uid="{48A2AE2B-7A42-420C-8BB3-5F9F2AA01721}" name="Mail" dataDxfId="36">
       <calculatedColumnFormula>CONCATENATE(C63,"@andez.com.ar")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{31D99612-66DC-4B54-A747-6C39765D7B66}" name="Activo" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{31D99612-66DC-4B54-A747-6C39765D7B66}" name="Activo" dataDxfId="35"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{2B2EAABA-4403-411A-98F0-A8284D43302C}" name="Tabla2021" displayName="Tabla2021" ref="G62:K65" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{2B2EAABA-4403-411A-98F0-A8284D43302C}" name="Tabla2021" displayName="Tabla2021" ref="G62:K65" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
   <autoFilter ref="G62:K65" xr:uid="{89087EED-CE2D-441A-9746-B0BA56EA9A63}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{6D3F8F4E-2473-4BE6-A51E-C3C3E4C26133}" name="ID" dataDxfId="25"/>
-    <tableColumn id="5" xr3:uid="{8C181956-53C7-4FD2-BAAB-42B1CDE2E84E}" name="IdEmpresa" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{12B007DF-889A-4CDB-93CC-EBEFCBD3A3E9}" name="Nombre" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{A94B5F86-8442-44DD-9C03-77F51D7F5B8D}" name="Telefono" dataDxfId="22">
+    <tableColumn id="1" xr3:uid="{6D3F8F4E-2473-4BE6-A51E-C3C3E4C26133}" name="ID" dataDxfId="32"/>
+    <tableColumn id="5" xr3:uid="{8C181956-53C7-4FD2-BAAB-42B1CDE2E84E}" name="IdEmpresa" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{12B007DF-889A-4CDB-93CC-EBEFCBD3A3E9}" name="Nombre" dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{A94B5F86-8442-44DD-9C03-77F51D7F5B8D}" name="Telefono" dataDxfId="29">
       <calculatedColumnFormula>CONCATENATE(I63,"@andez.com.ar")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{0E412ADD-9FF3-43E1-BDA1-A917D6B1E4D7}" name="Activo" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{0E412ADD-9FF3-43E1-BDA1-A917D6B1E4D7}" name="Activo" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{8F3FF2B6-156D-475C-B60E-2BBAE1F181CE}" name="Tabla21" displayName="Tabla21" ref="A69:E72" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19" tableBorderDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{8F3FF2B6-156D-475C-B60E-2BBAE1F181CE}" name="Tabla21" displayName="Tabla21" ref="A69:E72" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26" tableBorderDxfId="25">
   <autoFilter ref="A69:E72" xr:uid="{58000D4A-AEBA-4D49-B463-180C8FD8A937}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{E9F2D081-00F6-4B92-9DFE-6473CB6B3F38}" name="ID" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{FE107DC5-A1C2-4F54-BC82-5BBB32CCABC3}" name="IdEmpresa" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{DE65DD1F-F1BA-4548-A19A-4B9DD2857A6F}" name="Red" dataDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{23F951D4-E519-45F7-81C5-69ED4EA385E4}" name="URLRed" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{E5F1016C-C8F1-4FEA-B687-B57CB00F2E70}" name="Activo" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{E9F2D081-00F6-4B92-9DFE-6473CB6B3F38}" name="ID" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{FE107DC5-A1C2-4F54-BC82-5BBB32CCABC3}" name="IdEmpresa" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{DE65DD1F-F1BA-4548-A19A-4B9DD2857A6F}" name="Red" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{23F951D4-E519-45F7-81C5-69ED4EA385E4}" name="URLRed" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{E5F1016C-C8F1-4FEA-B687-B57CB00F2E70}" name="Activo" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1686,19 +1905,19 @@
 </file>
 
 <file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{C769ADF8-2405-479D-8112-7564F0940768}" name="Tabla22" displayName="Tabla22" ref="A76:J77" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{C769ADF8-2405-479D-8112-7564F0940768}" name="Tabla22" displayName="Tabla22" ref="A76:J77" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
   <autoFilter ref="A76:J77" xr:uid="{A2E83C68-75BA-4C98-B80E-E4E7E2B0B82C}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{173EAAD2-F12F-4372-8FA2-00B32059C1EB}" name="ID" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{3E7AAA46-3847-4587-A43F-E688C1582045}" name="RazonSocial" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{7727AE8E-759C-4DE1-86AE-BDFED86835D0}" name="CUIT" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{BBA783BB-BBBB-4233-929D-4BF68AFA091A}" name="Direccion" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{419A73DC-BE03-4D90-BE0C-9779F3EB2DDB}" name="Localidad" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{BE8C959F-F07F-4076-8E57-3EA25221B957}" name="Partido" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{DB60E2FA-C8A3-4C27-BCAB-41F7E5C99855}" name="IdProvincia" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{EC23197E-97BD-4D2B-AF77-BAEDEAEEEB33}" name="CP" dataDxfId="3"/>
-    <tableColumn id="10" xr3:uid="{7234FBEF-54AA-4FBE-8D11-84EDF024DAB3}" name="Horario" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{2D33166C-2999-4BC9-8B00-7F06B4D84FF1}" name="Activo" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{173EAAD2-F12F-4372-8FA2-00B32059C1EB}" name="ID" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{3E7AAA46-3847-4587-A43F-E688C1582045}" name="RazonSocial" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{7727AE8E-759C-4DE1-86AE-BDFED86835D0}" name="CUIT" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{BBA783BB-BBBB-4233-929D-4BF68AFA091A}" name="Direccion" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{419A73DC-BE03-4D90-BE0C-9779F3EB2DDB}" name="Localidad" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{BE8C959F-F07F-4076-8E57-3EA25221B957}" name="Partido" dataDxfId="12"/>
+    <tableColumn id="8" xr3:uid="{DB60E2FA-C8A3-4C27-BCAB-41F7E5C99855}" name="IdProvincia" dataDxfId="11"/>
+    <tableColumn id="9" xr3:uid="{EC23197E-97BD-4D2B-AF77-BAEDEAEEEB33}" name="CP" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{7234FBEF-54AA-4FBE-8D11-84EDF024DAB3}" name="Horario" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{2D33166C-2999-4BC9-8B00-7F06B4D84FF1}" name="Activo" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1714,7 +1933,7 @@
     <tableColumn id="3" xr3:uid="{473E571D-8BE9-4BD5-B8BD-FC16062FBA4A}" name="Nombre"/>
     <tableColumn id="4" xr3:uid="{BFCDC025-7291-43F4-BF51-02B5C205C0B1}" name="URLImagen"/>
     <tableColumn id="5" xr3:uid="{1AD6DCB5-B8FB-43FC-88CE-E58B0DF75376}" name="Titulo"/>
-    <tableColumn id="6" xr3:uid="{782D732A-1C91-4938-BDF6-8C352984694E}" name="Descripcion" dataDxfId="0"/>
+    <tableColumn id="6" xr3:uid="{782D732A-1C91-4938-BDF6-8C352984694E}" name="Descripcion" dataDxfId="7"/>
     <tableColumn id="7" xr3:uid="{37200F4F-B540-4A63-9F27-255BD55AD0BD}" name="Link"/>
     <tableColumn id="8" xr3:uid="{CB7E851F-8679-4467-A629-18DE76D9185B}" name="LinkSN"/>
     <tableColumn id="9" xr3:uid="{DF01FB7D-3582-4808-83E6-C0BF4EDCA881}" name="LanzamientoSN"/>
@@ -1818,17 +2037,20 @@
 </file>
 
 <file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="28" xr:uid="{E5C72C39-AEF7-4120-A1E5-FF7EB5A3BF17}" name="Tabla28" displayName="Tabla28" ref="A116:K119" totalsRowShown="0">
-  <autoFilter ref="A116:K119" xr:uid="{E5C72C39-AEF7-4120-A1E5-FF7EB5A3BF17}"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="28" xr:uid="{E5C72C39-AEF7-4120-A1E5-FF7EB5A3BF17}" name="Tabla28" displayName="Tabla28" ref="A116:N119" totalsRowShown="0">
+  <autoFilter ref="A116:N119" xr:uid="{E5C72C39-AEF7-4120-A1E5-FF7EB5A3BF17}"/>
+  <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{68690C7C-4428-4270-97EF-F62ECCF7314E}" name="ID"/>
     <tableColumn id="2" xr3:uid="{4ED8A294-C798-4D37-9F33-B2D6E944F3F4}" name="NombreApellido"/>
-    <tableColumn id="3" xr3:uid="{58ED13BD-9B17-4772-85AE-6842EAEE71E5}" name="Mail" dataCellStyle="Hipervínculo"/>
+    <tableColumn id="3" xr3:uid="{58ED13BD-9B17-4772-85AE-6842EAEE71E5}" name="Mail"/>
     <tableColumn id="4" xr3:uid="{94F35AE4-BB92-4E59-9201-C44956F3D992}" name="Telefono"/>
+    <tableColumn id="13" xr3:uid="{588B1BEF-E305-4E5D-9852-932C56C3C6A5}" name="DNI"/>
     <tableColumn id="5" xr3:uid="{B1749734-A73F-4D73-AA3D-233EA5C9D90A}" name="Direccion"/>
+    <tableColumn id="14" xr3:uid="{1A2E94D8-991E-4462-9DB5-6004571D530C}" name="Numeracion"/>
     <tableColumn id="6" xr3:uid="{34C9AECC-F209-4DEB-9823-F29D4B16D927}" name="Piso"/>
-    <tableColumn id="7" xr3:uid="{C0537B94-D9CA-4EAF-B400-6B36DD29ACEF}" name="Departamente"/>
+    <tableColumn id="7" xr3:uid="{C0537B94-D9CA-4EAF-B400-6B36DD29ACEF}" name="DtoLote"/>
     <tableColumn id="8" xr3:uid="{3361C285-84BA-43DF-9B87-BBEA471C74DB}" name="Localidad"/>
+    <tableColumn id="12" xr3:uid="{59C5B181-C2BD-45D3-80AB-DC7BD018DB07}" name="NombreBarrio"/>
     <tableColumn id="9" xr3:uid="{31F8994E-756A-43E8-ADCF-36CDB3FECA27}" name="IdProvincia"/>
     <tableColumn id="10" xr3:uid="{41A026C6-9E4F-4D56-911F-854C5718C114}" name="CodigoPostal "/>
     <tableColumn id="11" xr3:uid="{F8363EAB-1F66-4EC1-BD18-A407969A23F0}" name="Activo"/>
@@ -1865,6 +2087,129 @@
 </table>
 </file>
 
+<file path=xl/tables/table30.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="30" xr:uid="{ED86DA2A-25F1-4521-B911-4F2F84141754}" name="Tabla1131" displayName="Tabla1131" ref="I27:K30" totalsRowShown="0">
+  <autoFilter ref="I27:K30" xr:uid="{ED86DA2A-25F1-4521-B911-4F2F84141754}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{BD27862E-B69D-4739-9293-7780E7F50540}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{2CC93747-5739-472E-B45A-2A8C386A4698}" name="Tipo"/>
+    <tableColumn id="3" xr3:uid="{84D5CE0D-14AB-455F-87C5-2FEDB678E99D}" name="Activo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="31" xr:uid="{8E2D4759-525A-4BF6-8B43-742296BA770E}" name="Tabla2832" displayName="Tabla2832" ref="A130:AA133" totalsRowShown="0">
+  <autoFilter ref="A130:AA133" xr:uid="{8E2D4759-525A-4BF6-8B43-742296BA770E}"/>
+  <tableColumns count="27">
+    <tableColumn id="1" xr3:uid="{0E1797A3-50DB-4C00-8C7D-4E3C78B420E8}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{89511843-4E67-4DCC-9385-A72CA58CD9DF}" name="IdCliente"/>
+    <tableColumn id="3" xr3:uid="{AC688752-919C-4DEB-88C2-DF2E8EF3BD63}" name="IdFormaContacto"/>
+    <tableColumn id="4" xr3:uid="{7D3ED9E7-75FB-4DF7-91B5-E392871B8D43}" name="Fecha1erContacto"/>
+    <tableColumn id="13" xr3:uid="{9EA8476D-DBBE-471F-BFC8-6A291BA80F62}" name="Fecha1eraRespuesta" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{DBAD1119-0F40-4BD3-9842-1192A64CBD53}" name="FechaCierre"/>
+    <tableColumn id="14" xr3:uid="{E39840EE-9AE9-4080-8CE2-7FB8A7484DCE}" name="IdMotivoContacto"/>
+    <tableColumn id="6" xr3:uid="{3E40D0DD-319F-4EE0-B63A-0C3A0E154C0B}" name="IdCodigoReclamo"/>
+    <tableColumn id="7" xr3:uid="{4B7DE31B-73B8-4D00-834D-2635643BB279}" name="IdEstadoReclamo"/>
+    <tableColumn id="8" xr3:uid="{FE3B8DB4-2255-4BFC-9B37-C7BFF06B57C5}" name="Consulta" dataDxfId="5"/>
+    <tableColumn id="12" xr3:uid="{55F91CC0-9D26-4D31-B57A-EA6D64ADC6F2}" name="Solucion" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{617CB8EC-F821-47DB-8753-32FB1A107F1A}" name="IdDatosCompra"/>
+    <tableColumn id="10" xr3:uid="{6329DF96-E0FA-4B62-9E86-F32620647183}" name="FechaOT"/>
+    <tableColumn id="19" xr3:uid="{8C8B6D30-6532-40D3-AE91-9F85D048000E}" name="NumeroOT"/>
+    <tableColumn id="18" xr3:uid="{E9C1402D-DB4C-4575-821C-E3BCE8BFF92F}" name="Repuesto"/>
+    <tableColumn id="17" xr3:uid="{B0292754-890C-4528-9A8A-5828F4F9B90D}" name="Cantidad"/>
+    <tableColumn id="16" xr3:uid="{A6778FEE-2262-4CBF-838B-02B13127B068}" name="IdTipoRespuesto"/>
+    <tableColumn id="15" xr3:uid="{80B09B0D-614F-4682-AC48-16932A68FBE7}" name="IdModoSolucion"/>
+    <tableColumn id="26" xr3:uid="{D0CFCB6C-85C3-4203-BC88-B5B44D980875}" name="Observaciones"/>
+    <tableColumn id="25" xr3:uid="{F4BFD720-8E3F-426D-ADA4-7C9F90A4899F}" name="NumTiendanube"/>
+    <tableColumn id="24" xr3:uid="{6B3FFA65-2F68-49EB-B888-BBCC703D4A24}" name="NumOperacionML"/>
+    <tableColumn id="23" xr3:uid="{3FC47E06-C907-48AC-88A2-78A5DD774483}" name="FechaCompraTNyML"/>
+    <tableColumn id="22" xr3:uid="{66F4482D-A8A4-4473-BB5A-295CD474AC99}" name="MontoCompra"/>
+    <tableColumn id="21" xr3:uid="{542D0822-2C0C-4D15-9CF7-69786B2FAC9E}" name="NumFacturaRepuesto"/>
+    <tableColumn id="27" xr3:uid="{2042778B-F258-4301-ACB2-373EBA165DDE}" name="NumGuiaCorreo"/>
+    <tableColumn id="20" xr3:uid="{32B933EB-3FCC-4023-AEE3-097C0D15D848}" name="IdRegistro"/>
+    <tableColumn id="11" xr3:uid="{2D22868C-E2A5-4CBF-AB5B-372B1B35B2F1}" name="Activo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="32" xr:uid="{3120E102-167B-4968-9C4B-27E2DB027BCB}" name="Tabla32" displayName="Tabla32" ref="H123:J126" totalsRowShown="0">
+  <autoFilter ref="H123:J126" xr:uid="{3120E102-167B-4968-9C4B-27E2DB027BCB}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{EE3C83CC-21D0-401F-ACA8-188E9E4192B7}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{BFFDAC8F-7B87-4E2F-AD42-AC3AF42581A7}" name="Estado"/>
+    <tableColumn id="3" xr3:uid="{20032F58-F88C-40E9-AFEF-F03D88271F9B}" name="Activo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="33" xr:uid="{34A657EC-FBEA-404C-97B4-37560A8B1A66}" name="Tabla3234" displayName="Tabla3234" ref="L123:N126" totalsRowShown="0">
+  <autoFilter ref="L123:N126" xr:uid="{34A657EC-FBEA-404C-97B4-37560A8B1A66}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{658D1EAF-2C94-4837-B563-9F06CC1CA9EF}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{318D820E-B0F1-494E-9ACD-56B42577BACD}" name="ModoSolucion"/>
+    <tableColumn id="3" xr3:uid="{360683CD-7223-43C9-A749-F1ABB92CECD3}" name="Activo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table34.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="34" xr:uid="{C42E2A91-D18B-46C4-92DD-70DB8D684714}" name="Tabla3235" displayName="Tabla3235" ref="A137:C140" totalsRowShown="0">
+  <autoFilter ref="A137:C140" xr:uid="{C42E2A91-D18B-46C4-92DD-70DB8D684714}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{88C1E49B-9084-43B7-8C97-74BDA0019AE3}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{2970C4AF-BB3E-4C97-8BFF-23A5D49FA124}" name="TipoRepuesto"/>
+    <tableColumn id="3" xr3:uid="{F3C9A899-9552-4048-9F28-4D78497C0EAC}" name="Activo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table35.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="35" xr:uid="{2AE76666-B21F-4F04-9BC2-2C21A3B9D534}" name="Tabla323536" displayName="Tabla323536" ref="E137:G140" totalsRowShown="0">
+  <autoFilter ref="E137:G140" xr:uid="{2AE76666-B21F-4F04-9BC2-2C21A3B9D534}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{9344C3CF-9F17-4477-B852-2D61C58EE5B7}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{4FB40FD6-2D91-42DF-AC2E-AE94EEFD7AA1}" name="FormaContacto"/>
+    <tableColumn id="3" xr3:uid="{B40604D0-C82E-4B19-8045-D75B1EF483DB}" name="Activo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table36.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="36" xr:uid="{F957B04B-4005-4CCC-9E90-A3E625FA5D35}" name="Tabla32353637" displayName="Tabla32353637" ref="I137:L140" totalsRowShown="0">
+  <autoFilter ref="I137:L140" xr:uid="{F957B04B-4005-4CCC-9E90-A3E625FA5D35}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{CA64DBE0-508E-4B80-AC77-B1B1E7C15BDC}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{112228D4-9880-4A08-B8FC-D853213893FD}" name="CodigoMotivo"/>
+    <tableColumn id="4" xr3:uid="{83C3478C-1D40-4D25-A416-65C24BEC74A0}" name="MotivoContacto"/>
+    <tableColumn id="3" xr3:uid="{499D04F2-F038-4388-8B00-5454D94F0C5A}" name="Activo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table37.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="37" xr:uid="{FDA8E030-FF4B-4EFC-90D1-9EA6BEF24240}" name="Tabla3235363738" displayName="Tabla3235363738" ref="N137:R140" totalsRowShown="0">
+  <autoFilter ref="N137:R140" xr:uid="{FDA8E030-FF4B-4EFC-90D1-9EA6BEF24240}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{5560DF7C-FEE5-456B-92EA-203150657B26}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{1F149BD5-C727-437F-8393-C5987FBE588D}" name="CodigoMotivo"/>
+    <tableColumn id="4" xr3:uid="{8CFC6924-9C12-4FBB-9472-05F51F199A0A}" name="Fecha" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{47C9DE2B-FED3-499A-92E4-96789BCD9F70}" name="Registro" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{03ADB1E3-143F-49CF-A27C-B2C1272966DD}" name="Activo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{E93F9B0B-4EAC-4696-9C48-7CF3279FF43E}" name="Tabla136" displayName="Tabla136" ref="A20:D23" totalsRowShown="0">
   <autoFilter ref="A20:D23" xr:uid="{E93F9B0B-4EAC-4696-9C48-7CF3279FF43E}"/>
@@ -1888,7 +2233,7 @@
     <tableColumn id="4" xr3:uid="{33CF0639-7E0E-4323-ABAC-57E9E79BAC94}" name="URLManual"/>
     <tableColumn id="6" xr3:uid="{8FB3C041-5F4E-4C6B-BFEA-F7EF8CCA380F}" name="URLRepuestos"/>
     <tableColumn id="7" xr3:uid="{19883A37-D7EF-411E-B5D4-0F9C58EA4DF5}" name="URLPlanos"/>
-    <tableColumn id="5" xr3:uid="{9FBFC04D-E638-4A8E-BF60-60BF85B463B6}" name="Activo" dataDxfId="55"/>
+    <tableColumn id="5" xr3:uid="{9FBFC04D-E638-4A8E-BF60-60BF85B463B6}" name="Activo" dataDxfId="60"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1915,7 +2260,7 @@
   <autoFilter ref="A6:G9" xr:uid="{00F67F5D-77F7-41B7-A265-5E336044A6C5}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{F32EBD58-4145-475F-A8DD-60533C773560}" name="ID"/>
-    <tableColumn id="5" xr3:uid="{BA938A3C-223C-48BE-9D99-D519D9B88EDF}" name="Nombre" dataDxfId="54"/>
+    <tableColumn id="5" xr3:uid="{BA938A3C-223C-48BE-9D99-D519D9B88EDF}" name="Nombre" dataDxfId="59"/>
     <tableColumn id="2" xr3:uid="{BF58FE61-5919-4F9C-BC69-7F6F4B0BCCB1}" name="Apellido"/>
     <tableColumn id="4" xr3:uid="{B217BF12-7466-47C6-83EC-0600B0F7EE4B}" name="Mail">
       <calculatedColumnFormula>CONCATENATE(Tabla15[[#This Row],[Nombre]],Tabla15[[#This Row],[Apellido]],"@andez.com.ar")</calculatedColumnFormula>
@@ -1941,11 +2286,12 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{F6B3327E-5FDA-4BB7-AACF-FABE81E48666}" name="Tabla11" displayName="Tabla11" ref="I27:K30" totalsRowShown="0">
-  <autoFilter ref="I27:K30" xr:uid="{F6B3327E-5FDA-4BB7-AACF-FABE81E48666}"/>
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{F6B3327E-5FDA-4BB7-AACF-FABE81E48666}" name="Tabla11" displayName="Tabla11" ref="M27:P30" totalsRowShown="0">
+  <autoFilter ref="M27:P30" xr:uid="{F6B3327E-5FDA-4BB7-AACF-FABE81E48666}"/>
+  <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{26F76265-568B-4A28-AA28-6DA1CF7F5397}" name="ID"/>
     <tableColumn id="2" xr3:uid="{A81F65B5-D9C2-4F7A-9651-B297627921BE}" name="Tipo"/>
+    <tableColumn id="4" xr3:uid="{DAB68CD9-3919-4F19-B6D2-6F30B1F19B70}" name="Subtipo"/>
     <tableColumn id="3" xr3:uid="{6BF61F58-B964-4C51-B2A6-1D6E99603A94}" name="Activo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2269,25 +2615,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD350C1D-1850-4BF9-ABCF-FA1A23EC1542}">
-  <dimension ref="A1:P126"/>
+  <dimension ref="A1:AA140"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.21875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="28.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="24.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.21875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="27.21875" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="31.44140625" customWidth="1"/>
+    <col min="11" max="11" width="24.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="18.109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="24.88671875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="17" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="19.77734375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="22" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="23.21875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
@@ -2303,20 +2660,20 @@
     </row>
     <row r="4" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="5" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="18"/>
-      <c r="I5" s="16" t="s">
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="22"/>
+      <c r="I5" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="J5" s="17"/>
-      <c r="K5" s="18"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="22"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
@@ -2451,26 +2808,26 @@
     </row>
     <row r="11" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="21"/>
-      <c r="G12" s="19" t="s">
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="19"/>
+      <c r="G12" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="H12" s="20"/>
-      <c r="I12" s="20"/>
-      <c r="J12" s="20"/>
-      <c r="K12" s="21"/>
-      <c r="M12" s="19" t="s">
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
+      <c r="J12" s="18"/>
+      <c r="K12" s="19"/>
+      <c r="M12" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="N12" s="20"/>
-      <c r="O12" s="20"/>
-      <c r="P12" s="21"/>
+      <c r="N12" s="18"/>
+      <c r="O12" s="18"/>
+      <c r="P12" s="19"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
@@ -2648,25 +3005,25 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A19" s="19" t="s">
+    <row r="18" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A19" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="21"/>
-      <c r="F19" s="19" t="s">
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="19"/>
+      <c r="F19" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="20"/>
-      <c r="J19" s="20"/>
-      <c r="K19" s="20"/>
-      <c r="L19" s="21"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G19" s="18"/>
+      <c r="H19" s="18"/>
+      <c r="I19" s="18"/>
+      <c r="J19" s="18"/>
+      <c r="K19" s="18"/>
+      <c r="L19" s="19"/>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>1</v>
       </c>
@@ -2701,7 +3058,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>1</v>
       </c>
@@ -2736,7 +3093,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>2</v>
       </c>
@@ -2771,7 +3128,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
         <v>3</v>
       </c>
@@ -2806,24 +3163,30 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A26" s="19" t="s">
+    <row r="25" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A26" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
-      <c r="E26" s="20"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="21"/>
-      <c r="I26" s="19" t="s">
+      <c r="B26" s="18"/>
+      <c r="C26" s="18"/>
+      <c r="D26" s="18"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="19"/>
+      <c r="I26" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="J26" s="20"/>
-      <c r="K26" s="21"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="J26" s="18"/>
+      <c r="K26" s="19"/>
+      <c r="M26" s="17" t="s">
+        <v>222</v>
+      </c>
+      <c r="N26" s="18"/>
+      <c r="O26" s="18"/>
+      <c r="P26" s="19"/>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>1</v>
       </c>
@@ -2854,8 +3217,20 @@
       <c r="K27" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M27" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="N27" t="s">
+        <v>60</v>
+      </c>
+      <c r="O27" t="s">
+        <v>221</v>
+      </c>
+      <c r="P27" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>1</v>
       </c>
@@ -2881,13 +3256,25 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
+        <v>223</v>
+      </c>
+      <c r="K28" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M28" s="1">
+        <v>1</v>
+      </c>
+      <c r="N28">
+        <v>1</v>
+      </c>
+      <c r="O28" t="s">
         <v>61</v>
       </c>
-      <c r="K28" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="P28" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>2</v>
       </c>
@@ -2913,13 +3300,25 @@
         <v>2</v>
       </c>
       <c r="J29" t="s">
+        <v>224</v>
+      </c>
+      <c r="K29" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M29" s="1">
+        <v>2</v>
+      </c>
+      <c r="N29">
+        <v>1</v>
+      </c>
+      <c r="O29" t="s">
         <v>62</v>
       </c>
-      <c r="K29" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="P29" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="3">
         <v>3</v>
       </c>
@@ -2950,26 +3349,38 @@
       <c r="K30" s="5" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+      <c r="M30" s="3">
+        <v>3</v>
+      </c>
+      <c r="N30" s="4">
+        <v>3</v>
+      </c>
+      <c r="O30" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="P30" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A33" s="19" t="s">
+      <c r="A33" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
-      <c r="D33" s="20"/>
-      <c r="E33" s="20"/>
-      <c r="F33" s="20"/>
-      <c r="G33" s="20"/>
-      <c r="H33" s="20"/>
-      <c r="I33" s="21"/>
-      <c r="K33" s="19" t="s">
+      <c r="B33" s="18"/>
+      <c r="C33" s="18"/>
+      <c r="D33" s="18"/>
+      <c r="E33" s="18"/>
+      <c r="F33" s="18"/>
+      <c r="G33" s="18"/>
+      <c r="H33" s="18"/>
+      <c r="I33" s="19"/>
+      <c r="K33" s="17" t="s">
         <v>134</v>
       </c>
-      <c r="L33" s="20"/>
-      <c r="M33" s="20"/>
-      <c r="N33" s="21"/>
+      <c r="L33" s="18"/>
+      <c r="M33" s="18"/>
+      <c r="N33" s="19"/>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
@@ -3137,22 +3548,22 @@
     </row>
     <row r="39" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="40" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A40" s="19" t="s">
+      <c r="A40" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="B40" s="20"/>
-      <c r="C40" s="20"/>
-      <c r="D40" s="20"/>
-      <c r="E40" s="20"/>
-      <c r="F40" s="21"/>
-      <c r="H40" s="19" t="s">
+      <c r="B40" s="18"/>
+      <c r="C40" s="18"/>
+      <c r="D40" s="18"/>
+      <c r="E40" s="18"/>
+      <c r="F40" s="19"/>
+      <c r="H40" s="17" t="s">
         <v>152</v>
       </c>
-      <c r="I40" s="20"/>
-      <c r="J40" s="20"/>
-      <c r="K40" s="20"/>
-      <c r="L40" s="20"/>
-      <c r="M40" s="21"/>
+      <c r="I40" s="18"/>
+      <c r="J40" s="18"/>
+      <c r="K40" s="18"/>
+      <c r="L40" s="18"/>
+      <c r="M40" s="19"/>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
@@ -3308,21 +3719,22 @@
     </row>
     <row r="46" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A47" s="19" t="s">
+      <c r="A47" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="B47" s="20"/>
-      <c r="C47" s="20"/>
-      <c r="D47" s="21"/>
-      <c r="F47" s="19" t="s">
+      <c r="B47" s="18"/>
+      <c r="C47" s="18"/>
+      <c r="D47" s="19"/>
+      <c r="F47" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="G47" s="20"/>
-      <c r="H47" s="20"/>
-      <c r="I47" s="20"/>
-      <c r="J47" s="20"/>
-      <c r="K47" s="20"/>
-      <c r="L47" s="21"/>
+      <c r="G47" s="18"/>
+      <c r="H47" s="18"/>
+      <c r="I47" s="18"/>
+      <c r="J47" s="18"/>
+      <c r="K47" s="18"/>
+      <c r="L47" s="18"/>
+      <c r="M47" s="19"/>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
@@ -3340,26 +3752,29 @@
       <c r="F48" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G48" t="s">
+      <c r="G48" s="23" t="s">
         <v>73</v>
       </c>
-      <c r="H48" t="s">
+      <c r="H48" s="23" t="s">
         <v>74</v>
       </c>
-      <c r="I48" t="s">
+      <c r="I48" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="J48" t="s">
+      <c r="J48" s="23" t="s">
         <v>76</v>
       </c>
-      <c r="K48" t="s">
+      <c r="K48" s="23" t="s">
         <v>77</v>
       </c>
-      <c r="L48" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L48" s="23" t="s">
+        <v>280</v>
+      </c>
+      <c r="M48" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A49" s="1">
         <v>1</v>
       </c>
@@ -3375,26 +3790,29 @@
       <c r="F49" s="1">
         <v>1</v>
       </c>
-      <c r="G49" t="s">
+      <c r="G49" s="23" t="s">
         <v>78</v>
       </c>
-      <c r="H49">
-        <v>1</v>
-      </c>
-      <c r="I49" s="6" t="s">
+      <c r="H49" s="23">
+        <v>1</v>
+      </c>
+      <c r="I49" s="29" t="s">
         <v>80</v>
       </c>
-      <c r="J49" s="6" t="s">
+      <c r="J49" s="29" t="s">
         <v>80</v>
       </c>
-      <c r="K49">
+      <c r="K49" s="23">
         <v>4</v>
       </c>
-      <c r="L49" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L49" s="23" t="s">
+        <v>282</v>
+      </c>
+      <c r="M49" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A50" s="1">
         <v>2</v>
       </c>
@@ -3410,26 +3828,29 @@
       <c r="F50" s="1">
         <v>2</v>
       </c>
-      <c r="G50" t="s">
+      <c r="G50" s="23" t="s">
         <v>79</v>
       </c>
-      <c r="H50">
-        <v>1</v>
-      </c>
-      <c r="I50" s="6" t="s">
+      <c r="H50" s="23">
+        <v>1</v>
+      </c>
+      <c r="I50" s="29" t="s">
         <v>81</v>
       </c>
-      <c r="J50" s="6" t="s">
+      <c r="J50" s="29" t="s">
         <v>81</v>
       </c>
-      <c r="K50">
+      <c r="K50" s="23">
         <v>5</v>
       </c>
-      <c r="L50" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="L50" s="23" t="s">
+        <v>282</v>
+      </c>
+      <c r="M50" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="3">
         <v>3</v>
       </c>
@@ -3460,25 +3881,28 @@
       <c r="K51" s="4">
         <v>6</v>
       </c>
-      <c r="L51" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A54" s="19" t="s">
+      <c r="L51" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="M51" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A54" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="B54" s="20"/>
-      <c r="C54" s="20"/>
-      <c r="D54" s="20"/>
-      <c r="E54" s="20"/>
-      <c r="F54" s="20"/>
-      <c r="G54" s="20"/>
-      <c r="H54" s="20"/>
-      <c r="I54" s="21"/>
-    </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B54" s="18"/>
+      <c r="C54" s="18"/>
+      <c r="D54" s="18"/>
+      <c r="E54" s="18"/>
+      <c r="F54" s="18"/>
+      <c r="G54" s="18"/>
+      <c r="H54" s="18"/>
+      <c r="I54" s="19"/>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>1</v>
       </c>
@@ -3507,7 +3931,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A56" s="1">
         <v>1</v>
       </c>
@@ -3536,7 +3960,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A57" s="1">
         <v>2</v>
       </c>
@@ -3565,7 +3989,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A58" s="3">
         <v>3</v>
       </c>
@@ -3594,24 +4018,24 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A61" s="19" t="s">
+    <row r="60" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A61" s="17" t="s">
         <v>135</v>
       </c>
-      <c r="B61" s="20"/>
-      <c r="C61" s="20"/>
-      <c r="D61" s="20"/>
-      <c r="E61" s="21"/>
-      <c r="G61" s="19" t="s">
+      <c r="B61" s="18"/>
+      <c r="C61" s="18"/>
+      <c r="D61" s="18"/>
+      <c r="E61" s="19"/>
+      <c r="G61" s="17" t="s">
         <v>136</v>
       </c>
-      <c r="H61" s="20"/>
-      <c r="I61" s="20"/>
-      <c r="J61" s="20"/>
-      <c r="K61" s="21"/>
-    </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H61" s="18"/>
+      <c r="I61" s="18"/>
+      <c r="J61" s="18"/>
+      <c r="K61" s="19"/>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>1</v>
       </c>
@@ -3643,7 +4067,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A63" s="1">
         <v>1</v>
       </c>
@@ -3676,7 +4100,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A64" s="1">
         <v>2</v>
       </c>
@@ -3744,13 +4168,13 @@
     </row>
     <row r="67" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="68" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A68" s="19" t="s">
+      <c r="A68" s="17" t="s">
         <v>137</v>
       </c>
-      <c r="B68" s="20"/>
-      <c r="C68" s="20"/>
-      <c r="D68" s="20"/>
-      <c r="E68" s="21"/>
+      <c r="B68" s="18"/>
+      <c r="C68" s="18"/>
+      <c r="D68" s="18"/>
+      <c r="E68" s="19"/>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
@@ -3822,18 +4246,18 @@
     </row>
     <row r="74" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="75" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A75" s="19" t="s">
+      <c r="A75" s="17" t="s">
         <v>139</v>
       </c>
-      <c r="B75" s="20"/>
-      <c r="C75" s="20"/>
-      <c r="D75" s="20"/>
-      <c r="E75" s="20"/>
-      <c r="F75" s="20"/>
-      <c r="G75" s="20"/>
-      <c r="H75" s="20"/>
-      <c r="I75" s="20"/>
-      <c r="J75" s="21"/>
+      <c r="B75" s="18"/>
+      <c r="C75" s="18"/>
+      <c r="D75" s="18"/>
+      <c r="E75" s="18"/>
+      <c r="F75" s="18"/>
+      <c r="G75" s="18"/>
+      <c r="H75" s="18"/>
+      <c r="I75" s="18"/>
+      <c r="J75" s="19"/>
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
@@ -3901,20 +4325,20 @@
     </row>
     <row r="79" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="80" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A80" s="19" t="s">
+      <c r="A80" s="17" t="s">
         <v>153</v>
       </c>
-      <c r="B80" s="20"/>
-      <c r="C80" s="20"/>
-      <c r="D80" s="20"/>
-      <c r="E80" s="20"/>
-      <c r="F80" s="20"/>
-      <c r="G80" s="20"/>
-      <c r="H80" s="20"/>
-      <c r="I80" s="20"/>
-      <c r="J80" s="20"/>
-      <c r="K80" s="20"/>
-      <c r="L80" s="21"/>
+      <c r="B80" s="18"/>
+      <c r="C80" s="18"/>
+      <c r="D80" s="18"/>
+      <c r="E80" s="18"/>
+      <c r="F80" s="18"/>
+      <c r="G80" s="18"/>
+      <c r="H80" s="18"/>
+      <c r="I80" s="18"/>
+      <c r="J80" s="18"/>
+      <c r="K80" s="18"/>
+      <c r="L80" s="19"/>
     </row>
     <row r="81" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
@@ -4070,22 +4494,22 @@
     </row>
     <row r="86" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="87" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A87" s="19" t="s">
+      <c r="A87" s="17" t="s">
         <v>165</v>
       </c>
-      <c r="B87" s="21"/>
-      <c r="D87" s="19" t="s">
+      <c r="B87" s="19"/>
+      <c r="D87" s="17" t="s">
         <v>168</v>
       </c>
-      <c r="E87" s="20"/>
-      <c r="F87" s="21"/>
-      <c r="H87" s="19" t="s">
+      <c r="E87" s="18"/>
+      <c r="F87" s="19"/>
+      <c r="H87" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="I87" s="20"/>
-      <c r="J87" s="20"/>
-      <c r="K87" s="20"/>
-      <c r="L87" s="21"/>
+      <c r="I87" s="18"/>
+      <c r="J87" s="18"/>
+      <c r="K87" s="18"/>
+      <c r="L87" s="19"/>
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
@@ -4217,22 +4641,22 @@
     </row>
     <row r="93" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="94" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A94" s="19" t="s">
+      <c r="A94" s="17" t="s">
         <v>196</v>
       </c>
-      <c r="B94" s="20"/>
-      <c r="C94" s="20"/>
-      <c r="D94" s="20"/>
-      <c r="E94" s="20"/>
-      <c r="F94" s="20"/>
-      <c r="G94" s="20"/>
-      <c r="H94" s="20"/>
-      <c r="I94" s="20"/>
-      <c r="J94" s="20"/>
-      <c r="K94" s="20"/>
-      <c r="L94" s="20"/>
-      <c r="M94" s="20"/>
-      <c r="N94" s="21"/>
+      <c r="B94" s="18"/>
+      <c r="C94" s="18"/>
+      <c r="D94" s="18"/>
+      <c r="E94" s="18"/>
+      <c r="F94" s="18"/>
+      <c r="G94" s="18"/>
+      <c r="H94" s="18"/>
+      <c r="I94" s="18"/>
+      <c r="J94" s="18"/>
+      <c r="K94" s="18"/>
+      <c r="L94" s="18"/>
+      <c r="M94" s="18"/>
+      <c r="N94" s="19"/>
     </row>
     <row r="95" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
@@ -4412,17 +4836,17 @@
     </row>
     <row r="100" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="101" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A101" s="19" t="s">
+      <c r="A101" s="17" t="s">
         <v>195</v>
       </c>
-      <c r="B101" s="20"/>
-      <c r="C101" s="20"/>
-      <c r="D101" s="20"/>
-      <c r="E101" s="20"/>
-      <c r="F101" s="20"/>
-      <c r="G101" s="20"/>
-      <c r="H101" s="20"/>
-      <c r="I101" s="21"/>
+      <c r="B101" s="18"/>
+      <c r="C101" s="18"/>
+      <c r="D101" s="18"/>
+      <c r="E101" s="18"/>
+      <c r="F101" s="18"/>
+      <c r="G101" s="18"/>
+      <c r="H101" s="18"/>
+      <c r="I101" s="19"/>
     </row>
     <row r="102" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
@@ -4542,13 +4966,13 @@
     </row>
     <row r="107" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="108" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A108" s="19" t="s">
+      <c r="A108" s="17" t="s">
         <v>198</v>
       </c>
-      <c r="B108" s="20"/>
-      <c r="C108" s="20"/>
-      <c r="D108" s="20"/>
-      <c r="E108" s="21"/>
+      <c r="B108" s="18"/>
+      <c r="C108" s="18"/>
+      <c r="D108" s="18"/>
+      <c r="E108" s="19"/>
     </row>
     <row r="109" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
@@ -4618,241 +5042,344 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A115" s="16" t="s">
+    <row r="114" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="115" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A115" s="17" t="s">
         <v>205</v>
       </c>
-      <c r="B115" s="17"/>
-      <c r="C115" s="17"/>
-      <c r="D115" s="17"/>
-      <c r="E115" s="17"/>
-      <c r="F115" s="17"/>
-      <c r="G115" s="17"/>
-      <c r="H115" s="17"/>
-      <c r="I115" s="17"/>
-      <c r="J115" s="17"/>
+      <c r="B115" s="18"/>
+      <c r="C115" s="18"/>
+      <c r="D115" s="18"/>
+      <c r="E115" s="18"/>
+      <c r="F115" s="18"/>
+      <c r="G115" s="18"/>
+      <c r="H115" s="18"/>
+      <c r="I115" s="18"/>
+      <c r="J115" s="18"/>
       <c r="K115" s="18"/>
-    </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L115" s="18"/>
+      <c r="M115" s="18"/>
+      <c r="N115" s="19"/>
+    </row>
+    <row r="116" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B116" s="22" t="s">
+      <c r="B116" t="s">
         <v>206</v>
       </c>
-      <c r="C116" s="22" t="s">
+      <c r="C116" t="s">
         <v>39</v>
       </c>
-      <c r="D116" s="22" t="s">
+      <c r="D116" t="s">
         <v>90</v>
       </c>
-      <c r="E116" s="22" t="s">
+      <c r="E116" t="s">
+        <v>226</v>
+      </c>
+      <c r="F116" t="s">
         <v>88</v>
       </c>
-      <c r="F116" s="22" t="s">
+      <c r="G116" t="s">
+        <v>227</v>
+      </c>
+      <c r="H116" t="s">
         <v>207</v>
       </c>
-      <c r="G116" s="22" t="s">
+      <c r="I116" t="s">
+        <v>228</v>
+      </c>
+      <c r="J116" t="s">
+        <v>144</v>
+      </c>
+      <c r="K116" t="s">
+        <v>225</v>
+      </c>
+      <c r="L116" t="s">
+        <v>89</v>
+      </c>
+      <c r="M116" t="s">
         <v>208</v>
       </c>
-      <c r="H116" s="22" t="s">
-        <v>144</v>
-      </c>
-      <c r="I116" s="22" t="s">
-        <v>89</v>
-      </c>
-      <c r="J116" s="22" t="s">
+      <c r="N116" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="117" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A117" s="1">
+        <v>1</v>
+      </c>
+      <c r="B117" t="s">
         <v>209</v>
       </c>
-      <c r="K116" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A117" s="1">
-        <v>1</v>
-      </c>
-      <c r="B117" s="22" t="s">
+      <c r="C117" t="s">
+        <v>212</v>
+      </c>
+      <c r="D117">
+        <v>5555511111</v>
+      </c>
+      <c r="E117">
+        <v>3342342342</v>
+      </c>
+      <c r="F117" t="s">
+        <v>191</v>
+      </c>
+      <c r="G117">
+        <v>1545</v>
+      </c>
+      <c r="H117" t="s">
+        <v>191</v>
+      </c>
+      <c r="I117" t="s">
+        <v>191</v>
+      </c>
+      <c r="J117" t="s">
+        <v>191</v>
+      </c>
+      <c r="K117" t="s">
+        <v>191</v>
+      </c>
+      <c r="L117">
+        <v>1</v>
+      </c>
+      <c r="M117" t="s">
+        <v>191</v>
+      </c>
+      <c r="N117" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A118" s="1">
+        <v>2</v>
+      </c>
+      <c r="B118" t="s">
         <v>210</v>
       </c>
-      <c r="C117" s="23" t="s">
+      <c r="C118" t="s">
         <v>213</v>
       </c>
-      <c r="D117" s="22">
-        <v>5555511111</v>
-      </c>
-      <c r="E117" s="22" t="s">
-        <v>191</v>
-      </c>
-      <c r="F117" s="22" t="s">
-        <v>191</v>
-      </c>
-      <c r="G117" s="22" t="s">
-        <v>191</v>
-      </c>
-      <c r="H117" s="22" t="s">
-        <v>191</v>
-      </c>
-      <c r="I117" s="22">
-        <v>1</v>
-      </c>
-      <c r="J117" s="22" t="s">
-        <v>191</v>
-      </c>
-      <c r="K117" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A118" s="1">
-        <v>2</v>
-      </c>
-      <c r="B118" s="22" t="s">
+      <c r="D118">
+        <v>5555522222</v>
+      </c>
+      <c r="E118">
+        <v>3423423423</v>
+      </c>
+      <c r="F118" t="s">
+        <v>191</v>
+      </c>
+      <c r="G118">
+        <v>6985</v>
+      </c>
+      <c r="H118" t="s">
+        <v>191</v>
+      </c>
+      <c r="I118" t="s">
+        <v>191</v>
+      </c>
+      <c r="J118" t="s">
+        <v>191</v>
+      </c>
+      <c r="K118" t="s">
+        <v>191</v>
+      </c>
+      <c r="L118">
+        <v>1</v>
+      </c>
+      <c r="M118" t="s">
+        <v>191</v>
+      </c>
+      <c r="N118" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A119" s="3">
+        <v>3</v>
+      </c>
+      <c r="B119" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="C118" s="23" t="s">
+      <c r="C119" s="4" t="s">
         <v>214</v>
-      </c>
-      <c r="D118" s="22">
-        <v>5555522222</v>
-      </c>
-      <c r="E118" s="22" t="s">
-        <v>191</v>
-      </c>
-      <c r="F118" s="22" t="s">
-        <v>191</v>
-      </c>
-      <c r="G118" s="22" t="s">
-        <v>191</v>
-      </c>
-      <c r="H118" s="22" t="s">
-        <v>191</v>
-      </c>
-      <c r="I118" s="22">
-        <v>1</v>
-      </c>
-      <c r="J118" s="22" t="s">
-        <v>191</v>
-      </c>
-      <c r="K118" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="119" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A119" s="3">
-        <v>3</v>
-      </c>
-      <c r="B119" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="C119" s="24" t="s">
-        <v>215</v>
       </c>
       <c r="D119" s="4">
         <v>5555533332</v>
       </c>
-      <c r="E119" s="4" t="s">
+      <c r="E119" s="4">
+        <v>3423423423</v>
+      </c>
+      <c r="F119" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="G119" s="4">
+        <v>4784</v>
+      </c>
+      <c r="H119" s="4">
+        <v>2</v>
+      </c>
+      <c r="I119" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="J119" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="K119" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="L119" s="4">
+        <v>1</v>
+      </c>
+      <c r="M119" s="4">
+        <v>1605</v>
+      </c>
+      <c r="N119" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="122" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A122" s="17" t="s">
         <v>217</v>
       </c>
-      <c r="F119" s="4">
-        <v>2</v>
-      </c>
-      <c r="G119" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="H119" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="I119" s="4">
-        <v>1</v>
-      </c>
-      <c r="J119" s="4">
-        <v>1605</v>
-      </c>
-      <c r="K119" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="121" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A122" s="16" t="s">
+      <c r="B122" s="18"/>
+      <c r="C122" s="18"/>
+      <c r="D122" s="18"/>
+      <c r="E122" s="18"/>
+      <c r="F122" s="19"/>
+      <c r="H122" s="17" t="s">
+        <v>257</v>
+      </c>
+      <c r="I122" s="18"/>
+      <c r="J122" s="19"/>
+      <c r="L122" s="17" t="s">
+        <v>262</v>
+      </c>
+      <c r="M122" s="18"/>
+      <c r="N122" s="19"/>
+    </row>
+    <row r="123" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A123" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B123" t="s">
         <v>218</v>
       </c>
-      <c r="B122" s="17"/>
-      <c r="C122" s="17"/>
-      <c r="D122" s="17"/>
-      <c r="E122" s="17"/>
-      <c r="F122" s="18"/>
-    </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A123" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B123" s="22" t="s">
+      <c r="C123" t="s">
         <v>219</v>
       </c>
-      <c r="C123" s="22" t="s">
+      <c r="D123" t="s">
         <v>220</v>
       </c>
-      <c r="D123" s="22" t="s">
-        <v>221</v>
-      </c>
-      <c r="E123" s="22" t="s">
+      <c r="E123" t="s">
         <v>116</v>
       </c>
       <c r="F123" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H123" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I123" s="23" t="s">
+        <v>258</v>
+      </c>
+      <c r="J123" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="L123" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="M123" s="23" t="s">
+        <v>262</v>
+      </c>
+      <c r="N123" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="124" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A124" s="1">
         <v>1</v>
       </c>
-      <c r="B124" s="22">
-        <v>1</v>
-      </c>
-      <c r="C124" s="22" t="s">
-        <v>191</v>
-      </c>
-      <c r="D124" s="22" t="s">
-        <v>191</v>
-      </c>
-      <c r="E124" s="22">
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>191</v>
+      </c>
+      <c r="D124" t="s">
+        <v>191</v>
+      </c>
+      <c r="E124">
         <v>1</v>
       </c>
       <c r="F124" s="2" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H124" s="1">
+        <v>1</v>
+      </c>
+      <c r="I124" s="23" t="s">
+        <v>259</v>
+      </c>
+      <c r="J124" s="26" t="b">
+        <v>1</v>
+      </c>
+      <c r="L124" s="1">
+        <v>1</v>
+      </c>
+      <c r="M124" s="23" t="s">
+        <v>263</v>
+      </c>
+      <c r="N124" s="26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A125" s="1">
         <v>2</v>
       </c>
-      <c r="B125" s="22">
-        <v>2</v>
-      </c>
-      <c r="C125" s="22" t="s">
-        <v>191</v>
-      </c>
-      <c r="D125" s="22" t="s">
-        <v>191</v>
-      </c>
-      <c r="E125" s="22">
+      <c r="B125">
+        <v>2</v>
+      </c>
+      <c r="C125" t="s">
+        <v>191</v>
+      </c>
+      <c r="D125" t="s">
+        <v>191</v>
+      </c>
+      <c r="E125">
         <v>2</v>
       </c>
       <c r="F125" s="2" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="126" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="H125" s="1">
+        <v>2</v>
+      </c>
+      <c r="I125" s="23" t="s">
+        <v>260</v>
+      </c>
+      <c r="J125" s="27" t="b">
+        <v>1</v>
+      </c>
+      <c r="L125" s="1">
+        <v>2</v>
+      </c>
+      <c r="M125" s="23" t="s">
+        <v>264</v>
+      </c>
+      <c r="N125" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A126" s="3">
         <v>3</v>
       </c>
       <c r="B126" s="4">
         <v>2</v>
       </c>
-      <c r="C126" s="25">
+      <c r="C126" s="16">
         <v>44724</v>
       </c>
       <c r="D126" s="4">
@@ -4864,10 +5391,613 @@
       <c r="F126" s="5" t="b">
         <v>1</v>
       </c>
+      <c r="H126" s="3">
+        <v>3</v>
+      </c>
+      <c r="I126" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="J126" s="28" t="b">
+        <v>1</v>
+      </c>
+      <c r="L126" s="3">
+        <v>3</v>
+      </c>
+      <c r="M126" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="N126" s="28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="128" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="129" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A129" s="17" t="s">
+        <v>231</v>
+      </c>
+      <c r="B129" s="18"/>
+      <c r="C129" s="18"/>
+      <c r="D129" s="18"/>
+      <c r="E129" s="18"/>
+      <c r="F129" s="18"/>
+      <c r="G129" s="18"/>
+      <c r="H129" s="18"/>
+      <c r="I129" s="18"/>
+      <c r="J129" s="18"/>
+      <c r="K129" s="18"/>
+      <c r="L129" s="18"/>
+      <c r="M129" s="18"/>
+      <c r="N129" s="18"/>
+      <c r="O129" s="18"/>
+      <c r="P129" s="18"/>
+      <c r="Q129" s="18"/>
+      <c r="R129" s="18"/>
+      <c r="S129" s="18"/>
+      <c r="T129" s="18"/>
+      <c r="U129" s="18"/>
+      <c r="V129" s="18"/>
+      <c r="W129" s="18"/>
+      <c r="X129" s="18"/>
+      <c r="Y129" s="18"/>
+      <c r="Z129" s="18"/>
+      <c r="AA129" s="19"/>
+    </row>
+    <row r="130" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A130" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B130" s="23" t="s">
+        <v>229</v>
+      </c>
+      <c r="C130" s="23" t="s">
+        <v>230</v>
+      </c>
+      <c r="D130" s="23" t="s">
+        <v>232</v>
+      </c>
+      <c r="E130" s="23" t="s">
+        <v>233</v>
+      </c>
+      <c r="F130" s="23" t="s">
+        <v>234</v>
+      </c>
+      <c r="G130" s="23" t="s">
+        <v>235</v>
+      </c>
+      <c r="H130" s="23" t="s">
+        <v>236</v>
+      </c>
+      <c r="I130" s="23" t="s">
+        <v>237</v>
+      </c>
+      <c r="J130" s="23" t="s">
+        <v>238</v>
+      </c>
+      <c r="K130" s="23" t="s">
+        <v>239</v>
+      </c>
+      <c r="L130" s="23" t="s">
+        <v>240</v>
+      </c>
+      <c r="M130" s="23" t="s">
+        <v>241</v>
+      </c>
+      <c r="N130" s="23" t="s">
+        <v>242</v>
+      </c>
+      <c r="O130" s="23" t="s">
+        <v>243</v>
+      </c>
+      <c r="P130" s="23" t="s">
+        <v>244</v>
+      </c>
+      <c r="Q130" s="23" t="s">
+        <v>247</v>
+      </c>
+      <c r="R130" s="23" t="s">
+        <v>248</v>
+      </c>
+      <c r="S130" s="23" t="s">
+        <v>249</v>
+      </c>
+      <c r="T130" s="23" t="s">
+        <v>250</v>
+      </c>
+      <c r="U130" s="23" t="s">
+        <v>251</v>
+      </c>
+      <c r="V130" s="23" t="s">
+        <v>252</v>
+      </c>
+      <c r="W130" s="23" t="s">
+        <v>253</v>
+      </c>
+      <c r="X130" s="23" t="s">
+        <v>254</v>
+      </c>
+      <c r="Y130" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="Z130" s="23" t="s">
+        <v>256</v>
+      </c>
+      <c r="AA130" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="131" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A131" s="1">
+        <v>1</v>
+      </c>
+      <c r="B131" s="23">
+        <v>1</v>
+      </c>
+      <c r="C131" s="23">
+        <v>1</v>
+      </c>
+      <c r="D131" s="24">
+        <v>46058</v>
+      </c>
+      <c r="E131" s="24">
+        <v>46058</v>
+      </c>
+      <c r="F131" s="24">
+        <v>46063</v>
+      </c>
+      <c r="G131" s="23">
+        <v>1</v>
+      </c>
+      <c r="H131" s="23">
+        <v>5</v>
+      </c>
+      <c r="I131" s="23">
+        <v>2</v>
+      </c>
+      <c r="J131" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="K131" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="L131" s="23">
+        <v>1</v>
+      </c>
+      <c r="M131" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="N131" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="O131" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="P131" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="Q131" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="R131" s="23">
+        <v>1</v>
+      </c>
+      <c r="S131" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="T131" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="U131" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="V131" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="W131" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="X131" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="Y131" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="Z131" s="23">
+        <v>1</v>
+      </c>
+      <c r="AA131" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A132" s="1">
+        <v>2</v>
+      </c>
+      <c r="B132" s="23">
+        <v>2</v>
+      </c>
+      <c r="C132" s="23">
+        <v>1</v>
+      </c>
+      <c r="D132" s="24">
+        <v>46059</v>
+      </c>
+      <c r="E132" s="24">
+        <v>46059</v>
+      </c>
+      <c r="F132" s="24">
+        <v>46065</v>
+      </c>
+      <c r="G132" s="23">
+        <v>1</v>
+      </c>
+      <c r="H132" s="23">
+        <v>8</v>
+      </c>
+      <c r="I132" s="23">
+        <v>3</v>
+      </c>
+      <c r="J132" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="K132" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="L132" s="23">
+        <v>2</v>
+      </c>
+      <c r="M132" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="N132" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="O132" s="23" t="s">
+        <v>245</v>
+      </c>
+      <c r="P132" s="23">
+        <v>2</v>
+      </c>
+      <c r="Q132" s="23">
+        <v>1</v>
+      </c>
+      <c r="R132" s="23">
+        <v>1</v>
+      </c>
+      <c r="S132" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="T132" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="U132" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="V132" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="W132" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="X132" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="Y132" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="Z132" s="23">
+        <v>2</v>
+      </c>
+      <c r="AA132" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="133" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A133" s="3">
+        <v>3</v>
+      </c>
+      <c r="B133" s="4">
+        <v>3</v>
+      </c>
+      <c r="C133" s="4">
+        <v>2</v>
+      </c>
+      <c r="D133" s="16">
+        <v>46063</v>
+      </c>
+      <c r="E133" s="16">
+        <v>46063</v>
+      </c>
+      <c r="F133" s="16">
+        <v>46063</v>
+      </c>
+      <c r="G133" s="4">
+        <v>2</v>
+      </c>
+      <c r="H133" s="4">
+        <v>10</v>
+      </c>
+      <c r="I133" s="4">
+        <v>3</v>
+      </c>
+      <c r="J133" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="K133" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="L133" s="4">
+        <v>3</v>
+      </c>
+      <c r="M133" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="N133" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="O133" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="P133" s="4">
+        <v>1</v>
+      </c>
+      <c r="Q133" s="4">
+        <v>1</v>
+      </c>
+      <c r="R133" s="4">
+        <v>3</v>
+      </c>
+      <c r="S133" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="T133" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="U133" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="V133" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="W133" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="X133" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="Y133" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="Z133" s="4">
+        <v>3</v>
+      </c>
+      <c r="AA133" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="135" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="136" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A136" s="17" t="s">
+        <v>266</v>
+      </c>
+      <c r="B136" s="18"/>
+      <c r="C136" s="19"/>
+      <c r="E136" s="17" t="s">
+        <v>270</v>
+      </c>
+      <c r="F136" s="18"/>
+      <c r="G136" s="19"/>
+      <c r="I136" s="17" t="s">
+        <v>272</v>
+      </c>
+      <c r="J136" s="18"/>
+      <c r="K136" s="18"/>
+      <c r="L136" s="19"/>
+      <c r="N136" s="17" t="s">
+        <v>277</v>
+      </c>
+      <c r="O136" s="18"/>
+      <c r="P136" s="18"/>
+      <c r="Q136" s="18"/>
+      <c r="R136" s="19"/>
+    </row>
+    <row r="137" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A137" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B137" s="23" t="s">
+        <v>266</v>
+      </c>
+      <c r="C137" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E137" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F137" s="23" t="s">
+        <v>270</v>
+      </c>
+      <c r="G137" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="I137" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="J137" s="23" t="s">
+        <v>273</v>
+      </c>
+      <c r="K137" s="23" t="s">
+        <v>272</v>
+      </c>
+      <c r="L137" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="N137" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="O137" s="23" t="s">
+        <v>273</v>
+      </c>
+      <c r="P137" s="23" t="s">
+        <v>278</v>
+      </c>
+      <c r="Q137" s="23" t="s">
+        <v>279</v>
+      </c>
+      <c r="R137" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="138" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A138" s="1">
+        <v>1</v>
+      </c>
+      <c r="B138" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="C138" s="26" t="b">
+        <v>1</v>
+      </c>
+      <c r="E138" s="1">
+        <v>1</v>
+      </c>
+      <c r="F138" s="23" t="s">
+        <v>271</v>
+      </c>
+      <c r="G138" s="26" t="b">
+        <v>1</v>
+      </c>
+      <c r="I138" s="1">
+        <v>1</v>
+      </c>
+      <c r="J138" s="23">
+        <v>11</v>
+      </c>
+      <c r="K138" s="23" t="s">
+        <v>274</v>
+      </c>
+      <c r="L138" s="26" t="b">
+        <v>1</v>
+      </c>
+      <c r="N138" s="1">
+        <v>1</v>
+      </c>
+      <c r="O138" s="23">
+        <v>1</v>
+      </c>
+      <c r="P138" s="24">
+        <v>46058</v>
+      </c>
+      <c r="Q138" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="R138" s="26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="139" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A139" s="1">
+        <v>2</v>
+      </c>
+      <c r="B139" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="C139" s="27" t="b">
+        <v>1</v>
+      </c>
+      <c r="E139" s="1">
+        <v>2</v>
+      </c>
+      <c r="F139" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="G139" s="27" t="b">
+        <v>1</v>
+      </c>
+      <c r="I139" s="1">
+        <v>2</v>
+      </c>
+      <c r="J139" s="23">
+        <v>21</v>
+      </c>
+      <c r="K139" s="23" t="s">
+        <v>275</v>
+      </c>
+      <c r="L139" s="27" t="b">
+        <v>1</v>
+      </c>
+      <c r="N139" s="1">
+        <v>2</v>
+      </c>
+      <c r="O139" s="23">
+        <v>1</v>
+      </c>
+      <c r="P139" s="24">
+        <v>46059</v>
+      </c>
+      <c r="Q139" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="R139" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="140" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A140" s="3">
+        <v>3</v>
+      </c>
+      <c r="B140" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="C140" s="28" t="b">
+        <v>1</v>
+      </c>
+      <c r="E140" s="3">
+        <v>3</v>
+      </c>
+      <c r="F140" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="G140" s="28" t="b">
+        <v>1</v>
+      </c>
+      <c r="I140" s="3">
+        <v>3</v>
+      </c>
+      <c r="J140" s="4">
+        <v>31</v>
+      </c>
+      <c r="K140" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="L140" s="28" t="b">
+        <v>1</v>
+      </c>
+      <c r="N140" s="3">
+        <v>3</v>
+      </c>
+      <c r="O140" s="4">
+        <v>1</v>
+      </c>
+      <c r="P140" s="16">
+        <v>46063</v>
+      </c>
+      <c r="Q140" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="R140" s="28" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="29">
-    <mergeCell ref="A115:K115"/>
+  <mergeCells count="37">
+    <mergeCell ref="A129:AA129"/>
+    <mergeCell ref="H122:J122"/>
+    <mergeCell ref="L122:N122"/>
+    <mergeCell ref="A136:C136"/>
+    <mergeCell ref="E136:G136"/>
+    <mergeCell ref="I136:L136"/>
+    <mergeCell ref="N136:R136"/>
+    <mergeCell ref="M26:P26"/>
     <mergeCell ref="A122:F122"/>
     <mergeCell ref="A108:E108"/>
     <mergeCell ref="A94:N94"/>
@@ -4876,6 +6006,18 @@
     <mergeCell ref="A87:B87"/>
     <mergeCell ref="D87:F87"/>
     <mergeCell ref="H87:L87"/>
+    <mergeCell ref="A115:N115"/>
+    <mergeCell ref="F47:M47"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="A54:I54"/>
+    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="H40:M40"/>
+    <mergeCell ref="I5:K5"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="F19:L19"/>
+    <mergeCell ref="G12:K12"/>
+    <mergeCell ref="I26:K26"/>
     <mergeCell ref="A61:E61"/>
     <mergeCell ref="G61:K61"/>
     <mergeCell ref="A68:E68"/>
@@ -4885,23 +6027,12 @@
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="A33:I33"/>
     <mergeCell ref="K33:N33"/>
-    <mergeCell ref="A47:D47"/>
-    <mergeCell ref="I26:K26"/>
-    <mergeCell ref="F47:L47"/>
-    <mergeCell ref="A54:I54"/>
-    <mergeCell ref="A40:F40"/>
-    <mergeCell ref="H40:M40"/>
-    <mergeCell ref="I5:K5"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A26:G26"/>
-    <mergeCell ref="F19:L19"/>
-    <mergeCell ref="G12:K12"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
-  <tableParts count="29">
+  <tableParts count="37">
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
     <tablePart r:id="rId5"/>
@@ -4931,6 +6062,23 @@
     <tablePart r:id="rId29"/>
     <tablePart r:id="rId30"/>
     <tablePart r:id="rId31"/>
+    <tablePart r:id="rId32"/>
+    <tablePart r:id="rId33"/>
+    <tablePart r:id="rId34"/>
+    <tablePart r:id="rId35"/>
+    <tablePart r:id="rId36"/>
+    <tablePart r:id="rId37"/>
+    <tablePart r:id="rId38"/>
+    <tablePart r:id="rId39"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3088F35-A355-471A-8471-9A564A7FDE13}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Armado de DER y de la base de datos
</commit_message>
<xml_diff>
--- a/BBDD.xlsx
+++ b/BBDD.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyectos\Web_Andez\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F396AEE-830D-45C7-BF5C-F510F77D9436}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97FE8534-FBB5-4CDD-B326-E67CA819E0EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5D42B345-DB14-48C1-9A38-23908D3120ED}"/>
   </bookViews>
@@ -119,7 +119,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="295">
   <si>
     <t>Color</t>
   </si>
@@ -968,6 +968,42 @@
   </si>
   <si>
     <t>Centro</t>
+  </si>
+  <si>
+    <t>Permisos</t>
+  </si>
+  <si>
+    <t>NombrePermisos</t>
+  </si>
+  <si>
+    <t>Marketing Lineas</t>
+  </si>
+  <si>
+    <t>Postventa Dashboard</t>
+  </si>
+  <si>
+    <t>Marketing Catalogo</t>
+  </si>
+  <si>
+    <t>RolPermisos</t>
+  </si>
+  <si>
+    <t>IdRol</t>
+  </si>
+  <si>
+    <t>IdPermiso</t>
+  </si>
+  <si>
+    <t>TipoSubtipo</t>
+  </si>
+  <si>
+    <t>IdTipo</t>
+  </si>
+  <si>
+    <t>IdSubtipo</t>
+  </si>
+  <si>
+    <t>IDCaso</t>
   </si>
 </sst>
 </file>
@@ -1134,7 +1170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -1152,6 +1188,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1171,22 +1208,57 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="62">
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+  <dxfs count="67">
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <fill>
@@ -1546,6 +1618,12 @@
       </fill>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1726,7 +1804,7 @@
   <autoFilter ref="A13:E16" xr:uid="{D96833EF-4E6F-4FA0-A7A0-6E6817E2B38A}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{317907DD-843B-4FA4-8837-A0A78A4A0507}" name="ID"/>
-    <tableColumn id="5" xr3:uid="{E0921BEC-D870-4C51-B3FC-23E013804DC3}" name="CodigoColor" dataDxfId="61"/>
+    <tableColumn id="5" xr3:uid="{E0921BEC-D870-4C51-B3FC-23E013804DC3}" name="CodigoColor" dataDxfId="66"/>
     <tableColumn id="2" xr3:uid="{8053C3DC-ACA4-4AAB-9AFB-34FBDDEBC52B}" name="NombreColor"/>
     <tableColumn id="4" xr3:uid="{1D3A10F0-E8C4-471A-B4A8-2001816AFFF2}" name="URLColor"/>
     <tableColumn id="3" xr3:uid="{D04813E9-6E48-439B-A711-735DEB41533C}" name="Activo"/>
@@ -1759,8 +1837,8 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{C6605137-9E60-4417-BE9D-22DF41FEA57D}" name="ID"/>
     <tableColumn id="2" xr3:uid="{D82CDF84-BD14-4C63-ABBA-8F2236A9C0E4}" name="Pais"/>
-    <tableColumn id="3" xr3:uid="{FA78D055-E341-4362-A23A-0CCFC591E8FA}" name="Latitud" dataDxfId="58"/>
-    <tableColumn id="4" xr3:uid="{36EB177E-ACE1-4B78-A56A-A9F891312B25}" name="Longitud" dataDxfId="57"/>
+    <tableColumn id="3" xr3:uid="{FA78D055-E341-4362-A23A-0CCFC591E8FA}" name="Latitud" dataDxfId="63"/>
+    <tableColumn id="4" xr3:uid="{36EB177E-ACE1-4B78-A56A-A9F891312B25}" name="Longitud" dataDxfId="62"/>
     <tableColumn id="5" xr3:uid="{4122267C-292B-476B-8AB1-41CBE8A90AAF}" name="Zoom"/>
     <tableColumn id="7" xr3:uid="{0270C110-04E9-4179-AF06-958CA4E37E9B}" name="Activo"/>
   </tableColumns>
@@ -1769,15 +1847,15 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{EF32F6B3-AC45-462F-BE18-EFE2DD57FE9B}" name="Tabla17" displayName="Tabla17" ref="H41:M44" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{EF32F6B3-AC45-462F-BE18-EFE2DD57FE9B}" name="Tabla17" displayName="Tabla17" ref="H41:M44" totalsRowShown="0" headerRowDxfId="61" dataDxfId="60">
   <autoFilter ref="H41:M44" xr:uid="{EF32F6B3-AC45-462F-BE18-EFE2DD57FE9B}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{C8F6ED57-5FD2-4FB3-A4A5-BC3965E98B15}" name="ID" dataDxfId="54"/>
-    <tableColumn id="2" xr3:uid="{65B99387-EDCD-429B-B81B-A4F58479A304}" name="IdProducto" dataDxfId="53"/>
-    <tableColumn id="3" xr3:uid="{5D9C0348-2DF4-47CC-977C-AAFB9F19E959}" name="Titulo" dataDxfId="52"/>
-    <tableColumn id="4" xr3:uid="{1CACB54F-DC9D-41AC-A04F-171EF34060DC}" name="URLImagen" dataDxfId="51"/>
+    <tableColumn id="1" xr3:uid="{C8F6ED57-5FD2-4FB3-A4A5-BC3965E98B15}" name="ID" dataDxfId="59"/>
+    <tableColumn id="2" xr3:uid="{65B99387-EDCD-429B-B81B-A4F58479A304}" name="IdProducto" dataDxfId="58"/>
+    <tableColumn id="3" xr3:uid="{5D9C0348-2DF4-47CC-977C-AAFB9F19E959}" name="Titulo" dataDxfId="57"/>
+    <tableColumn id="4" xr3:uid="{1CACB54F-DC9D-41AC-A04F-171EF34060DC}" name="URLImagen" dataDxfId="56"/>
     <tableColumn id="5" xr3:uid="{E836C9A1-0FCD-4424-8667-FBB476A992FD}" name="Publicada"/>
-    <tableColumn id="7" xr3:uid="{824500A6-D872-42FD-9C38-60CB54869E2F}" name="Activo" dataDxfId="50"/>
+    <tableColumn id="7" xr3:uid="{824500A6-D872-42FD-9C38-60CB54869E2F}" name="Activo" dataDxfId="55"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1805,8 +1883,8 @@
     <tableColumn id="3" xr3:uid="{650899D4-4E19-437F-9FCF-B4D26F2AA0DB}" name="Direccion"/>
     <tableColumn id="4" xr3:uid="{1E07E83B-09DC-40FD-907E-40F4CBC0A570}" name="IdProvincia"/>
     <tableColumn id="5" xr3:uid="{6138418F-A367-4A68-8F05-2638E82A22BC}" name="Telefono"/>
-    <tableColumn id="6" xr3:uid="{80260CDA-43B3-49C5-B2E8-6D4D4EE4367B}" name="Latitud" dataDxfId="49"/>
-    <tableColumn id="7" xr3:uid="{D1025C6A-57D3-4E57-916D-CF79774C6EAF}" name="Longitud" dataDxfId="48"/>
+    <tableColumn id="6" xr3:uid="{80260CDA-43B3-49C5-B2E8-6D4D4EE4367B}" name="Latitud" dataDxfId="54"/>
+    <tableColumn id="7" xr3:uid="{D1025C6A-57D3-4E57-916D-CF79774C6EAF}" name="Longitud" dataDxfId="53"/>
     <tableColumn id="8" xr3:uid="{FACFCBBE-C8C5-4011-911D-7F4D64577C47}" name="IdPagina"/>
     <tableColumn id="9" xr3:uid="{3EE8280A-E1AE-43CB-8AA3-681D1032743D}" name="Activo"/>
   </tableColumns>
@@ -1815,13 +1893,13 @@
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{B6BCDECB-3201-4C98-AA8D-79812894A18B}" name="Tabla19" displayName="Tabla19" ref="K34:N37" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{B6BCDECB-3201-4C98-AA8D-79812894A18B}" name="Tabla19" displayName="Tabla19" ref="K34:N37" totalsRowShown="0" headerRowDxfId="52" dataDxfId="51">
   <autoFilter ref="K34:N37" xr:uid="{36798AE9-B843-4477-9F23-32045BDEF7D7}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{E050CEA3-2793-4698-9E45-C3447ADCD555}" name="ID" dataDxfId="45"/>
-    <tableColumn id="2" xr3:uid="{03295AE7-34B5-4134-9D2F-2268D15B310C}" name="IDProducto" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{1564E106-D50F-4573-A696-EE197325F0F3}" name="IDAtributo" dataDxfId="43"/>
-    <tableColumn id="4" xr3:uid="{5F701778-C720-415C-9979-8380EB9AB80C}" name="Activo" dataDxfId="42"/>
+    <tableColumn id="1" xr3:uid="{E050CEA3-2793-4698-9E45-C3447ADCD555}" name="ID" dataDxfId="50"/>
+    <tableColumn id="2" xr3:uid="{03295AE7-34B5-4134-9D2F-2268D15B310C}" name="IDProducto" dataDxfId="49"/>
+    <tableColumn id="3" xr3:uid="{1564E106-D50F-4573-A696-EE197325F0F3}" name="IDAtributo" dataDxfId="48"/>
+    <tableColumn id="4" xr3:uid="{5F701778-C720-415C-9979-8380EB9AB80C}" name="Activo" dataDxfId="47"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1834,8 +1912,8 @@
     <tableColumn id="1" xr3:uid="{76441B91-C9F3-418E-9F7A-2145EC66A51B}" name="ID"/>
     <tableColumn id="2" xr3:uid="{B7D7EADF-0604-4B90-A7CA-6537AE39152D}" name="Pronvincia"/>
     <tableColumn id="3" xr3:uid="{FBCCEEC7-DBEE-4480-8CBE-1F5805CA9202}" name="IdPais"/>
-    <tableColumn id="4" xr3:uid="{0A3D75EA-6C18-48E0-9489-C5D19B3AC70A}" name="Latitud" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{ACBD9873-D350-427F-993B-2B1B42296D9B}" name="Longitud" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{0A3D75EA-6C18-48E0-9489-C5D19B3AC70A}" name="Latitud" dataDxfId="46"/>
+    <tableColumn id="5" xr3:uid="{ACBD9873-D350-427F-993B-2B1B42296D9B}" name="Longitud" dataDxfId="45"/>
     <tableColumn id="6" xr3:uid="{957CA68C-6225-4C37-B8D5-8FF8C064FB1C}" name="Zoom"/>
     <tableColumn id="8" xr3:uid="{33319F29-BC62-4963-B0AA-34AC0E216488}" name="Zona"/>
     <tableColumn id="7" xr3:uid="{D19F9B22-3CC1-4E0E-B3DB-56D9B346F0CD}" name="Activo"/>
@@ -1845,46 +1923,46 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{D66B8F6B-A06F-42EB-B1CE-F5AC470DCC17}" name="Tabla20" displayName="Tabla20" ref="A62:E65" totalsRowShown="0" headerRowDxfId="41" dataDxfId="40">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{D66B8F6B-A06F-42EB-B1CE-F5AC470DCC17}" name="Tabla20" displayName="Tabla20" ref="A62:E65" totalsRowShown="0" headerRowDxfId="44" dataDxfId="43">
   <autoFilter ref="A62:E65" xr:uid="{6995137C-E78D-4F26-A126-F3AEFE2A2B13}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{7C1F763D-9A29-4F91-BB26-5F2CF68260F0}" name="ID" dataDxfId="39"/>
-    <tableColumn id="5" xr3:uid="{F0BF2187-ECA7-4173-9FAC-3BC72EFDB82F}" name="IdEmpresa" dataDxfId="38"/>
-    <tableColumn id="2" xr3:uid="{98E75056-4A9A-4C56-8FA5-EFD4D867777B}" name="Nombre" dataDxfId="37"/>
-    <tableColumn id="3" xr3:uid="{48A2AE2B-7A42-420C-8BB3-5F9F2AA01721}" name="Mail" dataDxfId="36">
+    <tableColumn id="1" xr3:uid="{7C1F763D-9A29-4F91-BB26-5F2CF68260F0}" name="ID" dataDxfId="42"/>
+    <tableColumn id="5" xr3:uid="{F0BF2187-ECA7-4173-9FAC-3BC72EFDB82F}" name="IdEmpresa" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{98E75056-4A9A-4C56-8FA5-EFD4D867777B}" name="Nombre" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{48A2AE2B-7A42-420C-8BB3-5F9F2AA01721}" name="Mail" dataDxfId="39">
       <calculatedColumnFormula>CONCATENATE(C63,"@andez.com.ar")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{31D99612-66DC-4B54-A747-6C39765D7B66}" name="Activo" dataDxfId="35"/>
+    <tableColumn id="4" xr3:uid="{31D99612-66DC-4B54-A747-6C39765D7B66}" name="Activo" dataDxfId="38"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{2B2EAABA-4403-411A-98F0-A8284D43302C}" name="Tabla2021" displayName="Tabla2021" ref="G62:K65" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{2B2EAABA-4403-411A-98F0-A8284D43302C}" name="Tabla2021" displayName="Tabla2021" ref="G62:K65" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
   <autoFilter ref="G62:K65" xr:uid="{89087EED-CE2D-441A-9746-B0BA56EA9A63}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{6D3F8F4E-2473-4BE6-A51E-C3C3E4C26133}" name="ID" dataDxfId="32"/>
-    <tableColumn id="5" xr3:uid="{8C181956-53C7-4FD2-BAAB-42B1CDE2E84E}" name="IdEmpresa" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{12B007DF-889A-4CDB-93CC-EBEFCBD3A3E9}" name="Nombre" dataDxfId="30"/>
-    <tableColumn id="3" xr3:uid="{A94B5F86-8442-44DD-9C03-77F51D7F5B8D}" name="Telefono" dataDxfId="29">
+    <tableColumn id="1" xr3:uid="{6D3F8F4E-2473-4BE6-A51E-C3C3E4C26133}" name="ID" dataDxfId="35"/>
+    <tableColumn id="5" xr3:uid="{8C181956-53C7-4FD2-BAAB-42B1CDE2E84E}" name="IdEmpresa" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{12B007DF-889A-4CDB-93CC-EBEFCBD3A3E9}" name="Nombre" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{A94B5F86-8442-44DD-9C03-77F51D7F5B8D}" name="Telefono" dataDxfId="32">
       <calculatedColumnFormula>CONCATENATE(I63,"@andez.com.ar")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{0E412ADD-9FF3-43E1-BDA1-A917D6B1E4D7}" name="Activo" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{0E412ADD-9FF3-43E1-BDA1-A917D6B1E4D7}" name="Activo" dataDxfId="31"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{8F3FF2B6-156D-475C-B60E-2BBAE1F181CE}" name="Tabla21" displayName="Tabla21" ref="A69:E72" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26" tableBorderDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{8F3FF2B6-156D-475C-B60E-2BBAE1F181CE}" name="Tabla21" displayName="Tabla21" ref="A69:E72" totalsRowShown="0" headerRowDxfId="30" dataDxfId="29" tableBorderDxfId="28">
   <autoFilter ref="A69:E72" xr:uid="{58000D4A-AEBA-4D49-B463-180C8FD8A937}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{E9F2D081-00F6-4B92-9DFE-6473CB6B3F38}" name="ID" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{FE107DC5-A1C2-4F54-BC82-5BBB32CCABC3}" name="IdEmpresa" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{DE65DD1F-F1BA-4548-A19A-4B9DD2857A6F}" name="Red" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{23F951D4-E519-45F7-81C5-69ED4EA385E4}" name="URLRed" dataDxfId="21"/>
-    <tableColumn id="4" xr3:uid="{E5F1016C-C8F1-4FEA-B687-B57CB00F2E70}" name="Activo" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{E9F2D081-00F6-4B92-9DFE-6473CB6B3F38}" name="ID" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{FE107DC5-A1C2-4F54-BC82-5BBB32CCABC3}" name="IdEmpresa" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{DE65DD1F-F1BA-4548-A19A-4B9DD2857A6F}" name="Red" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{23F951D4-E519-45F7-81C5-69ED4EA385E4}" name="URLRed" dataDxfId="24"/>
+    <tableColumn id="4" xr3:uid="{E5F1016C-C8F1-4FEA-B687-B57CB00F2E70}" name="Activo" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1905,19 +1983,19 @@
 </file>
 
 <file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{C769ADF8-2405-479D-8112-7564F0940768}" name="Tabla22" displayName="Tabla22" ref="A76:J77" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{C769ADF8-2405-479D-8112-7564F0940768}" name="Tabla22" displayName="Tabla22" ref="A76:J77" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
   <autoFilter ref="A76:J77" xr:uid="{A2E83C68-75BA-4C98-B80E-E4E7E2B0B82C}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{173EAAD2-F12F-4372-8FA2-00B32059C1EB}" name="ID" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{3E7AAA46-3847-4587-A43F-E688C1582045}" name="RazonSocial" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{7727AE8E-759C-4DE1-86AE-BDFED86835D0}" name="CUIT" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{BBA783BB-BBBB-4233-929D-4BF68AFA091A}" name="Direccion" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{419A73DC-BE03-4D90-BE0C-9779F3EB2DDB}" name="Localidad" dataDxfId="13"/>
-    <tableColumn id="7" xr3:uid="{BE8C959F-F07F-4076-8E57-3EA25221B957}" name="Partido" dataDxfId="12"/>
-    <tableColumn id="8" xr3:uid="{DB60E2FA-C8A3-4C27-BCAB-41F7E5C99855}" name="IdProvincia" dataDxfId="11"/>
-    <tableColumn id="9" xr3:uid="{EC23197E-97BD-4D2B-AF77-BAEDEAEEEB33}" name="CP" dataDxfId="10"/>
-    <tableColumn id="10" xr3:uid="{7234FBEF-54AA-4FBE-8D11-84EDF024DAB3}" name="Horario" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{2D33166C-2999-4BC9-8B00-7F06B4D84FF1}" name="Activo" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{173EAAD2-F12F-4372-8FA2-00B32059C1EB}" name="ID" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{3E7AAA46-3847-4587-A43F-E688C1582045}" name="RazonSocial" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{7727AE8E-759C-4DE1-86AE-BDFED86835D0}" name="CUIT" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{BBA783BB-BBBB-4233-929D-4BF68AFA091A}" name="Direccion" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{419A73DC-BE03-4D90-BE0C-9779F3EB2DDB}" name="Localidad" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{BE8C959F-F07F-4076-8E57-3EA25221B957}" name="Partido" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{DB60E2FA-C8A3-4C27-BCAB-41F7E5C99855}" name="IdProvincia" dataDxfId="14"/>
+    <tableColumn id="9" xr3:uid="{EC23197E-97BD-4D2B-AF77-BAEDEAEEEB33}" name="CP" dataDxfId="13"/>
+    <tableColumn id="10" xr3:uid="{7234FBEF-54AA-4FBE-8D11-84EDF024DAB3}" name="Horario" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{2D33166C-2999-4BC9-8B00-7F06B4D84FF1}" name="Activo" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1933,7 +2011,7 @@
     <tableColumn id="3" xr3:uid="{473E571D-8BE9-4BD5-B8BD-FC16062FBA4A}" name="Nombre"/>
     <tableColumn id="4" xr3:uid="{BFCDC025-7291-43F4-BF51-02B5C205C0B1}" name="URLImagen"/>
     <tableColumn id="5" xr3:uid="{1AD6DCB5-B8FB-43FC-88CE-E58B0DF75376}" name="Titulo"/>
-    <tableColumn id="6" xr3:uid="{782D732A-1C91-4938-BDF6-8C352984694E}" name="Descripcion" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{782D732A-1C91-4938-BDF6-8C352984694E}" name="Descripcion" dataDxfId="10"/>
     <tableColumn id="7" xr3:uid="{37200F4F-B540-4A63-9F27-255BD55AD0BD}" name="Link"/>
     <tableColumn id="8" xr3:uid="{CB7E851F-8679-4467-A629-18DE76D9185B}" name="LinkSN"/>
     <tableColumn id="9" xr3:uid="{DF01FB7D-3582-4808-83E6-C0BF4EDCA881}" name="LanzamientoSN"/>
@@ -2040,7 +2118,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="28" xr:uid="{E5C72C39-AEF7-4120-A1E5-FF7EB5A3BF17}" name="Tabla28" displayName="Tabla28" ref="A116:N119" totalsRowShown="0">
   <autoFilter ref="A116:N119" xr:uid="{E5C72C39-AEF7-4120-A1E5-FF7EB5A3BF17}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{68690C7C-4428-4270-97EF-F62ECCF7314E}" name="ID"/>
+    <tableColumn id="1" xr3:uid="{68690C7C-4428-4270-97EF-F62ECCF7314E}" name="IDCaso"/>
     <tableColumn id="2" xr3:uid="{4ED8A294-C798-4D37-9F33-B2D6E944F3F4}" name="NombreApellido"/>
     <tableColumn id="3" xr3:uid="{58ED13BD-9B17-4772-85AE-6842EAEE71E5}" name="Mail"/>
     <tableColumn id="4" xr3:uid="{94F35AE4-BB92-4E59-9201-C44956F3D992}" name="Telefono"/>
@@ -2107,13 +2185,13 @@
     <tableColumn id="2" xr3:uid="{89511843-4E67-4DCC-9385-A72CA58CD9DF}" name="IdCliente"/>
     <tableColumn id="3" xr3:uid="{AC688752-919C-4DEB-88C2-DF2E8EF3BD63}" name="IdFormaContacto"/>
     <tableColumn id="4" xr3:uid="{7D3ED9E7-75FB-4DF7-91B5-E392871B8D43}" name="Fecha1erContacto"/>
-    <tableColumn id="13" xr3:uid="{9EA8476D-DBBE-471F-BFC8-6A291BA80F62}" name="Fecha1eraRespuesta" dataDxfId="6"/>
+    <tableColumn id="13" xr3:uid="{9EA8476D-DBBE-471F-BFC8-6A291BA80F62}" name="Fecha1eraRespuesta" dataDxfId="9"/>
     <tableColumn id="5" xr3:uid="{DBAD1119-0F40-4BD3-9842-1192A64CBD53}" name="FechaCierre"/>
     <tableColumn id="14" xr3:uid="{E39840EE-9AE9-4080-8CE2-7FB8A7484DCE}" name="IdMotivoContacto"/>
     <tableColumn id="6" xr3:uid="{3E40D0DD-319F-4EE0-B63A-0C3A0E154C0B}" name="IdCodigoReclamo"/>
     <tableColumn id="7" xr3:uid="{4B7DE31B-73B8-4D00-834D-2635643BB279}" name="IdEstadoReclamo"/>
-    <tableColumn id="8" xr3:uid="{FE3B8DB4-2255-4BFC-9B37-C7BFF06B57C5}" name="Consulta" dataDxfId="5"/>
-    <tableColumn id="12" xr3:uid="{55F91CC0-9D26-4D31-B57A-EA6D64ADC6F2}" name="Solucion" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{FE3B8DB4-2255-4BFC-9B37-C7BFF06B57C5}" name="Consulta" dataDxfId="8"/>
+    <tableColumn id="12" xr3:uid="{55F91CC0-9D26-4D31-B57A-EA6D64ADC6F2}" name="Solucion" dataDxfId="7"/>
     <tableColumn id="9" xr3:uid="{617CB8EC-F821-47DB-8753-32FB1A107F1A}" name="IdDatosCompra"/>
     <tableColumn id="10" xr3:uid="{6329DF96-E0FA-4B62-9E86-F32620647183}" name="FechaOT"/>
     <tableColumn id="19" xr3:uid="{8C8B6D30-6532-40D3-AE91-9F85D048000E}" name="NumeroOT"/>
@@ -2202,9 +2280,33 @@
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{5560DF7C-FEE5-456B-92EA-203150657B26}" name="ID"/>
     <tableColumn id="2" xr3:uid="{1F149BD5-C727-437F-8393-C5987FBE588D}" name="CodigoMotivo"/>
-    <tableColumn id="4" xr3:uid="{8CFC6924-9C12-4FBB-9472-05F51F199A0A}" name="Fecha" dataDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{47C9DE2B-FED3-499A-92E4-96789BCD9F70}" name="Registro" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{8CFC6924-9C12-4FBB-9472-05F51F199A0A}" name="Fecha" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{47C9DE2B-FED3-499A-92E4-96789BCD9F70}" name="Registro" dataDxfId="5"/>
     <tableColumn id="3" xr3:uid="{03ADB1E3-143F-49CF-A27C-B2C1272966DD}" name="Activo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table38.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="38" xr:uid="{9EA5CA6A-CBAC-4676-9694-77DA98FB682B}" name="Tabla131139" displayName="Tabla131139" ref="M6:O9" totalsRowShown="0">
+  <autoFilter ref="M6:O9" xr:uid="{9EA5CA6A-CBAC-4676-9694-77DA98FB682B}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{51A4A014-16C2-42A7-B0AD-C7F058304A65}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{A71AA2BD-8D54-4D80-BFE6-8E66C62F1ECF}" name="NombrePermisos"/>
+    <tableColumn id="3" xr3:uid="{0D945ED6-1A5B-44A0-8EF1-C78FCB2E3EEB}" name="Activo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table39.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="39" xr:uid="{7D63C190-E1F5-4D37-BFDB-ED191FD282B0}" name="Tabla13113940" displayName="Tabla13113940" ref="Q6:S9" totalsRowShown="0">
+  <autoFilter ref="Q6:S9" xr:uid="{7D63C190-E1F5-4D37-BFDB-ED191FD282B0}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{5FC7BA14-7773-4DE3-A8E9-1332A4F73D91}" name="IdRol"/>
+    <tableColumn id="2" xr3:uid="{9CB85A1D-7FAA-41E9-B549-D07CE038F630}" name="IdPermiso"/>
+    <tableColumn id="3" xr3:uid="{E39C9128-25EA-4C6C-8F11-E791592D285C}" name="Activo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2223,6 +2325,18 @@
 </table>
 </file>
 
+<file path=xl/tables/table40.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="41" xr:uid="{E9CEDBD9-A9D4-416A-8C1F-145F45E58235}" name="Tabla41" displayName="Tabla41" ref="M27:O30" totalsRowShown="0">
+  <autoFilter ref="M27:O30" xr:uid="{E9CEDBD9-A9D4-416A-8C1F-145F45E58235}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{99819716-917A-4FCD-8CE5-0D5097287F00}" name="IdTipo"/>
+    <tableColumn id="2" xr3:uid="{F5C6F011-5340-48E5-85E8-2F9DDA0B9C94}" name="IdSubtipo"/>
+    <tableColumn id="3" xr3:uid="{1AB7F8AD-7F56-43C2-93DD-941FD95EF17C}" name="Activo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{917C16AE-1BA5-492E-ADA8-1AF74DE3B1D8}" name="Tabla6" displayName="Tabla6" ref="F20:L23" totalsRowShown="0">
   <autoFilter ref="F20:L23" xr:uid="{917C16AE-1BA5-492E-ADA8-1AF74DE3B1D8}"/>
@@ -2233,7 +2347,7 @@
     <tableColumn id="4" xr3:uid="{33CF0639-7E0E-4323-ABAC-57E9E79BAC94}" name="URLManual"/>
     <tableColumn id="6" xr3:uid="{8FB3C041-5F4E-4C6B-BFEA-F7EF8CCA380F}" name="URLRepuestos"/>
     <tableColumn id="7" xr3:uid="{19883A37-D7EF-411E-B5D4-0F9C58EA4DF5}" name="URLPlanos"/>
-    <tableColumn id="5" xr3:uid="{9FBFC04D-E638-4A8E-BF60-60BF85B463B6}" name="Activo" dataDxfId="60"/>
+    <tableColumn id="5" xr3:uid="{9FBFC04D-E638-4A8E-BF60-60BF85B463B6}" name="Activo" dataDxfId="65"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2260,7 +2374,7 @@
   <autoFilter ref="A6:G9" xr:uid="{00F67F5D-77F7-41B7-A265-5E336044A6C5}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{F32EBD58-4145-475F-A8DD-60533C773560}" name="ID"/>
-    <tableColumn id="5" xr3:uid="{BA938A3C-223C-48BE-9D99-D519D9B88EDF}" name="Nombre" dataDxfId="59"/>
+    <tableColumn id="5" xr3:uid="{BA938A3C-223C-48BE-9D99-D519D9B88EDF}" name="Nombre" dataDxfId="64"/>
     <tableColumn id="2" xr3:uid="{BF58FE61-5919-4F9C-BC69-7F6F4B0BCCB1}" name="Apellido"/>
     <tableColumn id="4" xr3:uid="{B217BF12-7466-47C6-83EC-0600B0F7EE4B}" name="Mail">
       <calculatedColumnFormula>CONCATENATE(Tabla15[[#This Row],[Nombre]],Tabla15[[#This Row],[Apellido]],"@andez.com.ar")</calculatedColumnFormula>
@@ -2286,13 +2400,12 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{F6B3327E-5FDA-4BB7-AACF-FABE81E48666}" name="Tabla11" displayName="Tabla11" ref="M27:P30" totalsRowShown="0">
-  <autoFilter ref="M27:P30" xr:uid="{F6B3327E-5FDA-4BB7-AACF-FABE81E48666}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{26F76265-568B-4A28-AA28-6DA1CF7F5397}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{A81F65B5-D9C2-4F7A-9651-B297627921BE}" name="Tipo"/>
-    <tableColumn id="4" xr3:uid="{DAB68CD9-3919-4F19-B6D2-6F30B1F19B70}" name="Subtipo"/>
-    <tableColumn id="3" xr3:uid="{6BF61F58-B964-4C51-B2A6-1D6E99603A94}" name="Activo"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{F6B3327E-5FDA-4BB7-AACF-FABE81E48666}" name="Tabla11" displayName="Tabla11" ref="Q27:S30" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+  <autoFilter ref="Q27:S30" xr:uid="{F6B3327E-5FDA-4BB7-AACF-FABE81E48666}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{26F76265-568B-4A28-AA28-6DA1CF7F5397}" name="ID" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{DAB68CD9-3919-4F19-B6D2-6F30B1F19B70}" name="Subtipo" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{6BF61F58-B964-4C51-B2A6-1D6E99603A94}" name="Activo" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2618,7 +2731,7 @@
   <dimension ref="A1:AA140"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.21875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.21875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="28.77734375" bestFit="1" customWidth="1"/>
@@ -2626,12 +2739,12 @@
     <col min="6" max="6" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="24.88671875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.33203125" customWidth="1"/>
     <col min="10" max="10" width="31.44140625" customWidth="1"/>
     <col min="11" max="11" width="24.88671875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="18" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.6640625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="16.109375" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11.77734375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="24.88671875" bestFit="1" customWidth="1"/>
@@ -2647,7 +2760,7 @@
     <col min="27" max="27" width="11.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
       <c r="B1" s="11" t="s">
         <v>105</v>
       </c>
@@ -2658,24 +2771,34 @@
         <v>107</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A5" s="20" t="s">
+    <row r="4" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A5" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="21"/>
-      <c r="C5" s="21"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21"/>
-      <c r="G5" s="22"/>
-      <c r="I5" s="20" t="s">
+      <c r="B5" s="22"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="23"/>
+      <c r="I5" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="J5" s="21"/>
-      <c r="K5" s="22"/>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="J5" s="22"/>
+      <c r="K5" s="23"/>
+      <c r="M5" s="21" t="s">
+        <v>283</v>
+      </c>
+      <c r="N5" s="22"/>
+      <c r="O5" s="23"/>
+      <c r="Q5" s="21" t="s">
+        <v>288</v>
+      </c>
+      <c r="R5" s="22"/>
+      <c r="S5" s="23"/>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
@@ -2706,8 +2829,26 @@
       <c r="K6" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="M6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="N6" t="s">
+        <v>284</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q6" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="R6" t="s">
+        <v>290</v>
+      </c>
+      <c r="S6" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>1</v>
       </c>
@@ -2739,8 +2880,26 @@
       <c r="K7" s="2" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="M7" s="1">
+        <v>1</v>
+      </c>
+      <c r="N7" t="s">
+        <v>285</v>
+      </c>
+      <c r="O7" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="1">
+        <v>1</v>
+      </c>
+      <c r="R7">
+        <v>1</v>
+      </c>
+      <c r="S7" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>2</v>
       </c>
@@ -2772,8 +2931,26 @@
       <c r="K8" s="2" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="M8" s="1">
+        <v>2</v>
+      </c>
+      <c r="N8" t="s">
+        <v>286</v>
+      </c>
+      <c r="O8" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="1">
+        <v>2</v>
+      </c>
+      <c r="R8">
+        <v>2</v>
+      </c>
+      <c r="S8" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>3</v>
       </c>
@@ -2805,31 +2982,49 @@
       <c r="K9" s="5" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A12" s="17" t="s">
+      <c r="M9" s="3">
+        <v>3</v>
+      </c>
+      <c r="N9" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="O9" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q9" s="3">
+        <v>3</v>
+      </c>
+      <c r="R9" s="4">
+        <v>3</v>
+      </c>
+      <c r="S9" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A12" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B12" s="18"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="19"/>
-      <c r="G12" s="17" t="s">
+      <c r="B12" s="19"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="20"/>
+      <c r="G12" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="H12" s="18"/>
-      <c r="I12" s="18"/>
-      <c r="J12" s="18"/>
-      <c r="K12" s="19"/>
-      <c r="M12" s="17" t="s">
+      <c r="H12" s="19"/>
+      <c r="I12" s="19"/>
+      <c r="J12" s="19"/>
+      <c r="K12" s="20"/>
+      <c r="M12" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="N12" s="18"/>
-      <c r="O12" s="18"/>
-      <c r="P12" s="19"/>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="N12" s="19"/>
+      <c r="O12" s="19"/>
+      <c r="P12" s="20"/>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>1</v>
       </c>
@@ -2873,7 +3068,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>1</v>
       </c>
@@ -2917,7 +3112,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>2</v>
       </c>
@@ -2961,7 +3156,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
         <v>3</v>
       </c>
@@ -3005,25 +3200,25 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A19" s="17" t="s">
+    <row r="18" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A19" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="18"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="19"/>
-      <c r="F19" s="17" t="s">
+      <c r="B19" s="19"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="20"/>
+      <c r="F19" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="18"/>
-      <c r="J19" s="18"/>
-      <c r="K19" s="18"/>
-      <c r="L19" s="19"/>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="G19" s="19"/>
+      <c r="H19" s="19"/>
+      <c r="I19" s="19"/>
+      <c r="J19" s="19"/>
+      <c r="K19" s="19"/>
+      <c r="L19" s="20"/>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>1</v>
       </c>
@@ -3058,7 +3253,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>1</v>
       </c>
@@ -3093,7 +3288,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>2</v>
       </c>
@@ -3128,7 +3323,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
         <v>3</v>
       </c>
@@ -3163,30 +3358,35 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A26" s="17" t="s">
+    <row r="25" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A26" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="B26" s="18"/>
-      <c r="C26" s="18"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
-      <c r="G26" s="19"/>
-      <c r="I26" s="17" t="s">
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
+      <c r="G26" s="20"/>
+      <c r="I26" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="J26" s="18"/>
-      <c r="K26" s="19"/>
-      <c r="M26" s="17" t="s">
+      <c r="J26" s="19"/>
+      <c r="K26" s="20"/>
+      <c r="M26" s="18" t="s">
+        <v>291</v>
+      </c>
+      <c r="N26" s="19"/>
+      <c r="O26" s="20"/>
+      <c r="Q26" s="18" t="s">
         <v>222</v>
       </c>
-      <c r="N26" s="18"/>
-      <c r="O26" s="18"/>
-      <c r="P26" s="19"/>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="R26" s="19"/>
+      <c r="S26" s="20"/>
+      <c r="T26" s="25"/>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>1</v>
       </c>
@@ -3218,19 +3418,25 @@
         <v>3</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="N27" t="s">
-        <v>60</v>
-      </c>
-      <c r="O27" t="s">
+        <v>292</v>
+      </c>
+      <c r="N27" s="24" t="s">
+        <v>293</v>
+      </c>
+      <c r="O27" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q27" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="R27" s="31" t="s">
         <v>221</v>
       </c>
-      <c r="P27" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="S27" s="27" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>1</v>
       </c>
@@ -3264,17 +3470,23 @@
       <c r="M28" s="1">
         <v>1</v>
       </c>
-      <c r="N28">
-        <v>1</v>
-      </c>
-      <c r="O28" t="s">
+      <c r="N28" s="24">
+        <v>1</v>
+      </c>
+      <c r="O28" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q28" s="26">
+        <v>1</v>
+      </c>
+      <c r="R28" s="31" t="s">
         <v>61</v>
       </c>
-      <c r="P28" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="S28" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>2</v>
       </c>
@@ -3306,19 +3518,25 @@
         <v>1</v>
       </c>
       <c r="M29" s="1">
-        <v>2</v>
-      </c>
-      <c r="N29">
-        <v>1</v>
-      </c>
-      <c r="O29" t="s">
+        <v>1</v>
+      </c>
+      <c r="N29" s="24">
+        <v>2</v>
+      </c>
+      <c r="O29" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q29" s="26">
+        <v>2</v>
+      </c>
+      <c r="R29" s="31" t="s">
         <v>62</v>
       </c>
-      <c r="P29" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="S29" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="3">
         <v>3</v>
       </c>
@@ -3350,37 +3568,43 @@
         <v>1</v>
       </c>
       <c r="M30" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N30" s="4">
-        <v>3</v>
-      </c>
-      <c r="O30" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="O30" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q30" s="28">
+        <v>3</v>
+      </c>
+      <c r="R30" s="29" t="s">
         <v>63</v>
       </c>
-      <c r="P30" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+      <c r="S30" s="30" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A33" s="17" t="s">
+      <c r="A33" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="B33" s="18"/>
-      <c r="C33" s="18"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
-      <c r="F33" s="18"/>
-      <c r="G33" s="18"/>
-      <c r="H33" s="18"/>
-      <c r="I33" s="19"/>
-      <c r="K33" s="17" t="s">
+      <c r="B33" s="19"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="19"/>
+      <c r="F33" s="19"/>
+      <c r="G33" s="19"/>
+      <c r="H33" s="19"/>
+      <c r="I33" s="20"/>
+      <c r="K33" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="L33" s="18"/>
-      <c r="M33" s="18"/>
-      <c r="N33" s="19"/>
+      <c r="L33" s="19"/>
+      <c r="M33" s="19"/>
+      <c r="N33" s="20"/>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
@@ -3548,22 +3772,22 @@
     </row>
     <row r="39" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="40" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A40" s="17" t="s">
+      <c r="A40" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="B40" s="18"/>
-      <c r="C40" s="18"/>
-      <c r="D40" s="18"/>
-      <c r="E40" s="18"/>
-      <c r="F40" s="19"/>
-      <c r="H40" s="17" t="s">
+      <c r="B40" s="19"/>
+      <c r="C40" s="19"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="20"/>
+      <c r="H40" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="I40" s="18"/>
-      <c r="J40" s="18"/>
-      <c r="K40" s="18"/>
-      <c r="L40" s="18"/>
-      <c r="M40" s="19"/>
+      <c r="I40" s="19"/>
+      <c r="J40" s="19"/>
+      <c r="K40" s="19"/>
+      <c r="L40" s="19"/>
+      <c r="M40" s="20"/>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
@@ -3719,22 +3943,22 @@
     </row>
     <row r="46" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A47" s="17" t="s">
+      <c r="A47" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="B47" s="18"/>
-      <c r="C47" s="18"/>
-      <c r="D47" s="19"/>
-      <c r="F47" s="17" t="s">
+      <c r="B47" s="19"/>
+      <c r="C47" s="19"/>
+      <c r="D47" s="20"/>
+      <c r="F47" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="G47" s="18"/>
-      <c r="H47" s="18"/>
-      <c r="I47" s="18"/>
-      <c r="J47" s="18"/>
-      <c r="K47" s="18"/>
-      <c r="L47" s="18"/>
-      <c r="M47" s="19"/>
+      <c r="G47" s="19"/>
+      <c r="H47" s="19"/>
+      <c r="I47" s="19"/>
+      <c r="J47" s="19"/>
+      <c r="K47" s="19"/>
+      <c r="L47" s="19"/>
+      <c r="M47" s="20"/>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
@@ -3752,22 +3976,22 @@
       <c r="F48" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G48" s="23" t="s">
+      <c r="G48" t="s">
         <v>73</v>
       </c>
-      <c r="H48" s="23" t="s">
+      <c r="H48" t="s">
         <v>74</v>
       </c>
-      <c r="I48" s="23" t="s">
+      <c r="I48" t="s">
         <v>75</v>
       </c>
-      <c r="J48" s="23" t="s">
+      <c r="J48" t="s">
         <v>76</v>
       </c>
-      <c r="K48" s="23" t="s">
+      <c r="K48" t="s">
         <v>77</v>
       </c>
-      <c r="L48" s="23" t="s">
+      <c r="L48" t="s">
         <v>280</v>
       </c>
       <c r="M48" s="2" t="s">
@@ -3790,22 +4014,22 @@
       <c r="F49" s="1">
         <v>1</v>
       </c>
-      <c r="G49" s="23" t="s">
+      <c r="G49" t="s">
         <v>78</v>
       </c>
-      <c r="H49" s="23">
-        <v>1</v>
-      </c>
-      <c r="I49" s="29" t="s">
+      <c r="H49">
+        <v>1</v>
+      </c>
+      <c r="I49" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="J49" s="29" t="s">
+      <c r="J49" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="K49" s="23">
+      <c r="K49">
         <v>4</v>
       </c>
-      <c r="L49" s="23" t="s">
+      <c r="L49" t="s">
         <v>282</v>
       </c>
       <c r="M49" s="2" t="b">
@@ -3828,22 +4052,22 @@
       <c r="F50" s="1">
         <v>2</v>
       </c>
-      <c r="G50" s="23" t="s">
+      <c r="G50" t="s">
         <v>79</v>
       </c>
-      <c r="H50" s="23">
-        <v>1</v>
-      </c>
-      <c r="I50" s="29" t="s">
+      <c r="H50">
+        <v>1</v>
+      </c>
+      <c r="I50" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="J50" s="29" t="s">
+      <c r="J50" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="K50" s="23">
+      <c r="K50">
         <v>5</v>
       </c>
-      <c r="L50" s="23" t="s">
+      <c r="L50" t="s">
         <v>282</v>
       </c>
       <c r="M50" s="2" t="b">
@@ -3890,17 +4114,17 @@
     </row>
     <row r="53" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="54" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A54" s="17" t="s">
+      <c r="A54" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="B54" s="18"/>
-      <c r="C54" s="18"/>
-      <c r="D54" s="18"/>
-      <c r="E54" s="18"/>
-      <c r="F54" s="18"/>
-      <c r="G54" s="18"/>
-      <c r="H54" s="18"/>
-      <c r="I54" s="19"/>
+      <c r="B54" s="19"/>
+      <c r="C54" s="19"/>
+      <c r="D54" s="19"/>
+      <c r="E54" s="19"/>
+      <c r="F54" s="19"/>
+      <c r="G54" s="19"/>
+      <c r="H54" s="19"/>
+      <c r="I54" s="20"/>
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
@@ -4020,20 +4244,20 @@
     </row>
     <row r="60" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="61" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A61" s="17" t="s">
+      <c r="A61" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="B61" s="18"/>
-      <c r="C61" s="18"/>
-      <c r="D61" s="18"/>
-      <c r="E61" s="19"/>
-      <c r="G61" s="17" t="s">
+      <c r="B61" s="19"/>
+      <c r="C61" s="19"/>
+      <c r="D61" s="19"/>
+      <c r="E61" s="20"/>
+      <c r="G61" s="18" t="s">
         <v>136</v>
       </c>
-      <c r="H61" s="18"/>
-      <c r="I61" s="18"/>
-      <c r="J61" s="18"/>
-      <c r="K61" s="19"/>
+      <c r="H61" s="19"/>
+      <c r="I61" s="19"/>
+      <c r="J61" s="19"/>
+      <c r="K61" s="20"/>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
@@ -4168,13 +4392,13 @@
     </row>
     <row r="67" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="68" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A68" s="17" t="s">
+      <c r="A68" s="18" t="s">
         <v>137</v>
       </c>
-      <c r="B68" s="18"/>
-      <c r="C68" s="18"/>
-      <c r="D68" s="18"/>
-      <c r="E68" s="19"/>
+      <c r="B68" s="19"/>
+      <c r="C68" s="19"/>
+      <c r="D68" s="19"/>
+      <c r="E68" s="20"/>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
@@ -4246,18 +4470,18 @@
     </row>
     <row r="74" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="75" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A75" s="17" t="s">
+      <c r="A75" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="B75" s="18"/>
-      <c r="C75" s="18"/>
-      <c r="D75" s="18"/>
-      <c r="E75" s="18"/>
-      <c r="F75" s="18"/>
-      <c r="G75" s="18"/>
-      <c r="H75" s="18"/>
-      <c r="I75" s="18"/>
-      <c r="J75" s="19"/>
+      <c r="B75" s="19"/>
+      <c r="C75" s="19"/>
+      <c r="D75" s="19"/>
+      <c r="E75" s="19"/>
+      <c r="F75" s="19"/>
+      <c r="G75" s="19"/>
+      <c r="H75" s="19"/>
+      <c r="I75" s="19"/>
+      <c r="J75" s="20"/>
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
@@ -4325,20 +4549,20 @@
     </row>
     <row r="79" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="80" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A80" s="17" t="s">
+      <c r="A80" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="B80" s="18"/>
-      <c r="C80" s="18"/>
-      <c r="D80" s="18"/>
-      <c r="E80" s="18"/>
-      <c r="F80" s="18"/>
-      <c r="G80" s="18"/>
-      <c r="H80" s="18"/>
-      <c r="I80" s="18"/>
-      <c r="J80" s="18"/>
-      <c r="K80" s="18"/>
-      <c r="L80" s="19"/>
+      <c r="B80" s="19"/>
+      <c r="C80" s="19"/>
+      <c r="D80" s="19"/>
+      <c r="E80" s="19"/>
+      <c r="F80" s="19"/>
+      <c r="G80" s="19"/>
+      <c r="H80" s="19"/>
+      <c r="I80" s="19"/>
+      <c r="J80" s="19"/>
+      <c r="K80" s="19"/>
+      <c r="L80" s="20"/>
     </row>
     <row r="81" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
@@ -4494,22 +4718,22 @@
     </row>
     <row r="86" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="87" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A87" s="17" t="s">
+      <c r="A87" s="18" t="s">
         <v>165</v>
       </c>
-      <c r="B87" s="19"/>
-      <c r="D87" s="17" t="s">
+      <c r="B87" s="20"/>
+      <c r="D87" s="18" t="s">
         <v>168</v>
       </c>
-      <c r="E87" s="18"/>
-      <c r="F87" s="19"/>
-      <c r="H87" s="17" t="s">
+      <c r="E87" s="19"/>
+      <c r="F87" s="20"/>
+      <c r="H87" s="18" t="s">
         <v>183</v>
       </c>
-      <c r="I87" s="18"/>
-      <c r="J87" s="18"/>
-      <c r="K87" s="18"/>
-      <c r="L87" s="19"/>
+      <c r="I87" s="19"/>
+      <c r="J87" s="19"/>
+      <c r="K87" s="19"/>
+      <c r="L87" s="20"/>
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
@@ -4641,22 +4865,22 @@
     </row>
     <row r="93" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="94" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A94" s="17" t="s">
+      <c r="A94" s="18" t="s">
         <v>196</v>
       </c>
-      <c r="B94" s="18"/>
-      <c r="C94" s="18"/>
-      <c r="D94" s="18"/>
-      <c r="E94" s="18"/>
-      <c r="F94" s="18"/>
-      <c r="G94" s="18"/>
-      <c r="H94" s="18"/>
-      <c r="I94" s="18"/>
-      <c r="J94" s="18"/>
-      <c r="K94" s="18"/>
-      <c r="L94" s="18"/>
-      <c r="M94" s="18"/>
-      <c r="N94" s="19"/>
+      <c r="B94" s="19"/>
+      <c r="C94" s="19"/>
+      <c r="D94" s="19"/>
+      <c r="E94" s="19"/>
+      <c r="F94" s="19"/>
+      <c r="G94" s="19"/>
+      <c r="H94" s="19"/>
+      <c r="I94" s="19"/>
+      <c r="J94" s="19"/>
+      <c r="K94" s="19"/>
+      <c r="L94" s="19"/>
+      <c r="M94" s="19"/>
+      <c r="N94" s="20"/>
     </row>
     <row r="95" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
@@ -4836,17 +5060,17 @@
     </row>
     <row r="100" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="101" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A101" s="17" t="s">
+      <c r="A101" s="18" t="s">
         <v>195</v>
       </c>
-      <c r="B101" s="18"/>
-      <c r="C101" s="18"/>
-      <c r="D101" s="18"/>
-      <c r="E101" s="18"/>
-      <c r="F101" s="18"/>
-      <c r="G101" s="18"/>
-      <c r="H101" s="18"/>
-      <c r="I101" s="19"/>
+      <c r="B101" s="19"/>
+      <c r="C101" s="19"/>
+      <c r="D101" s="19"/>
+      <c r="E101" s="19"/>
+      <c r="F101" s="19"/>
+      <c r="G101" s="19"/>
+      <c r="H101" s="19"/>
+      <c r="I101" s="20"/>
     </row>
     <row r="102" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
@@ -4966,13 +5190,13 @@
     </row>
     <row r="107" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="108" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A108" s="17" t="s">
+      <c r="A108" s="18" t="s">
         <v>198</v>
       </c>
-      <c r="B108" s="18"/>
-      <c r="C108" s="18"/>
-      <c r="D108" s="18"/>
-      <c r="E108" s="19"/>
+      <c r="B108" s="19"/>
+      <c r="C108" s="19"/>
+      <c r="D108" s="19"/>
+      <c r="E108" s="20"/>
     </row>
     <row r="109" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
@@ -5044,26 +5268,26 @@
     </row>
     <row r="114" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="115" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A115" s="17" t="s">
+      <c r="A115" s="18" t="s">
         <v>205</v>
       </c>
-      <c r="B115" s="18"/>
-      <c r="C115" s="18"/>
-      <c r="D115" s="18"/>
-      <c r="E115" s="18"/>
-      <c r="F115" s="18"/>
-      <c r="G115" s="18"/>
-      <c r="H115" s="18"/>
-      <c r="I115" s="18"/>
-      <c r="J115" s="18"/>
-      <c r="K115" s="18"/>
-      <c r="L115" s="18"/>
-      <c r="M115" s="18"/>
-      <c r="N115" s="19"/>
+      <c r="B115" s="19"/>
+      <c r="C115" s="19"/>
+      <c r="D115" s="19"/>
+      <c r="E115" s="19"/>
+      <c r="F115" s="19"/>
+      <c r="G115" s="19"/>
+      <c r="H115" s="19"/>
+      <c r="I115" s="19"/>
+      <c r="J115" s="19"/>
+      <c r="K115" s="19"/>
+      <c r="L115" s="19"/>
+      <c r="M115" s="19"/>
+      <c r="N115" s="20"/>
     </row>
     <row r="116" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
-        <v>1</v>
+        <v>294</v>
       </c>
       <c r="B116" t="s">
         <v>206</v>
@@ -5239,24 +5463,24 @@
     </row>
     <row r="121" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="122" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A122" s="17" t="s">
+      <c r="A122" s="18" t="s">
         <v>217</v>
       </c>
-      <c r="B122" s="18"/>
-      <c r="C122" s="18"/>
-      <c r="D122" s="18"/>
-      <c r="E122" s="18"/>
-      <c r="F122" s="19"/>
-      <c r="H122" s="17" t="s">
+      <c r="B122" s="19"/>
+      <c r="C122" s="19"/>
+      <c r="D122" s="19"/>
+      <c r="E122" s="19"/>
+      <c r="F122" s="20"/>
+      <c r="H122" s="18" t="s">
         <v>257</v>
       </c>
-      <c r="I122" s="18"/>
-      <c r="J122" s="19"/>
-      <c r="L122" s="17" t="s">
+      <c r="I122" s="19"/>
+      <c r="J122" s="20"/>
+      <c r="L122" s="18" t="s">
         <v>262</v>
       </c>
-      <c r="M122" s="18"/>
-      <c r="N122" s="19"/>
+      <c r="M122" s="19"/>
+      <c r="N122" s="20"/>
     </row>
     <row r="123" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A123" s="1" t="s">
@@ -5280,7 +5504,7 @@
       <c r="H123" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="I123" s="23" t="s">
+      <c r="I123" t="s">
         <v>258</v>
       </c>
       <c r="J123" s="2" t="s">
@@ -5289,7 +5513,7 @@
       <c r="L123" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="M123" s="23" t="s">
+      <c r="M123" t="s">
         <v>262</v>
       </c>
       <c r="N123" s="2" t="s">
@@ -5318,19 +5542,19 @@
       <c r="H124" s="1">
         <v>1</v>
       </c>
-      <c r="I124" s="23" t="s">
+      <c r="I124" t="s">
         <v>259</v>
       </c>
-      <c r="J124" s="26" t="b">
+      <c r="J124" s="8" t="b">
         <v>1</v>
       </c>
       <c r="L124" s="1">
         <v>1</v>
       </c>
-      <c r="M124" s="23" t="s">
+      <c r="M124" t="s">
         <v>263</v>
       </c>
-      <c r="N124" s="26" t="b">
+      <c r="N124" s="8" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5356,19 +5580,19 @@
       <c r="H125" s="1">
         <v>2</v>
       </c>
-      <c r="I125" s="23" t="s">
+      <c r="I125" t="s">
         <v>260</v>
       </c>
-      <c r="J125" s="27" t="b">
+      <c r="J125" s="2" t="b">
         <v>1</v>
       </c>
       <c r="L125" s="1">
         <v>2</v>
       </c>
-      <c r="M125" s="23" t="s">
+      <c r="M125" t="s">
         <v>264</v>
       </c>
-      <c r="N125" s="27" t="b">
+      <c r="N125" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5397,7 +5621,7 @@
       <c r="I126" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="J126" s="28" t="b">
+      <c r="J126" s="9" t="b">
         <v>1</v>
       </c>
       <c r="L126" s="3">
@@ -5406,119 +5630,119 @@
       <c r="M126" s="4" t="s">
         <v>265</v>
       </c>
-      <c r="N126" s="28" t="b">
+      <c r="N126" s="9" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="128" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="129" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A129" s="17" t="s">
+      <c r="A129" s="18" t="s">
         <v>231</v>
       </c>
-      <c r="B129" s="18"/>
-      <c r="C129" s="18"/>
-      <c r="D129" s="18"/>
-      <c r="E129" s="18"/>
-      <c r="F129" s="18"/>
-      <c r="G129" s="18"/>
-      <c r="H129" s="18"/>
-      <c r="I129" s="18"/>
-      <c r="J129" s="18"/>
-      <c r="K129" s="18"/>
-      <c r="L129" s="18"/>
-      <c r="M129" s="18"/>
-      <c r="N129" s="18"/>
-      <c r="O129" s="18"/>
-      <c r="P129" s="18"/>
-      <c r="Q129" s="18"/>
-      <c r="R129" s="18"/>
-      <c r="S129" s="18"/>
-      <c r="T129" s="18"/>
-      <c r="U129" s="18"/>
-      <c r="V129" s="18"/>
-      <c r="W129" s="18"/>
-      <c r="X129" s="18"/>
-      <c r="Y129" s="18"/>
-      <c r="Z129" s="18"/>
-      <c r="AA129" s="19"/>
+      <c r="B129" s="19"/>
+      <c r="C129" s="19"/>
+      <c r="D129" s="19"/>
+      <c r="E129" s="19"/>
+      <c r="F129" s="19"/>
+      <c r="G129" s="19"/>
+      <c r="H129" s="19"/>
+      <c r="I129" s="19"/>
+      <c r="J129" s="19"/>
+      <c r="K129" s="19"/>
+      <c r="L129" s="19"/>
+      <c r="M129" s="19"/>
+      <c r="N129" s="19"/>
+      <c r="O129" s="19"/>
+      <c r="P129" s="19"/>
+      <c r="Q129" s="19"/>
+      <c r="R129" s="19"/>
+      <c r="S129" s="19"/>
+      <c r="T129" s="19"/>
+      <c r="U129" s="19"/>
+      <c r="V129" s="19"/>
+      <c r="W129" s="19"/>
+      <c r="X129" s="19"/>
+      <c r="Y129" s="19"/>
+      <c r="Z129" s="19"/>
+      <c r="AA129" s="20"/>
     </row>
     <row r="130" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B130" s="23" t="s">
+      <c r="B130" t="s">
         <v>229</v>
       </c>
-      <c r="C130" s="23" t="s">
+      <c r="C130" t="s">
         <v>230</v>
       </c>
-      <c r="D130" s="23" t="s">
+      <c r="D130" t="s">
         <v>232</v>
       </c>
-      <c r="E130" s="23" t="s">
+      <c r="E130" t="s">
         <v>233</v>
       </c>
-      <c r="F130" s="23" t="s">
+      <c r="F130" t="s">
         <v>234</v>
       </c>
-      <c r="G130" s="23" t="s">
+      <c r="G130" t="s">
         <v>235</v>
       </c>
-      <c r="H130" s="23" t="s">
+      <c r="H130" t="s">
         <v>236</v>
       </c>
-      <c r="I130" s="23" t="s">
+      <c r="I130" t="s">
         <v>237</v>
       </c>
-      <c r="J130" s="23" t="s">
+      <c r="J130" t="s">
         <v>238</v>
       </c>
-      <c r="K130" s="23" t="s">
+      <c r="K130" t="s">
         <v>239</v>
       </c>
-      <c r="L130" s="23" t="s">
+      <c r="L130" t="s">
         <v>240</v>
       </c>
-      <c r="M130" s="23" t="s">
+      <c r="M130" t="s">
         <v>241</v>
       </c>
-      <c r="N130" s="23" t="s">
+      <c r="N130" t="s">
         <v>242</v>
       </c>
-      <c r="O130" s="23" t="s">
+      <c r="O130" t="s">
         <v>243</v>
       </c>
-      <c r="P130" s="23" t="s">
+      <c r="P130" t="s">
         <v>244</v>
       </c>
-      <c r="Q130" s="23" t="s">
+      <c r="Q130" t="s">
         <v>247</v>
       </c>
-      <c r="R130" s="23" t="s">
+      <c r="R130" t="s">
         <v>248</v>
       </c>
-      <c r="S130" s="23" t="s">
+      <c r="S130" t="s">
         <v>249</v>
       </c>
-      <c r="T130" s="23" t="s">
+      <c r="T130" t="s">
         <v>250</v>
       </c>
-      <c r="U130" s="23" t="s">
+      <c r="U130" t="s">
         <v>251</v>
       </c>
-      <c r="V130" s="23" t="s">
+      <c r="V130" t="s">
         <v>252</v>
       </c>
-      <c r="W130" s="23" t="s">
+      <c r="W130" t="s">
         <v>253</v>
       </c>
-      <c r="X130" s="23" t="s">
+      <c r="X130" t="s">
         <v>254</v>
       </c>
-      <c r="Y130" s="23" t="s">
+      <c r="Y130" t="s">
         <v>255</v>
       </c>
-      <c r="Z130" s="23" t="s">
+      <c r="Z130" t="s">
         <v>256</v>
       </c>
       <c r="AA130" s="2" t="s">
@@ -5529,79 +5753,79 @@
       <c r="A131" s="1">
         <v>1</v>
       </c>
-      <c r="B131" s="23">
-        <v>1</v>
-      </c>
-      <c r="C131" s="23">
-        <v>1</v>
-      </c>
-      <c r="D131" s="24">
+      <c r="B131">
+        <v>1</v>
+      </c>
+      <c r="C131">
+        <v>1</v>
+      </c>
+      <c r="D131" s="17">
         <v>46058</v>
       </c>
-      <c r="E131" s="24">
+      <c r="E131" s="17">
         <v>46058</v>
       </c>
-      <c r="F131" s="24">
+      <c r="F131" s="17">
         <v>46063</v>
       </c>
-      <c r="G131" s="23">
-        <v>1</v>
-      </c>
-      <c r="H131" s="23">
+      <c r="G131">
+        <v>1</v>
+      </c>
+      <c r="H131">
         <v>5</v>
       </c>
-      <c r="I131" s="23">
-        <v>2</v>
-      </c>
-      <c r="J131" s="25" t="s">
+      <c r="I131">
+        <v>2</v>
+      </c>
+      <c r="J131" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="K131" s="25" t="s">
+      <c r="K131" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="L131" s="23">
-        <v>1</v>
-      </c>
-      <c r="M131" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="N131" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="O131" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="P131" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="Q131" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="R131" s="23">
-        <v>1</v>
-      </c>
-      <c r="S131" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="T131" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="U131" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="V131" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="W131" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="X131" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="Y131" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="Z131" s="23">
+      <c r="L131">
+        <v>1</v>
+      </c>
+      <c r="M131" t="s">
+        <v>191</v>
+      </c>
+      <c r="N131" t="s">
+        <v>191</v>
+      </c>
+      <c r="O131" t="s">
+        <v>191</v>
+      </c>
+      <c r="P131" t="s">
+        <v>191</v>
+      </c>
+      <c r="Q131" t="s">
+        <v>191</v>
+      </c>
+      <c r="R131">
+        <v>1</v>
+      </c>
+      <c r="S131" t="s">
+        <v>191</v>
+      </c>
+      <c r="T131" t="s">
+        <v>191</v>
+      </c>
+      <c r="U131" t="s">
+        <v>191</v>
+      </c>
+      <c r="V131" t="s">
+        <v>191</v>
+      </c>
+      <c r="W131" t="s">
+        <v>191</v>
+      </c>
+      <c r="X131" t="s">
+        <v>191</v>
+      </c>
+      <c r="Y131" t="s">
+        <v>191</v>
+      </c>
+      <c r="Z131">
         <v>1</v>
       </c>
       <c r="AA131" s="2" t="b">
@@ -5612,79 +5836,79 @@
       <c r="A132" s="1">
         <v>2</v>
       </c>
-      <c r="B132" s="23">
-        <v>2</v>
-      </c>
-      <c r="C132" s="23">
-        <v>1</v>
-      </c>
-      <c r="D132" s="24">
+      <c r="B132">
+        <v>2</v>
+      </c>
+      <c r="C132">
+        <v>1</v>
+      </c>
+      <c r="D132" s="17">
         <v>46059</v>
       </c>
-      <c r="E132" s="24">
+      <c r="E132" s="17">
         <v>46059</v>
       </c>
-      <c r="F132" s="24">
+      <c r="F132" s="17">
         <v>46065</v>
       </c>
-      <c r="G132" s="23">
-        <v>1</v>
-      </c>
-      <c r="H132" s="23">
+      <c r="G132">
+        <v>1</v>
+      </c>
+      <c r="H132">
         <v>8</v>
       </c>
-      <c r="I132" s="23">
-        <v>3</v>
-      </c>
-      <c r="J132" s="25" t="s">
+      <c r="I132">
+        <v>3</v>
+      </c>
+      <c r="J132" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="K132" s="25" t="s">
+      <c r="K132" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="L132" s="23">
-        <v>2</v>
-      </c>
-      <c r="M132" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="N132" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="O132" s="23" t="s">
+      <c r="L132">
+        <v>2</v>
+      </c>
+      <c r="M132" t="s">
+        <v>191</v>
+      </c>
+      <c r="N132" t="s">
+        <v>191</v>
+      </c>
+      <c r="O132" t="s">
         <v>245</v>
       </c>
-      <c r="P132" s="23">
-        <v>2</v>
-      </c>
-      <c r="Q132" s="23">
-        <v>1</v>
-      </c>
-      <c r="R132" s="23">
-        <v>1</v>
-      </c>
-      <c r="S132" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="T132" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="U132" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="V132" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="W132" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="X132" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="Y132" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="Z132" s="23">
+      <c r="P132">
+        <v>2</v>
+      </c>
+      <c r="Q132">
+        <v>1</v>
+      </c>
+      <c r="R132">
+        <v>1</v>
+      </c>
+      <c r="S132" t="s">
+        <v>191</v>
+      </c>
+      <c r="T132" t="s">
+        <v>191</v>
+      </c>
+      <c r="U132" t="s">
+        <v>191</v>
+      </c>
+      <c r="V132" t="s">
+        <v>191</v>
+      </c>
+      <c r="W132" t="s">
+        <v>191</v>
+      </c>
+      <c r="X132" t="s">
+        <v>191</v>
+      </c>
+      <c r="Y132" t="s">
+        <v>191</v>
+      </c>
+      <c r="Z132">
         <v>2</v>
       </c>
       <c r="AA132" s="2" t="b">
@@ -5776,35 +6000,35 @@
     </row>
     <row r="135" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="136" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A136" s="17" t="s">
+      <c r="A136" s="18" t="s">
         <v>266</v>
       </c>
-      <c r="B136" s="18"/>
-      <c r="C136" s="19"/>
-      <c r="E136" s="17" t="s">
+      <c r="B136" s="19"/>
+      <c r="C136" s="20"/>
+      <c r="E136" s="18" t="s">
         <v>270</v>
       </c>
-      <c r="F136" s="18"/>
-      <c r="G136" s="19"/>
-      <c r="I136" s="17" t="s">
+      <c r="F136" s="19"/>
+      <c r="G136" s="20"/>
+      <c r="I136" s="18" t="s">
         <v>272</v>
       </c>
-      <c r="J136" s="18"/>
-      <c r="K136" s="18"/>
-      <c r="L136" s="19"/>
-      <c r="N136" s="17" t="s">
+      <c r="J136" s="19"/>
+      <c r="K136" s="19"/>
+      <c r="L136" s="20"/>
+      <c r="N136" s="18" t="s">
         <v>277</v>
       </c>
-      <c r="O136" s="18"/>
-      <c r="P136" s="18"/>
-      <c r="Q136" s="18"/>
-      <c r="R136" s="19"/>
+      <c r="O136" s="19"/>
+      <c r="P136" s="19"/>
+      <c r="Q136" s="19"/>
+      <c r="R136" s="20"/>
     </row>
     <row r="137" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A137" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B137" s="23" t="s">
+      <c r="B137" t="s">
         <v>266</v>
       </c>
       <c r="C137" s="2" t="s">
@@ -5813,7 +6037,7 @@
       <c r="E137" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F137" s="23" t="s">
+      <c r="F137" t="s">
         <v>270</v>
       </c>
       <c r="G137" s="2" t="s">
@@ -5822,10 +6046,10 @@
       <c r="I137" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J137" s="23" t="s">
+      <c r="J137" t="s">
         <v>273</v>
       </c>
-      <c r="K137" s="23" t="s">
+      <c r="K137" t="s">
         <v>272</v>
       </c>
       <c r="L137" s="2" t="s">
@@ -5834,13 +6058,13 @@
       <c r="N137" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="O137" s="23" t="s">
+      <c r="O137" t="s">
         <v>273</v>
       </c>
-      <c r="P137" s="23" t="s">
+      <c r="P137" t="s">
         <v>278</v>
       </c>
-      <c r="Q137" s="23" t="s">
+      <c r="Q137" t="s">
         <v>279</v>
       </c>
       <c r="R137" s="2" t="s">
@@ -5851,46 +6075,46 @@
       <c r="A138" s="1">
         <v>1</v>
       </c>
-      <c r="B138" s="23" t="s">
+      <c r="B138" t="s">
         <v>267</v>
       </c>
-      <c r="C138" s="26" t="b">
+      <c r="C138" s="8" t="b">
         <v>1</v>
       </c>
       <c r="E138" s="1">
         <v>1</v>
       </c>
-      <c r="F138" s="23" t="s">
+      <c r="F138" t="s">
         <v>271</v>
       </c>
-      <c r="G138" s="26" t="b">
+      <c r="G138" s="8" t="b">
         <v>1</v>
       </c>
       <c r="I138" s="1">
         <v>1</v>
       </c>
-      <c r="J138" s="23">
+      <c r="J138">
         <v>11</v>
       </c>
-      <c r="K138" s="23" t="s">
+      <c r="K138" t="s">
         <v>274</v>
       </c>
-      <c r="L138" s="26" t="b">
+      <c r="L138" s="8" t="b">
         <v>1</v>
       </c>
       <c r="N138" s="1">
         <v>1</v>
       </c>
-      <c r="O138" s="23">
-        <v>1</v>
-      </c>
-      <c r="P138" s="24">
+      <c r="O138">
+        <v>1</v>
+      </c>
+      <c r="P138" s="17">
         <v>46058</v>
       </c>
-      <c r="Q138" s="25" t="s">
+      <c r="Q138" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="R138" s="26" t="b">
+      <c r="R138" s="8" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5898,46 +6122,46 @@
       <c r="A139" s="1">
         <v>2</v>
       </c>
-      <c r="B139" s="23" t="s">
+      <c r="B139" t="s">
         <v>268</v>
       </c>
-      <c r="C139" s="27" t="b">
+      <c r="C139" s="2" t="b">
         <v>1</v>
       </c>
       <c r="E139" s="1">
         <v>2</v>
       </c>
-      <c r="F139" s="23" t="s">
+      <c r="F139" t="s">
         <v>39</v>
       </c>
-      <c r="G139" s="27" t="b">
+      <c r="G139" s="2" t="b">
         <v>1</v>
       </c>
       <c r="I139" s="1">
         <v>2</v>
       </c>
-      <c r="J139" s="23">
+      <c r="J139">
         <v>21</v>
       </c>
-      <c r="K139" s="23" t="s">
+      <c r="K139" t="s">
         <v>275</v>
       </c>
-      <c r="L139" s="27" t="b">
+      <c r="L139" s="2" t="b">
         <v>1</v>
       </c>
       <c r="N139" s="1">
         <v>2</v>
       </c>
-      <c r="O139" s="23">
-        <v>1</v>
-      </c>
-      <c r="P139" s="24">
+      <c r="O139">
+        <v>1</v>
+      </c>
+      <c r="P139" s="17">
         <v>46059</v>
       </c>
-      <c r="Q139" s="25" t="s">
+      <c r="Q139" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="R139" s="27" t="b">
+      <c r="R139" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5948,7 +6172,7 @@
       <c r="B140" s="4" t="s">
         <v>269</v>
       </c>
-      <c r="C140" s="28" t="b">
+      <c r="C140" s="9" t="b">
         <v>1</v>
       </c>
       <c r="E140" s="3">
@@ -5957,7 +6181,7 @@
       <c r="F140" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="G140" s="28" t="b">
+      <c r="G140" s="9" t="b">
         <v>1</v>
       </c>
       <c r="I140" s="3">
@@ -5969,7 +6193,7 @@
       <c r="K140" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="L140" s="28" t="b">
+      <c r="L140" s="9" t="b">
         <v>1</v>
       </c>
       <c r="N140" s="3">
@@ -5984,20 +6208,30 @@
       <c r="Q140" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="R140" s="28" t="b">
+      <c r="R140" s="9" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="37">
-    <mergeCell ref="A129:AA129"/>
-    <mergeCell ref="H122:J122"/>
-    <mergeCell ref="L122:N122"/>
-    <mergeCell ref="A136:C136"/>
-    <mergeCell ref="E136:G136"/>
-    <mergeCell ref="I136:L136"/>
-    <mergeCell ref="N136:R136"/>
-    <mergeCell ref="M26:P26"/>
+  <mergeCells count="40">
+    <mergeCell ref="M5:O5"/>
+    <mergeCell ref="Q5:S5"/>
+    <mergeCell ref="Q26:S26"/>
+    <mergeCell ref="M26:O26"/>
+    <mergeCell ref="G61:K61"/>
+    <mergeCell ref="A68:E68"/>
+    <mergeCell ref="A75:J75"/>
+    <mergeCell ref="M12:P12"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A33:I33"/>
+    <mergeCell ref="K33:N33"/>
+    <mergeCell ref="I5:K5"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="F19:L19"/>
+    <mergeCell ref="G12:K12"/>
+    <mergeCell ref="I26:K26"/>
     <mergeCell ref="A122:F122"/>
     <mergeCell ref="A108:E108"/>
     <mergeCell ref="A94:N94"/>
@@ -6012,27 +6246,20 @@
     <mergeCell ref="A54:I54"/>
     <mergeCell ref="A40:F40"/>
     <mergeCell ref="H40:M40"/>
-    <mergeCell ref="I5:K5"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A26:G26"/>
-    <mergeCell ref="F19:L19"/>
-    <mergeCell ref="G12:K12"/>
-    <mergeCell ref="I26:K26"/>
     <mergeCell ref="A61:E61"/>
-    <mergeCell ref="G61:K61"/>
-    <mergeCell ref="A68:E68"/>
-    <mergeCell ref="A75:J75"/>
-    <mergeCell ref="M12:P12"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A33:I33"/>
-    <mergeCell ref="K33:N33"/>
+    <mergeCell ref="A129:AA129"/>
+    <mergeCell ref="H122:J122"/>
+    <mergeCell ref="L122:N122"/>
+    <mergeCell ref="A136:C136"/>
+    <mergeCell ref="E136:G136"/>
+    <mergeCell ref="I136:L136"/>
+    <mergeCell ref="N136:R136"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
-  <tableParts count="37">
+  <tableParts count="40">
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
     <tablePart r:id="rId5"/>
@@ -6070,6 +6297,9 @@
     <tablePart r:id="rId37"/>
     <tablePart r:id="rId38"/>
     <tablePart r:id="rId39"/>
+    <tablePart r:id="rId40"/>
+    <tablePart r:id="rId41"/>
+    <tablePart r:id="rId42"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>